<commit_message>
Added railway blueprints and updated some factory diagrams. Missing the savegame! Im really sorry
</commit_message>
<xml_diff>
--- a/Game Stuff/Spreadsheet.xlsx
+++ b/Game Stuff/Spreadsheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Nicos Blueprints_Riveteers District - Final\Game Stuff\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Nicos Blueprints_Trains\Game Stuff\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C2E70E9-A7EE-4AF7-9F91-96A7B04A868D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7822684-F23A-4D8D-A970-8ADD0544EEAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="45972" yWindow="-4944" windowWidth="17496" windowHeight="30216" firstSheet="11" activeTab="11" xr2:uid="{E9D95B66-7EA4-4203-9BE9-B35EAC251241}"/>
+    <workbookView xWindow="45972" yWindow="-4944" windowWidth="17496" windowHeight="30216" firstSheet="2" activeTab="3" xr2:uid="{E9D95B66-7EA4-4203-9BE9-B35EAC251241}"/>
   </bookViews>
   <sheets>
     <sheet name="Material Summary" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="584" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="589" uniqueCount="157">
   <si>
     <t>Item</t>
   </si>
@@ -202,15 +202,6 @@
     <t>Oran-Rief Mines</t>
   </si>
   <si>
-    <t>803.3 MW</t>
-  </si>
-  <si>
-    <t>-803.3 MW</t>
-  </si>
-  <si>
-    <t>2.74 Hours</t>
-  </si>
-  <si>
     <t>2200 MWh</t>
   </si>
   <si>
@@ -334,18 +325,9 @@
     <t>Raw Quartz</t>
   </si>
   <si>
-    <t>1016.2 MW</t>
-  </si>
-  <si>
-    <t>-1016.2 MW</t>
-  </si>
-  <si>
     <t>4300 Wh</t>
   </si>
   <si>
-    <t>4.23 Hours</t>
-  </si>
-  <si>
     <t>Ghirapur Gridworks</t>
   </si>
   <si>
@@ -469,9 +451,6 @@
     <t>63.39 Hours</t>
   </si>
   <si>
-    <t>Bottom Right going to Riveteers District has an extra 233.33 Copper Ingots</t>
-  </si>
-  <si>
     <t>Riverteers District</t>
   </si>
   <si>
@@ -512,6 +491,33 @@
   </si>
   <si>
     <t>4.80 Hours</t>
+  </si>
+  <si>
+    <t>1011.1 MW</t>
+  </si>
+  <si>
+    <t>-1011.1 MW</t>
+  </si>
+  <si>
+    <t>2.17 Hours</t>
+  </si>
+  <si>
+    <t>Alclad Aluminum Sheet</t>
+  </si>
+  <si>
+    <t>1108 MW</t>
+  </si>
+  <si>
+    <t>-1108 MW</t>
+  </si>
+  <si>
+    <t>3.88 Hours</t>
+  </si>
+  <si>
+    <t>On the desert</t>
+  </si>
+  <si>
+    <t>Top belt going to Riveteers district has an extra 533.33 Copper</t>
   </si>
 </sst>
 </file>
@@ -842,7 +848,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -918,6 +924,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -930,14 +944,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1285,18 +1294,18 @@
   <sheetData>
     <row r="3" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="4" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C4" s="39" t="s">
+      <c r="C4" s="43" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="40"/>
-      <c r="E4" s="41"/>
+      <c r="D4" s="44"/>
+      <c r="E4" s="45"/>
       <c r="F4" s="16"/>
       <c r="G4" s="16"/>
-      <c r="H4" s="39" t="s">
+      <c r="H4" s="43" t="s">
         <v>8</v>
       </c>
-      <c r="I4" s="40"/>
-      <c r="J4" s="41"/>
+      <c r="I4" s="44"/>
+      <c r="J4" s="45"/>
     </row>
     <row r="5" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C5" s="17" t="s">
@@ -1310,13 +1319,13 @@
       </c>
       <c r="F5" s="18"/>
       <c r="G5" s="18"/>
-      <c r="H5" s="43" t="s">
+      <c r="H5" s="39" t="s">
         <v>0</v>
       </c>
       <c r="I5" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="J5" s="44" t="s">
+      <c r="J5" s="40" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1330,13 +1339,13 @@
       <c r="E6" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="H6" s="45" t="s">
+      <c r="H6" s="41" t="s">
         <v>5</v>
       </c>
       <c r="I6" s="35">
         <v>15</v>
       </c>
-      <c r="J6" s="46" t="s">
+      <c r="J6" s="42" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1371,13 +1380,13 @@
         <v>42</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="I8" s="13">
         <v>1.4065000000000001</v>
       </c>
       <c r="J8" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="9" spans="3:10" x14ac:dyDescent="0.35">
@@ -1391,113 +1400,113 @@
         <v>44</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="I9" s="13">
         <v>2.25</v>
       </c>
       <c r="J9" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10" spans="3:10" x14ac:dyDescent="0.35">
       <c r="C10" s="2" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D10" s="11">
-        <v>204</v>
+        <v>252</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>50</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="I10" s="13">
         <v>2.5</v>
       </c>
       <c r="J10" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="11" spans="3:10" x14ac:dyDescent="0.35">
       <c r="C11" s="2" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D11" s="11">
         <v>1140</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="I11" s="13">
         <v>45</v>
       </c>
       <c r="J11" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="12" spans="3:10" x14ac:dyDescent="0.35">
       <c r="C12" s="4" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="D12" s="11">
-        <v>669.33299999999997</v>
+        <v>759.75</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I12" s="13">
         <v>5</v>
       </c>
       <c r="J12" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="13" spans="3:10" x14ac:dyDescent="0.35">
       <c r="C13" s="4" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="D13" s="11">
         <v>635.40554999999995</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="I13" s="13">
         <v>7.3125</v>
       </c>
       <c r="J13" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="14" spans="3:10" x14ac:dyDescent="0.35">
       <c r="C14" s="4" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="D14" s="11">
         <v>467.5</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="I14" s="13">
         <v>3</v>
       </c>
       <c r="J14" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="15" spans="3:10" x14ac:dyDescent="0.35">
@@ -1508,50 +1517,56 @@
         <v>348</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="I15" s="13">
         <v>30</v>
       </c>
       <c r="J15" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="16" spans="3:10" x14ac:dyDescent="0.35">
       <c r="C16" s="6" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D16" s="13">
         <v>246.666</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="I16" s="13">
         <v>0.5</v>
       </c>
       <c r="J16" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="17" spans="3:10" x14ac:dyDescent="0.35">
-      <c r="C17" s="4"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="4"/>
+      <c r="C17" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="D17" s="11">
+        <v>410</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>136</v>
+      </c>
       <c r="H17" s="6" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="I17" s="13">
         <v>33.125</v>
       </c>
       <c r="J17" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="18" spans="3:10" x14ac:dyDescent="0.35">
@@ -1559,13 +1574,13 @@
       <c r="D18" s="11"/>
       <c r="E18" s="2"/>
       <c r="H18" s="6" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="I18" s="13">
         <v>61.6875</v>
       </c>
       <c r="J18" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="19" spans="3:10" x14ac:dyDescent="0.35">
@@ -1573,13 +1588,13 @@
       <c r="D19" s="11"/>
       <c r="E19" s="2"/>
       <c r="H19" s="6" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="I19" s="13">
         <v>7.25</v>
       </c>
       <c r="J19" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="20" spans="3:10" x14ac:dyDescent="0.35">
@@ -1587,13 +1602,13 @@
       <c r="D20" s="11"/>
       <c r="E20" s="2"/>
       <c r="H20" s="6" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="I20" s="13">
         <v>30</v>
       </c>
       <c r="J20" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="21" spans="3:10" x14ac:dyDescent="0.35">
@@ -1601,13 +1616,13 @@
       <c r="D21" s="11"/>
       <c r="E21" s="2"/>
       <c r="H21" s="6" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="I21" s="13">
         <v>45</v>
       </c>
       <c r="J21" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="22" spans="3:10" x14ac:dyDescent="0.35">
@@ -1615,13 +1630,13 @@
       <c r="D22" s="11"/>
       <c r="E22" s="2"/>
       <c r="H22" s="6" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="I22" s="13">
         <v>22.5</v>
       </c>
       <c r="J22" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="23" spans="3:10" x14ac:dyDescent="0.35">
@@ -1629,13 +1644,13 @@
       <c r="D23" s="11"/>
       <c r="E23" s="2"/>
       <c r="H23" s="6" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="I23" s="13">
         <v>20.5</v>
       </c>
       <c r="J23" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="24" spans="3:10" x14ac:dyDescent="0.35">
@@ -1643,13 +1658,13 @@
       <c r="D24" s="11"/>
       <c r="E24" s="2"/>
       <c r="H24" s="6" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="I24" s="13">
         <v>15</v>
       </c>
       <c r="J24" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="25" spans="3:10" x14ac:dyDescent="0.35">
@@ -1657,13 +1672,13 @@
       <c r="D25" s="11"/>
       <c r="E25" s="2"/>
       <c r="H25" s="6" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="I25" s="13">
         <v>25</v>
       </c>
       <c r="J25" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="26" spans="3:10" x14ac:dyDescent="0.35">
@@ -1671,13 +1686,13 @@
       <c r="D26" s="11"/>
       <c r="E26" s="2"/>
       <c r="H26" s="6" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="I26" s="13">
-        <v>23.332999999999998</v>
+        <v>26.25</v>
       </c>
       <c r="J26" s="8" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="27" spans="3:10" x14ac:dyDescent="0.35">
@@ -1685,13 +1700,13 @@
       <c r="D27" s="11"/>
       <c r="E27" s="2"/>
       <c r="H27" s="6" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="I27" s="13">
         <v>19.443999999999999</v>
       </c>
       <c r="J27" s="8" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="28" spans="3:10" x14ac:dyDescent="0.35">
@@ -1699,13 +1714,13 @@
       <c r="D28" s="11"/>
       <c r="E28" s="2"/>
       <c r="H28" s="6" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="I28" s="13">
         <v>1.5</v>
       </c>
       <c r="J28" s="8" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
     </row>
     <row r="29" spans="3:10" x14ac:dyDescent="0.35">
@@ -1713,13 +1728,13 @@
       <c r="D29" s="11"/>
       <c r="E29" s="2"/>
       <c r="H29" s="6" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="I29" s="13">
         <v>1.5</v>
       </c>
       <c r="J29" s="8" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
     </row>
     <row r="30" spans="3:10" x14ac:dyDescent="0.35">
@@ -1727,13 +1742,13 @@
       <c r="D30" s="11"/>
       <c r="E30" s="2"/>
       <c r="H30" s="6" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="I30" s="13">
         <v>2.25</v>
       </c>
       <c r="J30" s="8" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
     </row>
     <row r="31" spans="3:10" x14ac:dyDescent="0.35">
@@ -1741,13 +1756,13 @@
       <c r="D31" s="11"/>
       <c r="E31" s="2"/>
       <c r="H31" s="6" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="I31" s="13">
         <v>3</v>
       </c>
       <c r="J31" s="8" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
     </row>
     <row r="32" spans="3:10" x14ac:dyDescent="0.35">
@@ -1755,13 +1770,13 @@
       <c r="D32" s="11"/>
       <c r="E32" s="2"/>
       <c r="H32" s="6" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="I32" s="13">
         <v>6</v>
       </c>
       <c r="J32" s="8" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
     </row>
     <row r="33" spans="3:10" x14ac:dyDescent="0.35">
@@ -1769,13 +1784,13 @@
       <c r="D33" s="11"/>
       <c r="E33" s="2"/>
       <c r="H33" s="6" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="I33" s="13">
         <v>25</v>
       </c>
       <c r="J33" s="8" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
     </row>
     <row r="34" spans="3:10" x14ac:dyDescent="0.35">
@@ -1783,13 +1798,13 @@
       <c r="D34" s="11"/>
       <c r="E34" s="2"/>
       <c r="H34" s="6" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="I34" s="13">
         <v>20</v>
       </c>
       <c r="J34" s="8" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
     </row>
     <row r="35" spans="3:10" x14ac:dyDescent="0.35">
@@ -1797,13 +1812,13 @@
       <c r="D35" s="11"/>
       <c r="E35" s="2"/>
       <c r="H35" s="6" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="I35" s="13">
         <v>0.5</v>
       </c>
       <c r="J35" s="8" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
     </row>
     <row r="36" spans="3:10" x14ac:dyDescent="0.35">
@@ -1811,13 +1826,13 @@
       <c r="D36" s="11"/>
       <c r="E36" s="2"/>
       <c r="H36" s="6" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="I36" s="13">
         <v>0.5</v>
       </c>
       <c r="J36" s="8" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
     </row>
     <row r="37" spans="3:10" x14ac:dyDescent="0.35">
@@ -1825,13 +1840,13 @@
       <c r="D37" s="11"/>
       <c r="E37" s="2"/>
       <c r="H37" s="6" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="I37" s="13">
         <v>49.332999999999998</v>
       </c>
       <c r="J37" s="8" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
     </row>
     <row r="38" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -1839,35 +1854,35 @@
       <c r="D38" s="12"/>
       <c r="E38" s="3"/>
       <c r="H38" s="6" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="I38" s="13">
         <v>12</v>
       </c>
       <c r="J38" s="8" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
     </row>
     <row r="39" spans="3:10" x14ac:dyDescent="0.35">
       <c r="H39" s="6" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="I39" s="13">
         <v>200</v>
       </c>
       <c r="J39" s="8" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
     </row>
     <row r="40" spans="3:10" x14ac:dyDescent="0.35">
       <c r="H40" s="6" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="I40" s="13">
         <v>222</v>
       </c>
       <c r="J40" s="8" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
     </row>
     <row r="41" spans="3:10" x14ac:dyDescent="0.35">
@@ -1996,7 +2011,7 @@
         <v>9</v>
       </c>
       <c r="C2" s="27" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
     </row>
     <row r="3" spans="2:20" x14ac:dyDescent="0.35">
@@ -2028,7 +2043,7 @@
         <v>13</v>
       </c>
       <c r="C6" s="28" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
     </row>
     <row r="7" spans="2:20" x14ac:dyDescent="0.35">
@@ -2036,7 +2051,7 @@
         <v>14</v>
       </c>
       <c r="C7" s="28" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
     </row>
     <row r="8" spans="2:20" x14ac:dyDescent="0.35">
@@ -2052,22 +2067,22 @@
         <v>32</v>
       </c>
       <c r="C9" s="29" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="10" spans="2:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C10" s="26"/>
-      <c r="E10" s="39" t="s">
+      <c r="E10" s="43" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="40"/>
-      <c r="G10" s="41"/>
-      <c r="J10" s="39" t="s">
+      <c r="F10" s="44"/>
+      <c r="G10" s="45"/>
+      <c r="J10" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="K10" s="40"/>
-      <c r="L10" s="40"/>
-      <c r="M10" s="41"/>
+      <c r="K10" s="44"/>
+      <c r="L10" s="44"/>
+      <c r="M10" s="45"/>
     </row>
     <row r="11" spans="2:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C11" s="26"/>
@@ -2090,13 +2105,13 @@
         <v>24</v>
       </c>
       <c r="M11" s="38" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
     </row>
     <row r="12" spans="2:20" x14ac:dyDescent="0.35">
       <c r="C12" s="26"/>
       <c r="E12" s="4" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="F12" s="10">
         <v>300</v>
@@ -2105,7 +2120,7 @@
         <v>23</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="K12" s="10">
         <v>25</v>
@@ -2114,14 +2129,14 @@
         <v>8</v>
       </c>
       <c r="M12" s="22"/>
-      <c r="O12" s="42" t="s">
-        <v>132</v>
-      </c>
-      <c r="P12" s="42"/>
-      <c r="Q12" s="42"/>
-      <c r="R12" s="42"/>
-      <c r="S12" s="42"/>
-      <c r="T12" s="42"/>
+      <c r="O12" s="46" t="s">
+        <v>126</v>
+      </c>
+      <c r="P12" s="46"/>
+      <c r="Q12" s="46"/>
+      <c r="R12" s="46"/>
+      <c r="S12" s="46"/>
+      <c r="T12" s="46"/>
     </row>
     <row r="13" spans="2:20" x14ac:dyDescent="0.35">
       <c r="C13" s="26"/>
@@ -2135,7 +2150,7 @@
         <v>19</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="K13" s="11">
         <v>467.5</v>
@@ -2144,12 +2159,12 @@
         <v>25</v>
       </c>
       <c r="M13" s="2"/>
-      <c r="O13" s="42"/>
-      <c r="P13" s="42"/>
-      <c r="Q13" s="42"/>
-      <c r="R13" s="42"/>
-      <c r="S13" s="42"/>
-      <c r="T13" s="42"/>
+      <c r="O13" s="46"/>
+      <c r="P13" s="46"/>
+      <c r="Q13" s="46"/>
+      <c r="R13" s="46"/>
+      <c r="S13" s="46"/>
+      <c r="T13" s="46"/>
     </row>
     <row r="14" spans="2:20" x14ac:dyDescent="0.35">
       <c r="C14" s="26"/>
@@ -2166,12 +2181,12 @@
         <v>25</v>
       </c>
       <c r="M14" s="2"/>
-      <c r="O14" s="42"/>
-      <c r="P14" s="42"/>
-      <c r="Q14" s="42"/>
-      <c r="R14" s="42"/>
-      <c r="S14" s="42"/>
-      <c r="T14" s="42"/>
+      <c r="O14" s="46"/>
+      <c r="P14" s="46"/>
+      <c r="Q14" s="46"/>
+      <c r="R14" s="46"/>
+      <c r="S14" s="46"/>
+      <c r="T14" s="46"/>
     </row>
     <row r="15" spans="2:20" x14ac:dyDescent="0.35">
       <c r="C15" s="26"/>
@@ -2179,7 +2194,7 @@
       <c r="F15" s="11"/>
       <c r="G15" s="2"/>
       <c r="J15" s="4" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="K15" s="11">
         <v>20</v>
@@ -2188,12 +2203,12 @@
         <v>8</v>
       </c>
       <c r="M15" s="2"/>
-      <c r="O15" s="42"/>
-      <c r="P15" s="42"/>
-      <c r="Q15" s="42"/>
-      <c r="R15" s="42"/>
-      <c r="S15" s="42"/>
-      <c r="T15" s="42"/>
+      <c r="O15" s="46"/>
+      <c r="P15" s="46"/>
+      <c r="Q15" s="46"/>
+      <c r="R15" s="46"/>
+      <c r="S15" s="46"/>
+      <c r="T15" s="46"/>
     </row>
     <row r="16" spans="2:20" x14ac:dyDescent="0.35">
       <c r="C16" s="26"/>
@@ -2201,23 +2216,23 @@
       <c r="F16" s="11"/>
       <c r="G16" s="2"/>
       <c r="J16" s="4" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="K16" s="11">
         <v>7.5</v>
       </c>
       <c r="L16" s="4" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="M16" s="2"/>
-      <c r="O16" s="42" t="s">
-        <v>131</v>
-      </c>
-      <c r="P16" s="42"/>
-      <c r="Q16" s="42"/>
-      <c r="R16" s="42"/>
-      <c r="S16" s="42"/>
-      <c r="T16" s="42"/>
+      <c r="O16" s="46" t="s">
+        <v>125</v>
+      </c>
+      <c r="P16" s="46"/>
+      <c r="Q16" s="46"/>
+      <c r="R16" s="46"/>
+      <c r="S16" s="46"/>
+      <c r="T16" s="46"/>
     </row>
     <row r="17" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C17" s="26"/>
@@ -2231,15 +2246,15 @@
         <v>42</v>
       </c>
       <c r="L17" s="4" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="M17" s="2"/>
-      <c r="O17" s="42"/>
-      <c r="P17" s="42"/>
-      <c r="Q17" s="42"/>
-      <c r="R17" s="42"/>
-      <c r="S17" s="42"/>
-      <c r="T17" s="42"/>
+      <c r="O17" s="46"/>
+      <c r="P17" s="46"/>
+      <c r="Q17" s="46"/>
+      <c r="R17" s="46"/>
+      <c r="S17" s="46"/>
+      <c r="T17" s="46"/>
     </row>
     <row r="18" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C18" s="26"/>
@@ -2250,12 +2265,12 @@
       <c r="K18" s="11"/>
       <c r="L18" s="4"/>
       <c r="M18" s="2"/>
-      <c r="O18" s="42"/>
-      <c r="P18" s="42"/>
-      <c r="Q18" s="42"/>
-      <c r="R18" s="42"/>
-      <c r="S18" s="42"/>
-      <c r="T18" s="42"/>
+      <c r="O18" s="46"/>
+      <c r="P18" s="46"/>
+      <c r="Q18" s="46"/>
+      <c r="R18" s="46"/>
+      <c r="S18" s="46"/>
+      <c r="T18" s="46"/>
     </row>
     <row r="19" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C19" s="26"/>
@@ -2266,12 +2281,12 @@
       <c r="K19" s="11"/>
       <c r="L19" s="4"/>
       <c r="M19" s="2"/>
-      <c r="O19" s="42"/>
-      <c r="P19" s="42"/>
-      <c r="Q19" s="42"/>
-      <c r="R19" s="42"/>
-      <c r="S19" s="42"/>
-      <c r="T19" s="42"/>
+      <c r="O19" s="46"/>
+      <c r="P19" s="46"/>
+      <c r="Q19" s="46"/>
+      <c r="R19" s="46"/>
+      <c r="S19" s="46"/>
+      <c r="T19" s="46"/>
     </row>
     <row r="20" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C20" s="26"/>
@@ -2547,7 +2562,7 @@
         <v>9</v>
       </c>
       <c r="C2" s="27" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
     </row>
     <row r="3" spans="2:12" ht="87" x14ac:dyDescent="0.35">
@@ -2555,7 +2570,7 @@
         <v>10</v>
       </c>
       <c r="C3" s="31" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.35">
@@ -2579,7 +2594,7 @@
         <v>13</v>
       </c>
       <c r="C6" s="28" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.35">
@@ -2587,7 +2602,7 @@
         <v>14</v>
       </c>
       <c r="C7" s="28" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.35">
@@ -2595,7 +2610,7 @@
         <v>31</v>
       </c>
       <c r="C8" s="28" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
     </row>
     <row r="9" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -2603,21 +2618,21 @@
         <v>32</v>
       </c>
       <c r="C9" s="29" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
     </row>
     <row r="10" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C10" s="26"/>
-      <c r="E10" s="39" t="s">
+      <c r="E10" s="43" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="40"/>
-      <c r="G10" s="41"/>
-      <c r="J10" s="39" t="s">
+      <c r="F10" s="44"/>
+      <c r="G10" s="45"/>
+      <c r="J10" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="K10" s="40"/>
-      <c r="L10" s="41"/>
+      <c r="K10" s="44"/>
+      <c r="L10" s="45"/>
     </row>
     <row r="11" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C11" s="26"/>
@@ -2643,16 +2658,16 @@
     <row r="12" spans="2:12" x14ac:dyDescent="0.35">
       <c r="C12" s="26"/>
       <c r="E12" s="4" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="F12" s="10">
         <v>18.75</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="K12" s="10">
         <v>0.5</v>
@@ -2670,10 +2685,10 @@
         <v>28.625</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="K13" s="11">
         <v>0.5</v>
@@ -2721,7 +2736,7 @@
         <v>42</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="J16" s="4"/>
       <c r="K16" s="11"/>
@@ -2730,13 +2745,13 @@
     <row r="17" spans="3:12" x14ac:dyDescent="0.35">
       <c r="C17" s="26"/>
       <c r="E17" s="2" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="F17" s="11">
         <v>7.5</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="J17" s="4"/>
       <c r="K17" s="11"/>
@@ -3008,7 +3023,7 @@
         <v>9</v>
       </c>
       <c r="C2" s="27" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.35">
@@ -3040,7 +3055,7 @@
         <v>13</v>
       </c>
       <c r="C6" s="28" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.35">
@@ -3048,7 +3063,7 @@
         <v>14</v>
       </c>
       <c r="C7" s="28" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.35">
@@ -3056,7 +3071,7 @@
         <v>31</v>
       </c>
       <c r="C8" s="28" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
     </row>
     <row r="9" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -3064,21 +3079,21 @@
         <v>32</v>
       </c>
       <c r="C9" s="29" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
     </row>
     <row r="10" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C10" s="26"/>
-      <c r="E10" s="39" t="s">
+      <c r="E10" s="43" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="40"/>
-      <c r="G10" s="41"/>
-      <c r="J10" s="39" t="s">
+      <c r="F10" s="44"/>
+      <c r="G10" s="45"/>
+      <c r="J10" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="K10" s="40"/>
-      <c r="L10" s="41"/>
+      <c r="K10" s="44"/>
+      <c r="L10" s="45"/>
     </row>
     <row r="11" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C11" s="26"/>
@@ -3104,16 +3119,16 @@
     <row r="12" spans="2:12" x14ac:dyDescent="0.35">
       <c r="C12" s="26"/>
       <c r="E12" s="4" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="F12" s="10">
         <v>600</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="K12" s="10">
         <v>49.332999999999998</v>
@@ -3125,16 +3140,16 @@
     <row r="13" spans="2:12" x14ac:dyDescent="0.35">
       <c r="C13" s="26"/>
       <c r="E13" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="F13" s="11">
         <v>1000</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="K13" s="11">
         <v>246.666</v>
@@ -3152,10 +3167,10 @@
         <v>400</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="K14" s="11">
         <v>12</v>
@@ -3173,10 +3188,10 @@
         <v>200</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="K15" s="11">
         <v>200</v>
@@ -3194,10 +3209,10 @@
         <v>240</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="K16" s="11">
         <v>222</v>
@@ -3215,11 +3230,17 @@
         <v>246.67</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="J17" s="4"/>
-      <c r="K17" s="11"/>
-      <c r="L17" s="4"/>
+        <v>139</v>
+      </c>
+      <c r="J17" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="K17" s="11">
+        <v>410</v>
+      </c>
+      <c r="L17" s="4" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="18" spans="3:12" x14ac:dyDescent="0.35">
       <c r="C18" s="26"/>
@@ -3488,16 +3509,16 @@
       <c r="D4" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="39" t="s">
+      <c r="F4" s="43" t="s">
         <v>15</v>
       </c>
-      <c r="G4" s="40"/>
-      <c r="H4" s="41"/>
-      <c r="K4" s="39" t="s">
+      <c r="G4" s="44"/>
+      <c r="H4" s="45"/>
+      <c r="K4" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="L4" s="40"/>
-      <c r="M4" s="41"/>
+      <c r="L4" s="44"/>
+      <c r="M4" s="45"/>
     </row>
     <row r="5" spans="3:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C5" s="20" t="s">
@@ -3909,7 +3930,7 @@
         <v>11</v>
       </c>
       <c r="D6" s="33" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7" spans="3:20" x14ac:dyDescent="0.35">
@@ -3954,17 +3975,17 @@
     </row>
     <row r="12" spans="3:20" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="13" spans="3:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="F13" s="39" t="s">
+      <c r="F13" s="43" t="s">
         <v>15</v>
       </c>
-      <c r="G13" s="40"/>
-      <c r="H13" s="41"/>
-      <c r="K13" s="39" t="s">
+      <c r="G13" s="44"/>
+      <c r="H13" s="45"/>
+      <c r="K13" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="L13" s="40"/>
-      <c r="M13" s="40"/>
-      <c r="N13" s="41"/>
+      <c r="L13" s="44"/>
+      <c r="M13" s="44"/>
+      <c r="N13" s="45"/>
     </row>
     <row r="14" spans="3:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="F14" s="17" t="s">
@@ -3986,15 +4007,15 @@
         <v>24</v>
       </c>
       <c r="N14" s="38" t="s">
-        <v>123</v>
-      </c>
-      <c r="P14" s="42" t="s">
-        <v>126</v>
-      </c>
-      <c r="Q14" s="42"/>
-      <c r="R14" s="42"/>
-      <c r="S14" s="42"/>
-      <c r="T14" s="42"/>
+        <v>117</v>
+      </c>
+      <c r="P14" s="46" t="s">
+        <v>120</v>
+      </c>
+      <c r="Q14" s="46"/>
+      <c r="R14" s="46"/>
+      <c r="S14" s="46"/>
+      <c r="T14" s="46"/>
     </row>
     <row r="15" spans="3:20" x14ac:dyDescent="0.35">
       <c r="F15" s="4" t="s">
@@ -4016,11 +4037,11 @@
         <v>25</v>
       </c>
       <c r="N15" s="22"/>
-      <c r="P15" s="42"/>
-      <c r="Q15" s="42"/>
-      <c r="R15" s="42"/>
-      <c r="S15" s="42"/>
-      <c r="T15" s="42"/>
+      <c r="P15" s="46"/>
+      <c r="Q15" s="46"/>
+      <c r="R15" s="46"/>
+      <c r="S15" s="46"/>
+      <c r="T15" s="46"/>
     </row>
     <row r="16" spans="3:20" x14ac:dyDescent="0.35">
       <c r="F16" s="2" t="s">
@@ -4039,16 +4060,16 @@
         <v>960</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="P16" s="42"/>
-      <c r="Q16" s="42"/>
-      <c r="R16" s="42"/>
-      <c r="S16" s="42"/>
-      <c r="T16" s="42"/>
+        <v>122</v>
+      </c>
+      <c r="P16" s="46"/>
+      <c r="Q16" s="46"/>
+      <c r="R16" s="46"/>
+      <c r="S16" s="46"/>
+      <c r="T16" s="46"/>
     </row>
     <row r="17" spans="6:20" x14ac:dyDescent="0.35">
       <c r="F17" s="2"/>
@@ -4061,16 +4082,16 @@
         <v>111.25</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="P17" s="42"/>
-      <c r="Q17" s="42"/>
-      <c r="R17" s="42"/>
-      <c r="S17" s="42"/>
-      <c r="T17" s="42"/>
+        <v>121</v>
+      </c>
+      <c r="P17" s="46"/>
+      <c r="Q17" s="46"/>
+      <c r="R17" s="46"/>
+      <c r="S17" s="46"/>
+      <c r="T17" s="46"/>
     </row>
     <row r="18" spans="6:20" x14ac:dyDescent="0.35">
       <c r="F18" s="2"/>
@@ -4083,10 +4104,10 @@
         <v>37.5</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
     </row>
     <row r="19" spans="6:20" x14ac:dyDescent="0.35">
@@ -4094,16 +4115,16 @@
       <c r="G19" s="11"/>
       <c r="H19" s="2"/>
       <c r="K19" s="4" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="L19" s="11">
         <v>234.25</v>
       </c>
       <c r="M19" s="2" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="N19" s="2" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
     </row>
     <row r="20" spans="6:20" x14ac:dyDescent="0.35">
@@ -4414,7 +4435,7 @@
         <v>11</v>
       </c>
       <c r="C4" s="34" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
     </row>
     <row r="5" spans="2:20" x14ac:dyDescent="0.35">
@@ -4462,17 +4483,17 @@
     </row>
     <row r="11" spans="2:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C11" s="26"/>
-      <c r="E11" s="39" t="s">
+      <c r="E11" s="43" t="s">
         <v>15</v>
       </c>
-      <c r="F11" s="40"/>
-      <c r="G11" s="41"/>
-      <c r="J11" s="39" t="s">
+      <c r="F11" s="44"/>
+      <c r="G11" s="45"/>
+      <c r="J11" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="K11" s="40"/>
-      <c r="L11" s="40"/>
-      <c r="M11" s="41"/>
+      <c r="K11" s="44"/>
+      <c r="L11" s="44"/>
+      <c r="M11" s="45"/>
     </row>
     <row r="12" spans="2:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C12" s="26"/>
@@ -4495,16 +4516,16 @@
         <v>24</v>
       </c>
       <c r="M12" s="38" t="s">
-        <v>123</v>
-      </c>
-      <c r="O12" s="42" t="s">
-        <v>104</v>
-      </c>
-      <c r="P12" s="42"/>
-      <c r="Q12" s="42"/>
-      <c r="R12" s="42"/>
-      <c r="S12" s="42"/>
-      <c r="T12" s="42"/>
+        <v>117</v>
+      </c>
+      <c r="O12" s="46" t="s">
+        <v>98</v>
+      </c>
+      <c r="P12" s="46"/>
+      <c r="Q12" s="46"/>
+      <c r="R12" s="46"/>
+      <c r="S12" s="46"/>
+      <c r="T12" s="46"/>
     </row>
     <row r="13" spans="2:20" x14ac:dyDescent="0.35">
       <c r="C13" s="26"/>
@@ -4527,12 +4548,12 @@
         <v>25</v>
       </c>
       <c r="M13" s="22"/>
-      <c r="O13" s="42"/>
-      <c r="P13" s="42"/>
-      <c r="Q13" s="42"/>
-      <c r="R13" s="42"/>
-      <c r="S13" s="42"/>
-      <c r="T13" s="42"/>
+      <c r="O13" s="46"/>
+      <c r="P13" s="46"/>
+      <c r="Q13" s="46"/>
+      <c r="R13" s="46"/>
+      <c r="S13" s="46"/>
+      <c r="T13" s="46"/>
     </row>
     <row r="14" spans="2:20" x14ac:dyDescent="0.35">
       <c r="C14" s="26"/>
@@ -4552,17 +4573,17 @@
         <v>142.5</v>
       </c>
       <c r="L14" s="6" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="O14" s="42"/>
-      <c r="P14" s="42"/>
-      <c r="Q14" s="42"/>
-      <c r="R14" s="42"/>
-      <c r="S14" s="42"/>
-      <c r="T14" s="42"/>
+        <v>119</v>
+      </c>
+      <c r="O14" s="46"/>
+      <c r="P14" s="46"/>
+      <c r="Q14" s="46"/>
+      <c r="R14" s="46"/>
+      <c r="S14" s="46"/>
+      <c r="T14" s="46"/>
     </row>
     <row r="15" spans="2:20" x14ac:dyDescent="0.35">
       <c r="C15" s="26"/>
@@ -4576,17 +4597,17 @@
         <v>104.65</v>
       </c>
       <c r="L15" s="6" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="O15" s="42"/>
-      <c r="P15" s="42"/>
-      <c r="Q15" s="42"/>
-      <c r="R15" s="42"/>
-      <c r="S15" s="42"/>
-      <c r="T15" s="42"/>
+        <v>119</v>
+      </c>
+      <c r="O15" s="46"/>
+      <c r="P15" s="46"/>
+      <c r="Q15" s="46"/>
+      <c r="R15" s="46"/>
+      <c r="S15" s="46"/>
+      <c r="T15" s="46"/>
     </row>
     <row r="16" spans="2:20" x14ac:dyDescent="0.35">
       <c r="C16" s="26"/>
@@ -4600,19 +4621,19 @@
         <v>113.833</v>
       </c>
       <c r="L16" s="6" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="O16" s="42" t="s">
-        <v>121</v>
-      </c>
-      <c r="P16" s="42"/>
-      <c r="Q16" s="42"/>
-      <c r="R16" s="42"/>
-      <c r="S16" s="42"/>
-      <c r="T16" s="42"/>
+        <v>118</v>
+      </c>
+      <c r="O16" s="46" t="s">
+        <v>115</v>
+      </c>
+      <c r="P16" s="46"/>
+      <c r="Q16" s="46"/>
+      <c r="R16" s="46"/>
+      <c r="S16" s="46"/>
+      <c r="T16" s="46"/>
     </row>
     <row r="17" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C17" s="26"/>
@@ -4626,17 +4647,17 @@
         <v>246.67</v>
       </c>
       <c r="L17" s="6" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="O17" s="42"/>
-      <c r="P17" s="42"/>
-      <c r="Q17" s="42"/>
-      <c r="R17" s="42"/>
-      <c r="S17" s="42"/>
-      <c r="T17" s="42"/>
+        <v>135</v>
+      </c>
+      <c r="O17" s="46"/>
+      <c r="P17" s="46"/>
+      <c r="Q17" s="46"/>
+      <c r="R17" s="46"/>
+      <c r="S17" s="46"/>
+      <c r="T17" s="46"/>
     </row>
     <row r="18" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C18" s="26"/>
@@ -4647,12 +4668,12 @@
       <c r="K18" s="11"/>
       <c r="L18" s="6"/>
       <c r="M18" s="2"/>
-      <c r="O18" s="42"/>
-      <c r="P18" s="42"/>
-      <c r="Q18" s="42"/>
-      <c r="R18" s="42"/>
-      <c r="S18" s="42"/>
-      <c r="T18" s="42"/>
+      <c r="O18" s="46"/>
+      <c r="P18" s="46"/>
+      <c r="Q18" s="46"/>
+      <c r="R18" s="46"/>
+      <c r="S18" s="46"/>
+      <c r="T18" s="46"/>
     </row>
     <row r="19" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C19" s="26"/>
@@ -4663,14 +4684,14 @@
       <c r="K19" s="11"/>
       <c r="L19" s="6"/>
       <c r="M19" s="2"/>
-      <c r="O19" s="42"/>
-      <c r="P19" s="42"/>
-      <c r="Q19" s="42"/>
-      <c r="R19" s="42"/>
-      <c r="S19" s="42"/>
-      <c r="T19" s="42"/>
-    </row>
-    <row r="20" spans="3:20" x14ac:dyDescent="0.35">
+      <c r="O19" s="46"/>
+      <c r="P19" s="46"/>
+      <c r="Q19" s="46"/>
+      <c r="R19" s="46"/>
+      <c r="S19" s="46"/>
+      <c r="T19" s="46"/>
+    </row>
+    <row r="20" spans="3:20" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C20" s="26"/>
       <c r="E20" s="2"/>
       <c r="F20" s="11"/>
@@ -4679,14 +4700,6 @@
       <c r="K20" s="11"/>
       <c r="L20" s="6"/>
       <c r="M20" s="2"/>
-      <c r="O20" s="42" t="s">
-        <v>140</v>
-      </c>
-      <c r="P20" s="42"/>
-      <c r="Q20" s="42"/>
-      <c r="R20" s="42"/>
-      <c r="S20" s="42"/>
-      <c r="T20" s="42"/>
     </row>
     <row r="21" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C21" s="26"/>
@@ -4697,12 +4710,14 @@
       <c r="K21" s="11"/>
       <c r="L21" s="6"/>
       <c r="M21" s="2"/>
-      <c r="O21" s="42"/>
-      <c r="P21" s="42"/>
-      <c r="Q21" s="42"/>
-      <c r="R21" s="42"/>
-      <c r="S21" s="42"/>
-      <c r="T21" s="42"/>
+      <c r="O21" s="47" t="s">
+        <v>155</v>
+      </c>
+      <c r="P21" s="47"/>
+      <c r="Q21" s="47"/>
+      <c r="R21" s="47"/>
+      <c r="S21" s="47"/>
+      <c r="T21" s="47"/>
     </row>
     <row r="22" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C22" s="26"/>
@@ -4713,12 +4728,6 @@
       <c r="K22" s="11"/>
       <c r="L22" s="6"/>
       <c r="M22" s="2"/>
-      <c r="O22" s="42"/>
-      <c r="P22" s="42"/>
-      <c r="Q22" s="42"/>
-      <c r="R22" s="42"/>
-      <c r="S22" s="42"/>
-      <c r="T22" s="42"/>
     </row>
     <row r="23" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C23" s="26"/>
@@ -4729,12 +4738,14 @@
       <c r="K23" s="11"/>
       <c r="L23" s="6"/>
       <c r="M23" s="2"/>
-      <c r="O23" s="42"/>
-      <c r="P23" s="42"/>
-      <c r="Q23" s="42"/>
-      <c r="R23" s="42"/>
-      <c r="S23" s="42"/>
-      <c r="T23" s="42"/>
+      <c r="O23" s="46" t="s">
+        <v>156</v>
+      </c>
+      <c r="P23" s="46"/>
+      <c r="Q23" s="46"/>
+      <c r="R23" s="46"/>
+      <c r="S23" s="46"/>
+      <c r="T23" s="46"/>
     </row>
     <row r="24" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C24" s="26"/>
@@ -4745,6 +4756,12 @@
       <c r="K24" s="11"/>
       <c r="L24" s="6"/>
       <c r="M24" s="2"/>
+      <c r="O24" s="46"/>
+      <c r="P24" s="46"/>
+      <c r="Q24" s="46"/>
+      <c r="R24" s="46"/>
+      <c r="S24" s="46"/>
+      <c r="T24" s="46"/>
     </row>
     <row r="25" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C25" s="26"/>
@@ -4755,6 +4772,12 @@
       <c r="K25" s="11"/>
       <c r="L25" s="6"/>
       <c r="M25" s="2"/>
+      <c r="O25" s="46"/>
+      <c r="P25" s="46"/>
+      <c r="Q25" s="46"/>
+      <c r="R25" s="46"/>
+      <c r="S25" s="46"/>
+      <c r="T25" s="46"/>
     </row>
     <row r="26" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C26" s="26"/>
@@ -4765,6 +4788,12 @@
       <c r="K26" s="11"/>
       <c r="L26" s="6"/>
       <c r="M26" s="2"/>
+      <c r="O26" s="46"/>
+      <c r="P26" s="46"/>
+      <c r="Q26" s="46"/>
+      <c r="R26" s="46"/>
+      <c r="S26" s="46"/>
+      <c r="T26" s="46"/>
     </row>
     <row r="27" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C27" s="26"/>
@@ -4948,12 +4977,13 @@
       <c r="M45" s="3"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="E11:G11"/>
     <mergeCell ref="O12:T15"/>
     <mergeCell ref="O16:T19"/>
     <mergeCell ref="J11:M11"/>
-    <mergeCell ref="O20:T23"/>
+    <mergeCell ref="O23:T26"/>
+    <mergeCell ref="O21:T21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4996,7 +5026,7 @@
         <v>11</v>
       </c>
       <c r="C4" s="34" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.35">
@@ -5012,7 +5042,7 @@
         <v>13</v>
       </c>
       <c r="C6" s="28" t="s">
-        <v>51</v>
+        <v>148</v>
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.35">
@@ -5020,7 +5050,7 @@
         <v>14</v>
       </c>
       <c r="C7" s="28" t="s">
-        <v>52</v>
+        <v>149</v>
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.35">
@@ -5028,7 +5058,7 @@
         <v>31</v>
       </c>
       <c r="C8" s="28" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -5036,7 +5066,7 @@
         <v>32</v>
       </c>
       <c r="C9" s="29" t="s">
-        <v>53</v>
+        <v>150</v>
       </c>
     </row>
     <row r="10" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -5044,16 +5074,16 @@
     </row>
     <row r="11" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C11" s="26"/>
-      <c r="E11" s="39" t="s">
+      <c r="E11" s="43" t="s">
         <v>15</v>
       </c>
-      <c r="F11" s="40"/>
-      <c r="G11" s="41"/>
-      <c r="J11" s="39" t="s">
+      <c r="F11" s="44"/>
+      <c r="G11" s="45"/>
+      <c r="J11" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="K11" s="40"/>
-      <c r="L11" s="41"/>
+      <c r="K11" s="44"/>
+      <c r="L11" s="45"/>
     </row>
     <row r="12" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C12" s="26"/>
@@ -5079,19 +5109,19 @@
     <row r="13" spans="2:12" x14ac:dyDescent="0.35">
       <c r="C13" s="26"/>
       <c r="E13" s="4" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F13" s="10">
-        <v>480</v>
+        <v>576</v>
       </c>
       <c r="G13" s="4" t="s">
         <v>21</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="K13" s="10">
-        <v>204</v>
+        <v>252</v>
       </c>
       <c r="L13" s="4" t="s">
         <v>25</v>
@@ -5103,19 +5133,19 @@
         <v>19</v>
       </c>
       <c r="F14" s="11">
-        <v>480</v>
+        <v>576</v>
       </c>
       <c r="G14" s="4" t="s">
         <v>22</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="K14" s="11">
         <v>18</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.35">
@@ -5124,13 +5154,13 @@
       <c r="F15" s="11"/>
       <c r="G15" s="2"/>
       <c r="J15" s="4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="K15" s="11">
         <v>18</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.35">
@@ -5424,18 +5454,18 @@
         <v>9</v>
       </c>
       <c r="C2" s="27" t="s">
-        <v>58</v>
-      </c>
-      <c r="E2" s="39" t="s">
+        <v>55</v>
+      </c>
+      <c r="E2" s="43" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="40"/>
-      <c r="G2" s="41"/>
-      <c r="J2" s="39" t="s">
+      <c r="F2" s="44"/>
+      <c r="G2" s="45"/>
+      <c r="J2" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="K2" s="40"/>
-      <c r="L2" s="41"/>
+      <c r="K2" s="44"/>
+      <c r="L2" s="45"/>
     </row>
     <row r="3" spans="2:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B3" s="24" t="s">
@@ -5462,21 +5492,21 @@
       <c r="L3" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="N3" s="42" t="s">
-        <v>90</v>
-      </c>
-      <c r="O3" s="42"/>
-      <c r="P3" s="42"/>
-      <c r="Q3" s="42"/>
-      <c r="R3" s="42"/>
-      <c r="S3" s="42"/>
+      <c r="N3" s="46" t="s">
+        <v>87</v>
+      </c>
+      <c r="O3" s="46"/>
+      <c r="P3" s="46"/>
+      <c r="Q3" s="46"/>
+      <c r="R3" s="46"/>
+      <c r="S3" s="46"/>
     </row>
     <row r="4" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B4" s="24" t="s">
         <v>11</v>
       </c>
       <c r="C4" s="28" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>41</v>
@@ -5488,7 +5518,7 @@
         <v>33</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="K4" s="10">
         <v>1140</v>
@@ -5496,12 +5526,12 @@
       <c r="L4" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="N4" s="42"/>
-      <c r="O4" s="42"/>
-      <c r="P4" s="42"/>
-      <c r="Q4" s="42"/>
-      <c r="R4" s="42"/>
-      <c r="S4" s="42"/>
+      <c r="N4" s="46"/>
+      <c r="O4" s="46"/>
+      <c r="P4" s="46"/>
+      <c r="Q4" s="46"/>
+      <c r="R4" s="46"/>
+      <c r="S4" s="46"/>
     </row>
     <row r="5" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B5" s="24" t="s">
@@ -5517,30 +5547,30 @@
         <v>960</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="K5" s="11">
         <v>300</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="N5" s="42"/>
-      <c r="O5" s="42"/>
-      <c r="P5" s="42"/>
-      <c r="Q5" s="42"/>
-      <c r="R5" s="42"/>
-      <c r="S5" s="42"/>
+        <v>81</v>
+      </c>
+      <c r="N5" s="46"/>
+      <c r="O5" s="46"/>
+      <c r="P5" s="46"/>
+      <c r="Q5" s="46"/>
+      <c r="R5" s="46"/>
+      <c r="S5" s="46"/>
     </row>
     <row r="6" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B6" s="24" t="s">
         <v>13</v>
       </c>
       <c r="C6" s="28" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E6" s="2"/>
       <c r="F6" s="11"/>
@@ -5548,19 +5578,19 @@
       <c r="J6" s="4"/>
       <c r="K6" s="11"/>
       <c r="L6" s="2"/>
-      <c r="N6" s="42"/>
-      <c r="O6" s="42"/>
-      <c r="P6" s="42"/>
-      <c r="Q6" s="42"/>
-      <c r="R6" s="42"/>
-      <c r="S6" s="42"/>
+      <c r="N6" s="46"/>
+      <c r="O6" s="46"/>
+      <c r="P6" s="46"/>
+      <c r="Q6" s="46"/>
+      <c r="R6" s="46"/>
+      <c r="S6" s="46"/>
     </row>
     <row r="7" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B7" s="24" t="s">
         <v>14</v>
       </c>
       <c r="C7" s="28" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E7" s="2"/>
       <c r="F7" s="11"/>
@@ -5574,7 +5604,7 @@
         <v>31</v>
       </c>
       <c r="C8" s="28" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="E8" s="2"/>
       <c r="F8" s="11"/>
@@ -5588,7 +5618,7 @@
         <v>32</v>
       </c>
       <c r="C9" s="29" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="E9" s="2"/>
       <c r="F9" s="11"/>
@@ -5871,7 +5901,7 @@
         <v>9</v>
       </c>
       <c r="C2" s="27" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3" spans="2:12" ht="46" customHeight="1" x14ac:dyDescent="0.35">
@@ -5879,7 +5909,7 @@
         <v>10</v>
       </c>
       <c r="C3" s="31" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.35">
@@ -5903,7 +5933,7 @@
         <v>13</v>
       </c>
       <c r="C6" s="28" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.35">
@@ -5911,7 +5941,7 @@
         <v>14</v>
       </c>
       <c r="C7" s="28" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.35">
@@ -5919,7 +5949,7 @@
         <v>31</v>
       </c>
       <c r="C8" s="28" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
     </row>
     <row r="9" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -5927,21 +5957,21 @@
         <v>32</v>
       </c>
       <c r="C9" s="29" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="10" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C10" s="26"/>
-      <c r="E10" s="39" t="s">
+      <c r="E10" s="43" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="40"/>
-      <c r="G10" s="41"/>
-      <c r="J10" s="39" t="s">
+      <c r="F10" s="44"/>
+      <c r="G10" s="45"/>
+      <c r="J10" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="K10" s="40"/>
-      <c r="L10" s="41"/>
+      <c r="K10" s="44"/>
+      <c r="L10" s="45"/>
     </row>
     <row r="11" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C11" s="26"/>
@@ -5967,16 +5997,16 @@
     <row r="12" spans="2:12" x14ac:dyDescent="0.35">
       <c r="C12" s="26"/>
       <c r="E12" s="4" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="F12" s="10">
         <v>480</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="K12" s="10">
         <v>61.6875</v>
@@ -5994,10 +6024,10 @@
         <v>422.5</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="K13" s="11">
         <v>45</v>
@@ -6009,16 +6039,16 @@
     <row r="14" spans="2:12" x14ac:dyDescent="0.35">
       <c r="C14" s="26"/>
       <c r="E14" s="2" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="F14" s="11">
         <v>300</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="K14" s="11">
         <v>45</v>
@@ -6039,7 +6069,7 @@
         <v>44</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="K15" s="11">
         <v>33.125</v>
@@ -6060,7 +6090,7 @@
         <v>42</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="K16" s="11">
         <v>30</v>
@@ -6072,7 +6102,7 @@
     <row r="17" spans="3:12" x14ac:dyDescent="0.35">
       <c r="C17" s="26"/>
       <c r="E17" s="2" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F17" s="11">
         <v>18</v>
@@ -6081,7 +6111,7 @@
         <v>50</v>
       </c>
       <c r="J17" s="4" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="K17" s="11">
         <v>30</v>
@@ -6096,7 +6126,7 @@
       <c r="F18" s="11"/>
       <c r="G18" s="2"/>
       <c r="J18" s="4" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="K18" s="11">
         <v>25</v>
@@ -6111,7 +6141,7 @@
       <c r="F19" s="11"/>
       <c r="G19" s="2"/>
       <c r="J19" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="K19" s="11">
         <v>22.5</v>
@@ -6126,7 +6156,7 @@
       <c r="F20" s="11"/>
       <c r="G20" s="2"/>
       <c r="J20" s="2" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="K20" s="11">
         <v>20.5</v>
@@ -6141,7 +6171,7 @@
       <c r="F21" s="11"/>
       <c r="G21" s="2"/>
       <c r="J21" s="2" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="K21" s="11">
         <v>15</v>
@@ -6156,7 +6186,7 @@
       <c r="F22" s="11"/>
       <c r="G22" s="2"/>
       <c r="J22" s="2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="K22" s="11">
         <v>7.3125</v>
@@ -6171,7 +6201,7 @@
       <c r="F23" s="11"/>
       <c r="G23" s="2"/>
       <c r="J23" s="2" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="K23" s="11">
         <v>7.25</v>
@@ -6186,7 +6216,7 @@
       <c r="F24" s="11"/>
       <c r="G24" s="2"/>
       <c r="J24" s="2" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="K24" s="11">
         <v>5</v>
@@ -6201,7 +6231,7 @@
       <c r="F25" s="11"/>
       <c r="G25" s="2"/>
       <c r="J25" s="2" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="K25" s="11">
         <v>3</v>
@@ -6216,7 +6246,7 @@
       <c r="F26" s="11"/>
       <c r="G26" s="2"/>
       <c r="J26" s="2" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="K26" s="11">
         <v>2.5</v>
@@ -6231,7 +6261,7 @@
       <c r="F27" s="11"/>
       <c r="G27" s="2"/>
       <c r="J27" s="2" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="K27" s="11">
         <v>2.25</v>
@@ -6246,7 +6276,7 @@
       <c r="F28" s="11"/>
       <c r="G28" s="2"/>
       <c r="J28" s="2" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="K28" s="11">
         <v>1.4065000000000001</v>
@@ -6261,7 +6291,7 @@
       <c r="F29" s="11"/>
       <c r="G29" s="2"/>
       <c r="J29" s="2" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="K29" s="11">
         <v>0.5</v>
@@ -6432,7 +6462,7 @@
         <v>9</v>
       </c>
       <c r="C2" s="27" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" spans="2:16" x14ac:dyDescent="0.35">
@@ -6448,7 +6478,7 @@
         <v>11</v>
       </c>
       <c r="C4" s="28" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
     </row>
     <row r="5" spans="2:16" x14ac:dyDescent="0.35">
@@ -6464,7 +6494,7 @@
         <v>13</v>
       </c>
       <c r="C6" s="28" t="s">
-        <v>95</v>
+        <v>152</v>
       </c>
     </row>
     <row r="7" spans="2:16" x14ac:dyDescent="0.35">
@@ -6472,7 +6502,7 @@
         <v>14</v>
       </c>
       <c r="C7" s="28" t="s">
-        <v>96</v>
+        <v>153</v>
       </c>
     </row>
     <row r="8" spans="2:16" x14ac:dyDescent="0.35">
@@ -6480,7 +6510,7 @@
         <v>31</v>
       </c>
       <c r="C8" s="28" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
     </row>
     <row r="9" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -6488,21 +6518,21 @@
         <v>32</v>
       </c>
       <c r="C9" s="29" t="s">
-        <v>98</v>
+        <v>154</v>
       </c>
     </row>
     <row r="10" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C10" s="26"/>
-      <c r="E10" s="39" t="s">
+      <c r="E10" s="43" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="40"/>
-      <c r="G10" s="41"/>
-      <c r="J10" s="39" t="s">
+      <c r="F10" s="44"/>
+      <c r="G10" s="45"/>
+      <c r="J10" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="K10" s="40"/>
-      <c r="L10" s="41"/>
+      <c r="K10" s="44"/>
+      <c r="L10" s="45"/>
     </row>
     <row r="11" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C11" s="26"/>
@@ -6525,46 +6555,46 @@
         <v>24</v>
       </c>
       <c r="P11" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
     </row>
     <row r="12" spans="2:16" x14ac:dyDescent="0.35">
       <c r="C12" s="26"/>
       <c r="E12" s="4" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="F12" s="10">
-        <v>1260</v>
+        <v>1380</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="K12" s="10">
-        <v>23.332999999999998</v>
+        <v>26.25</v>
       </c>
       <c r="L12" s="4" t="s">
         <v>8</v>
       </c>
       <c r="P12" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
     </row>
     <row r="13" spans="2:16" x14ac:dyDescent="0.35">
       <c r="C13" s="26"/>
       <c r="E13" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="F13" s="11">
         <v>500</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="K13" s="11">
         <v>19.443999999999999</v>
@@ -6579,16 +6609,16 @@
         <v>19</v>
       </c>
       <c r="F14" s="11">
-        <v>533.33299999999997</v>
+        <v>600</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="K14" s="11">
-        <v>669.33299999999997</v>
+        <v>759.75</v>
       </c>
       <c r="L14" s="4" t="s">
         <v>25</v>
@@ -6600,7 +6630,7 @@
       <c r="F15" s="11"/>
       <c r="G15" s="2"/>
       <c r="J15" s="4" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="K15" s="11">
         <v>635.40554999999995</v>
@@ -6615,13 +6645,13 @@
       <c r="F16" s="11"/>
       <c r="G16" s="2"/>
       <c r="J16" s="4" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="K16" s="11">
         <v>54</v>
       </c>
       <c r="L16" s="4" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
     </row>
     <row r="17" spans="3:12" x14ac:dyDescent="0.35">
@@ -6630,13 +6660,13 @@
       <c r="F17" s="11"/>
       <c r="G17" s="2"/>
       <c r="J17" s="4" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="K17" s="11">
         <v>45.15</v>
       </c>
       <c r="L17" s="4" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
     </row>
     <row r="18" spans="3:12" x14ac:dyDescent="0.35">
@@ -6904,7 +6934,7 @@
         <v>9</v>
       </c>
       <c r="C2" s="27" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.35">
@@ -6936,7 +6966,7 @@
         <v>13</v>
       </c>
       <c r="C6" s="28" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.35">
@@ -6944,7 +6974,7 @@
         <v>14</v>
       </c>
       <c r="C7" s="28" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.35">
@@ -6952,7 +6982,7 @@
         <v>31</v>
       </c>
       <c r="C8" s="28" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
     </row>
     <row r="9" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -6960,21 +6990,21 @@
         <v>32</v>
       </c>
       <c r="C9" s="29" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
     </row>
     <row r="10" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C10" s="26"/>
-      <c r="E10" s="39" t="s">
+      <c r="E10" s="43" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="40"/>
-      <c r="G10" s="41"/>
-      <c r="J10" s="39" t="s">
+      <c r="F10" s="44"/>
+      <c r="G10" s="45"/>
+      <c r="J10" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="K10" s="40"/>
-      <c r="L10" s="41"/>
+      <c r="K10" s="44"/>
+      <c r="L10" s="45"/>
     </row>
     <row r="11" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C11" s="26"/>
@@ -7000,7 +7030,7 @@
     <row r="12" spans="2:12" x14ac:dyDescent="0.35">
       <c r="C12" s="26"/>
       <c r="E12" s="4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F12" s="10">
         <v>18</v>
@@ -7009,7 +7039,7 @@
         <v>50</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="K12" s="10">
         <v>1.5</v>
@@ -7030,7 +7060,7 @@
         <v>33</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="K13" s="11">
         <v>1.5</v>
@@ -7048,10 +7078,10 @@
         <v>37.65</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="K14" s="11">
         <v>2.25</v>
@@ -7063,16 +7093,16 @@
     <row r="15" spans="2:12" x14ac:dyDescent="0.35">
       <c r="C15" s="26"/>
       <c r="E15" s="2" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="F15" s="11">
         <v>45.15</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="K15" s="11">
         <v>3</v>
@@ -7084,16 +7114,16 @@
     <row r="16" spans="2:12" x14ac:dyDescent="0.35">
       <c r="C16" s="26"/>
       <c r="E16" s="2" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="F16" s="11">
         <v>54</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="K16" s="11">
         <v>6</v>
@@ -7111,7 +7141,7 @@
         <v>104.65</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="J17" s="4"/>
       <c r="K17" s="11"/>

</xml_diff>

<commit_message>
Fixed error on spreadsheet
</commit_message>
<xml_diff>
--- a/Game Stuff/Spreadsheet.xlsx
+++ b/Game Stuff/Spreadsheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Nicos Blueprints_Phyrexian Datavault\Game Stuff\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDE4B23D-EA0A-4594-9859-6DBA38760E81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F15F8E50-39B7-4FEC-916E-ACB1662AFF3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{E9D95B66-7EA4-4203-9BE9-B35EAC251241}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" firstSheet="3" activeTab="11" xr2:uid="{E9D95B66-7EA4-4203-9BE9-B35EAC251241}"/>
   </bookViews>
   <sheets>
     <sheet name="Material Summary" sheetId="1" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="659" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="663" uniqueCount="176">
   <si>
     <t>Item</t>
   </si>
@@ -573,6 +573,9 @@
   </si>
   <si>
     <t>1.76 Hours</t>
+  </si>
+  <si>
+    <t>Empty Fluid Tank</t>
   </si>
 </sst>
 </file>
@@ -864,7 +867,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -944,6 +947,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -959,11 +968,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1312,18 +1318,18 @@
   <sheetData>
     <row r="3" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="4" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C4" s="39" t="s">
+      <c r="C4" s="41" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="40"/>
-      <c r="E4" s="41"/>
+      <c r="D4" s="42"/>
+      <c r="E4" s="43"/>
       <c r="F4" s="14"/>
       <c r="G4" s="14"/>
-      <c r="H4" s="39" t="s">
+      <c r="H4" s="41" t="s">
         <v>8</v>
       </c>
-      <c r="I4" s="40"/>
-      <c r="J4" s="41"/>
+      <c r="I4" s="42"/>
+      <c r="J4" s="43"/>
     </row>
     <row r="5" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C5" s="15" t="s">
@@ -1886,7 +1892,7 @@
         <v>140</v>
       </c>
       <c r="I39" s="11">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="J39" s="2" t="s">
         <v>134</v>
@@ -1904,7 +1910,7 @@
       </c>
     </row>
     <row r="41" spans="3:10" x14ac:dyDescent="0.35">
-      <c r="H41" s="11" t="s">
+      <c r="H41" s="46" t="s">
         <v>169</v>
       </c>
       <c r="I41" s="11">
@@ -1915,7 +1921,7 @@
       </c>
     </row>
     <row r="42" spans="3:10" x14ac:dyDescent="0.35">
-      <c r="H42" s="11" t="s">
+      <c r="H42" s="46" t="s">
         <v>170</v>
       </c>
       <c r="I42" s="11">
@@ -1926,9 +1932,15 @@
       </c>
     </row>
     <row r="43" spans="3:10" x14ac:dyDescent="0.35">
-      <c r="H43" s="2"/>
-      <c r="I43" s="11"/>
-      <c r="J43" s="2"/>
+      <c r="H43" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="I43" s="11">
+        <v>5</v>
+      </c>
+      <c r="J43" s="2" t="s">
+        <v>134</v>
+      </c>
     </row>
     <row r="44" spans="3:10" x14ac:dyDescent="0.35">
       <c r="H44" s="2"/>
@@ -2056,7 +2068,7 @@
       <c r="B4" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="44" t="s">
+      <c r="C4" s="39" t="s">
         <v>167</v>
       </c>
     </row>
@@ -2102,17 +2114,17 @@
     </row>
     <row r="10" spans="2:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C10" s="24"/>
-      <c r="E10" s="39" t="s">
+      <c r="E10" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="40"/>
-      <c r="G10" s="41"/>
-      <c r="J10" s="39" t="s">
+      <c r="F10" s="42"/>
+      <c r="G10" s="43"/>
+      <c r="J10" s="41" t="s">
         <v>16</v>
       </c>
-      <c r="K10" s="40"/>
-      <c r="L10" s="40"/>
-      <c r="M10" s="41"/>
+      <c r="K10" s="42"/>
+      <c r="L10" s="42"/>
+      <c r="M10" s="43"/>
     </row>
     <row r="11" spans="2:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C11" s="24"/>
@@ -2159,14 +2171,14 @@
         <v>8</v>
       </c>
       <c r="M12" s="20"/>
-      <c r="O12" s="42" t="s">
+      <c r="O12" s="44" t="s">
         <v>124</v>
       </c>
-      <c r="P12" s="42"/>
-      <c r="Q12" s="42"/>
-      <c r="R12" s="42"/>
-      <c r="S12" s="42"/>
-      <c r="T12" s="42"/>
+      <c r="P12" s="44"/>
+      <c r="Q12" s="44"/>
+      <c r="R12" s="44"/>
+      <c r="S12" s="44"/>
+      <c r="T12" s="44"/>
     </row>
     <row r="13" spans="2:20" x14ac:dyDescent="0.35">
       <c r="C13" s="24"/>
@@ -2189,12 +2201,12 @@
         <v>25</v>
       </c>
       <c r="M13" s="2"/>
-      <c r="O13" s="42"/>
-      <c r="P13" s="42"/>
-      <c r="Q13" s="42"/>
-      <c r="R13" s="42"/>
-      <c r="S13" s="42"/>
-      <c r="T13" s="42"/>
+      <c r="O13" s="44"/>
+      <c r="P13" s="44"/>
+      <c r="Q13" s="44"/>
+      <c r="R13" s="44"/>
+      <c r="S13" s="44"/>
+      <c r="T13" s="44"/>
     </row>
     <row r="14" spans="2:20" x14ac:dyDescent="0.35">
       <c r="C14" s="24"/>
@@ -2211,12 +2223,12 @@
         <v>25</v>
       </c>
       <c r="M14" s="2"/>
-      <c r="O14" s="42"/>
-      <c r="P14" s="42"/>
-      <c r="Q14" s="42"/>
-      <c r="R14" s="42"/>
-      <c r="S14" s="42"/>
-      <c r="T14" s="42"/>
+      <c r="O14" s="44"/>
+      <c r="P14" s="44"/>
+      <c r="Q14" s="44"/>
+      <c r="R14" s="44"/>
+      <c r="S14" s="44"/>
+      <c r="T14" s="44"/>
     </row>
     <row r="15" spans="2:20" x14ac:dyDescent="0.35">
       <c r="C15" s="24"/>
@@ -2233,12 +2245,12 @@
         <v>8</v>
       </c>
       <c r="M15" s="2"/>
-      <c r="O15" s="42"/>
-      <c r="P15" s="42"/>
-      <c r="Q15" s="42"/>
-      <c r="R15" s="42"/>
-      <c r="S15" s="42"/>
-      <c r="T15" s="42"/>
+      <c r="O15" s="44"/>
+      <c r="P15" s="44"/>
+      <c r="Q15" s="44"/>
+      <c r="R15" s="44"/>
+      <c r="S15" s="44"/>
+      <c r="T15" s="44"/>
     </row>
     <row r="16" spans="2:20" x14ac:dyDescent="0.35">
       <c r="C16" s="24"/>
@@ -2255,14 +2267,14 @@
         <v>114</v>
       </c>
       <c r="M16" s="2"/>
-      <c r="O16" s="42" t="s">
+      <c r="O16" s="44" t="s">
         <v>123</v>
       </c>
-      <c r="P16" s="42"/>
-      <c r="Q16" s="42"/>
-      <c r="R16" s="42"/>
-      <c r="S16" s="42"/>
-      <c r="T16" s="42"/>
+      <c r="P16" s="44"/>
+      <c r="Q16" s="44"/>
+      <c r="R16" s="44"/>
+      <c r="S16" s="44"/>
+      <c r="T16" s="44"/>
     </row>
     <row r="17" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C17" s="24"/>
@@ -2279,12 +2291,12 @@
         <v>114</v>
       </c>
       <c r="M17" s="2"/>
-      <c r="O17" s="42"/>
-      <c r="P17" s="42"/>
-      <c r="Q17" s="42"/>
-      <c r="R17" s="42"/>
-      <c r="S17" s="42"/>
-      <c r="T17" s="42"/>
+      <c r="O17" s="44"/>
+      <c r="P17" s="44"/>
+      <c r="Q17" s="44"/>
+      <c r="R17" s="44"/>
+      <c r="S17" s="44"/>
+      <c r="T17" s="44"/>
     </row>
     <row r="18" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C18" s="24"/>
@@ -2301,12 +2313,12 @@
         <v>154</v>
       </c>
       <c r="M18" s="2"/>
-      <c r="O18" s="42"/>
-      <c r="P18" s="42"/>
-      <c r="Q18" s="42"/>
-      <c r="R18" s="42"/>
-      <c r="S18" s="42"/>
-      <c r="T18" s="42"/>
+      <c r="O18" s="44"/>
+      <c r="P18" s="44"/>
+      <c r="Q18" s="44"/>
+      <c r="R18" s="44"/>
+      <c r="S18" s="44"/>
+      <c r="T18" s="44"/>
     </row>
     <row r="19" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C19" s="24"/>
@@ -2323,12 +2335,12 @@
         <v>154</v>
       </c>
       <c r="M19" s="2"/>
-      <c r="O19" s="42"/>
-      <c r="P19" s="42"/>
-      <c r="Q19" s="42"/>
-      <c r="R19" s="42"/>
-      <c r="S19" s="42"/>
-      <c r="T19" s="42"/>
+      <c r="O19" s="44"/>
+      <c r="P19" s="44"/>
+      <c r="Q19" s="44"/>
+      <c r="R19" s="44"/>
+      <c r="S19" s="44"/>
+      <c r="T19" s="44"/>
     </row>
     <row r="20" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C20" s="24"/>
@@ -2349,14 +2361,14 @@
       <c r="K21" s="9"/>
       <c r="L21" s="4"/>
       <c r="M21" s="2"/>
-      <c r="O21" s="43" t="s">
+      <c r="O21" s="45" t="s">
         <v>153</v>
       </c>
-      <c r="P21" s="43"/>
-      <c r="Q21" s="43"/>
-      <c r="R21" s="43"/>
-      <c r="S21" s="43"/>
-      <c r="T21" s="43"/>
+      <c r="P21" s="45"/>
+      <c r="Q21" s="45"/>
+      <c r="R21" s="45"/>
+      <c r="S21" s="45"/>
+      <c r="T21" s="45"/>
     </row>
     <row r="22" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C22" s="24"/>
@@ -2377,14 +2389,14 @@
       <c r="K23" s="9"/>
       <c r="L23" s="4"/>
       <c r="M23" s="2"/>
-      <c r="O23" s="42" t="s">
+      <c r="O23" s="44" t="s">
         <v>156</v>
       </c>
-      <c r="P23" s="42"/>
-      <c r="Q23" s="42"/>
-      <c r="R23" s="42"/>
-      <c r="S23" s="42"/>
-      <c r="T23" s="42"/>
+      <c r="P23" s="44"/>
+      <c r="Q23" s="44"/>
+      <c r="R23" s="44"/>
+      <c r="S23" s="44"/>
+      <c r="T23" s="44"/>
     </row>
     <row r="24" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C24" s="24"/>
@@ -2395,12 +2407,12 @@
       <c r="K24" s="9"/>
       <c r="L24" s="4"/>
       <c r="M24" s="2"/>
-      <c r="O24" s="42"/>
-      <c r="P24" s="42"/>
-      <c r="Q24" s="42"/>
-      <c r="R24" s="42"/>
-      <c r="S24" s="42"/>
-      <c r="T24" s="42"/>
+      <c r="O24" s="44"/>
+      <c r="P24" s="44"/>
+      <c r="Q24" s="44"/>
+      <c r="R24" s="44"/>
+      <c r="S24" s="44"/>
+      <c r="T24" s="44"/>
     </row>
     <row r="25" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C25" s="24"/>
@@ -2411,12 +2423,12 @@
       <c r="K25" s="9"/>
       <c r="L25" s="4"/>
       <c r="M25" s="2"/>
-      <c r="O25" s="42"/>
-      <c r="P25" s="42"/>
-      <c r="Q25" s="42"/>
-      <c r="R25" s="42"/>
-      <c r="S25" s="42"/>
-      <c r="T25" s="42"/>
+      <c r="O25" s="44"/>
+      <c r="P25" s="44"/>
+      <c r="Q25" s="44"/>
+      <c r="R25" s="44"/>
+      <c r="S25" s="44"/>
+      <c r="T25" s="44"/>
     </row>
     <row r="26" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C26" s="24"/>
@@ -2427,12 +2439,12 @@
       <c r="K26" s="9"/>
       <c r="L26" s="4"/>
       <c r="M26" s="2"/>
-      <c r="O26" s="42"/>
-      <c r="P26" s="42"/>
-      <c r="Q26" s="42"/>
-      <c r="R26" s="42"/>
-      <c r="S26" s="42"/>
-      <c r="T26" s="42"/>
+      <c r="O26" s="44"/>
+      <c r="P26" s="44"/>
+      <c r="Q26" s="44"/>
+      <c r="R26" s="44"/>
+      <c r="S26" s="44"/>
+      <c r="T26" s="44"/>
     </row>
     <row r="27" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C27" s="24"/>
@@ -2443,14 +2455,14 @@
       <c r="K27" s="9"/>
       <c r="L27" s="4"/>
       <c r="M27" s="2"/>
-      <c r="O27" s="42" t="s">
+      <c r="O27" s="44" t="s">
         <v>157</v>
       </c>
-      <c r="P27" s="42"/>
-      <c r="Q27" s="42"/>
-      <c r="R27" s="42"/>
-      <c r="S27" s="42"/>
-      <c r="T27" s="42"/>
+      <c r="P27" s="44"/>
+      <c r="Q27" s="44"/>
+      <c r="R27" s="44"/>
+      <c r="S27" s="44"/>
+      <c r="T27" s="44"/>
     </row>
     <row r="28" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C28" s="24"/>
@@ -2461,12 +2473,12 @@
       <c r="K28" s="9"/>
       <c r="L28" s="4"/>
       <c r="M28" s="2"/>
-      <c r="O28" s="42"/>
-      <c r="P28" s="42"/>
-      <c r="Q28" s="42"/>
-      <c r="R28" s="42"/>
-      <c r="S28" s="42"/>
-      <c r="T28" s="42"/>
+      <c r="O28" s="44"/>
+      <c r="P28" s="44"/>
+      <c r="Q28" s="44"/>
+      <c r="R28" s="44"/>
+      <c r="S28" s="44"/>
+      <c r="T28" s="44"/>
     </row>
     <row r="29" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C29" s="24"/>
@@ -2477,12 +2489,12 @@
       <c r="K29" s="9"/>
       <c r="L29" s="4"/>
       <c r="M29" s="2"/>
-      <c r="O29" s="42"/>
-      <c r="P29" s="42"/>
-      <c r="Q29" s="42"/>
-      <c r="R29" s="42"/>
-      <c r="S29" s="42"/>
-      <c r="T29" s="42"/>
+      <c r="O29" s="44"/>
+      <c r="P29" s="44"/>
+      <c r="Q29" s="44"/>
+      <c r="R29" s="44"/>
+      <c r="S29" s="44"/>
+      <c r="T29" s="44"/>
     </row>
     <row r="30" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C30" s="24"/>
@@ -2493,12 +2505,12 @@
       <c r="K30" s="9"/>
       <c r="L30" s="2"/>
       <c r="M30" s="2"/>
-      <c r="O30" s="42"/>
-      <c r="P30" s="42"/>
-      <c r="Q30" s="42"/>
-      <c r="R30" s="42"/>
-      <c r="S30" s="42"/>
-      <c r="T30" s="42"/>
+      <c r="O30" s="44"/>
+      <c r="P30" s="44"/>
+      <c r="Q30" s="44"/>
+      <c r="R30" s="44"/>
+      <c r="S30" s="44"/>
+      <c r="T30" s="44"/>
     </row>
     <row r="31" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C31" s="24"/>
@@ -2728,16 +2740,16 @@
     </row>
     <row r="10" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C10" s="24"/>
-      <c r="E10" s="39" t="s">
+      <c r="E10" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="40"/>
-      <c r="G10" s="41"/>
-      <c r="J10" s="39" t="s">
+      <c r="F10" s="42"/>
+      <c r="G10" s="43"/>
+      <c r="J10" s="41" t="s">
         <v>16</v>
       </c>
-      <c r="K10" s="40"/>
-      <c r="L10" s="41"/>
+      <c r="K10" s="42"/>
+      <c r="L10" s="43"/>
     </row>
     <row r="11" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C11" s="24"/>
@@ -3189,16 +3201,16 @@
     </row>
     <row r="10" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C10" s="24"/>
-      <c r="E10" s="39" t="s">
+      <c r="E10" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="40"/>
-      <c r="G10" s="41"/>
-      <c r="J10" s="39" t="s">
+      <c r="F10" s="42"/>
+      <c r="G10" s="43"/>
+      <c r="J10" s="41" t="s">
         <v>16</v>
       </c>
-      <c r="K10" s="40"/>
-      <c r="L10" s="41"/>
+      <c r="K10" s="42"/>
+      <c r="L10" s="43"/>
     </row>
     <row r="11" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C11" s="24"/>
@@ -3299,7 +3311,7 @@
         <v>140</v>
       </c>
       <c r="K15" s="9">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="L15" s="4" t="s">
         <v>8</v>
@@ -3367,9 +3379,15 @@
       <c r="E19" s="2"/>
       <c r="F19" s="9"/>
       <c r="G19" s="2"/>
-      <c r="J19" s="2"/>
-      <c r="K19" s="9"/>
-      <c r="L19" s="4"/>
+      <c r="J19" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="K19" s="9">
+        <v>5</v>
+      </c>
+      <c r="L19" s="4" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="20" spans="3:12" x14ac:dyDescent="0.35">
       <c r="C20" s="24"/>
@@ -3679,16 +3697,16 @@
     </row>
     <row r="10" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C10" s="24"/>
-      <c r="E10" s="39" t="s">
+      <c r="E10" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="40"/>
-      <c r="G10" s="41"/>
-      <c r="J10" s="39" t="s">
+      <c r="F10" s="42"/>
+      <c r="G10" s="43"/>
+      <c r="J10" s="41" t="s">
         <v>16</v>
       </c>
-      <c r="K10" s="40"/>
-      <c r="L10" s="41"/>
+      <c r="K10" s="42"/>
+      <c r="L10" s="43"/>
     </row>
     <row r="11" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C11" s="24"/>
@@ -3722,7 +3740,7 @@
       <c r="G12" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="J12" s="45">
+      <c r="J12" s="40">
         <v>10</v>
       </c>
       <c r="K12" s="8" t="s">
@@ -3743,7 +3761,7 @@
       <c r="G13" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="J13" s="45">
+      <c r="J13" s="40">
         <v>10</v>
       </c>
       <c r="K13" s="9" t="s">
@@ -3764,7 +3782,7 @@
       <c r="G14" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="J14" s="45"/>
+      <c r="J14" s="40"/>
       <c r="K14" s="9"/>
       <c r="L14" s="4"/>
     </row>
@@ -3779,7 +3797,7 @@
       <c r="G15" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="J15" s="45"/>
+      <c r="J15" s="40"/>
       <c r="K15" s="9"/>
       <c r="L15" s="4"/>
     </row>
@@ -3794,7 +3812,7 @@
       <c r="G16" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="J16" s="45"/>
+      <c r="J16" s="40"/>
       <c r="K16" s="9"/>
       <c r="L16" s="4"/>
     </row>
@@ -3809,7 +3827,7 @@
       <c r="G17" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="J17" s="45"/>
+      <c r="J17" s="40"/>
       <c r="K17" s="9"/>
       <c r="L17" s="4"/>
     </row>
@@ -3824,7 +3842,7 @@
       <c r="G18" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="J18" s="45"/>
+      <c r="J18" s="40"/>
       <c r="K18" s="9"/>
       <c r="L18" s="4"/>
     </row>
@@ -4092,16 +4110,16 @@
       <c r="D4" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="39" t="s">
+      <c r="F4" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="G4" s="40"/>
-      <c r="H4" s="41"/>
-      <c r="K4" s="39" t="s">
+      <c r="G4" s="42"/>
+      <c r="H4" s="43"/>
+      <c r="K4" s="41" t="s">
         <v>16</v>
       </c>
-      <c r="L4" s="40"/>
-      <c r="M4" s="41"/>
+      <c r="L4" s="42"/>
+      <c r="M4" s="43"/>
     </row>
     <row r="5" spans="3:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C5" s="18" t="s">
@@ -4558,17 +4576,17 @@
     </row>
     <row r="12" spans="3:20" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="13" spans="3:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="F13" s="39" t="s">
+      <c r="F13" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="G13" s="40"/>
-      <c r="H13" s="41"/>
-      <c r="K13" s="39" t="s">
+      <c r="G13" s="42"/>
+      <c r="H13" s="43"/>
+      <c r="K13" s="41" t="s">
         <v>16</v>
       </c>
-      <c r="L13" s="40"/>
-      <c r="M13" s="40"/>
-      <c r="N13" s="41"/>
+      <c r="L13" s="42"/>
+      <c r="M13" s="42"/>
+      <c r="N13" s="43"/>
     </row>
     <row r="14" spans="3:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="F14" s="15" t="s">
@@ -4592,13 +4610,13 @@
       <c r="N14" s="36" t="s">
         <v>115</v>
       </c>
-      <c r="P14" s="42" t="s">
+      <c r="P14" s="44" t="s">
         <v>118</v>
       </c>
-      <c r="Q14" s="42"/>
-      <c r="R14" s="42"/>
-      <c r="S14" s="42"/>
-      <c r="T14" s="42"/>
+      <c r="Q14" s="44"/>
+      <c r="R14" s="44"/>
+      <c r="S14" s="44"/>
+      <c r="T14" s="44"/>
     </row>
     <row r="15" spans="3:20" x14ac:dyDescent="0.35">
       <c r="F15" s="4" t="s">
@@ -4620,11 +4638,11 @@
         <v>25</v>
       </c>
       <c r="N15" s="20"/>
-      <c r="P15" s="42"/>
-      <c r="Q15" s="42"/>
-      <c r="R15" s="42"/>
-      <c r="S15" s="42"/>
-      <c r="T15" s="42"/>
+      <c r="P15" s="44"/>
+      <c r="Q15" s="44"/>
+      <c r="R15" s="44"/>
+      <c r="S15" s="44"/>
+      <c r="T15" s="44"/>
     </row>
     <row r="16" spans="3:20" x14ac:dyDescent="0.35">
       <c r="F16" s="2" t="s">
@@ -4648,11 +4666,11 @@
       <c r="N16" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="P16" s="42"/>
-      <c r="Q16" s="42"/>
-      <c r="R16" s="42"/>
-      <c r="S16" s="42"/>
-      <c r="T16" s="42"/>
+      <c r="P16" s="44"/>
+      <c r="Q16" s="44"/>
+      <c r="R16" s="44"/>
+      <c r="S16" s="44"/>
+      <c r="T16" s="44"/>
     </row>
     <row r="17" spans="6:20" x14ac:dyDescent="0.35">
       <c r="F17" s="2"/>
@@ -4670,11 +4688,11 @@
       <c r="N17" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="P17" s="42"/>
-      <c r="Q17" s="42"/>
-      <c r="R17" s="42"/>
-      <c r="S17" s="42"/>
-      <c r="T17" s="42"/>
+      <c r="P17" s="44"/>
+      <c r="Q17" s="44"/>
+      <c r="R17" s="44"/>
+      <c r="S17" s="44"/>
+      <c r="T17" s="44"/>
     </row>
     <row r="18" spans="6:20" x14ac:dyDescent="0.35">
       <c r="F18" s="2"/>
@@ -5064,16 +5082,16 @@
     </row>
     <row r="11" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C11" s="24"/>
-      <c r="E11" s="39" t="s">
+      <c r="E11" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="F11" s="40"/>
-      <c r="G11" s="41"/>
-      <c r="J11" s="39" t="s">
+      <c r="F11" s="42"/>
+      <c r="G11" s="43"/>
+      <c r="J11" s="41" t="s">
         <v>16</v>
       </c>
-      <c r="K11" s="40"/>
-      <c r="L11" s="41"/>
+      <c r="K11" s="42"/>
+      <c r="L11" s="43"/>
     </row>
     <row r="12" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C12" s="24"/>
@@ -5517,17 +5535,17 @@
     </row>
     <row r="11" spans="2:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C11" s="24"/>
-      <c r="E11" s="39" t="s">
+      <c r="E11" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="F11" s="40"/>
-      <c r="G11" s="41"/>
-      <c r="J11" s="39" t="s">
+      <c r="F11" s="42"/>
+      <c r="G11" s="43"/>
+      <c r="J11" s="41" t="s">
         <v>16</v>
       </c>
-      <c r="K11" s="40"/>
-      <c r="L11" s="40"/>
-      <c r="M11" s="41"/>
+      <c r="K11" s="42"/>
+      <c r="L11" s="42"/>
+      <c r="M11" s="43"/>
     </row>
     <row r="12" spans="2:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C12" s="24"/>
@@ -5552,14 +5570,14 @@
       <c r="M12" s="36" t="s">
         <v>115</v>
       </c>
-      <c r="O12" s="42" t="s">
+      <c r="O12" s="44" t="s">
         <v>96</v>
       </c>
-      <c r="P12" s="42"/>
-      <c r="Q12" s="42"/>
-      <c r="R12" s="42"/>
-      <c r="S12" s="42"/>
-      <c r="T12" s="42"/>
+      <c r="P12" s="44"/>
+      <c r="Q12" s="44"/>
+      <c r="R12" s="44"/>
+      <c r="S12" s="44"/>
+      <c r="T12" s="44"/>
     </row>
     <row r="13" spans="2:20" x14ac:dyDescent="0.35">
       <c r="C13" s="24"/>
@@ -5583,12 +5601,12 @@
         <v>25</v>
       </c>
       <c r="M13" s="20"/>
-      <c r="O13" s="42"/>
-      <c r="P13" s="42"/>
-      <c r="Q13" s="42"/>
-      <c r="R13" s="42"/>
-      <c r="S13" s="42"/>
-      <c r="T13" s="42"/>
+      <c r="O13" s="44"/>
+      <c r="P13" s="44"/>
+      <c r="Q13" s="44"/>
+      <c r="R13" s="44"/>
+      <c r="S13" s="44"/>
+      <c r="T13" s="44"/>
     </row>
     <row r="14" spans="2:20" x14ac:dyDescent="0.35">
       <c r="C14" s="24"/>
@@ -5613,12 +5631,12 @@
       <c r="M14" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="O14" s="42"/>
-      <c r="P14" s="42"/>
-      <c r="Q14" s="42"/>
-      <c r="R14" s="42"/>
-      <c r="S14" s="42"/>
-      <c r="T14" s="42"/>
+      <c r="O14" s="44"/>
+      <c r="P14" s="44"/>
+      <c r="Q14" s="44"/>
+      <c r="R14" s="44"/>
+      <c r="S14" s="44"/>
+      <c r="T14" s="44"/>
     </row>
     <row r="15" spans="2:20" x14ac:dyDescent="0.35">
       <c r="C15" s="24"/>
@@ -5637,12 +5655,12 @@
       <c r="M15" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="O15" s="42"/>
-      <c r="P15" s="42"/>
-      <c r="Q15" s="42"/>
-      <c r="R15" s="42"/>
-      <c r="S15" s="42"/>
-      <c r="T15" s="42"/>
+      <c r="O15" s="44"/>
+      <c r="P15" s="44"/>
+      <c r="Q15" s="44"/>
+      <c r="R15" s="44"/>
+      <c r="S15" s="44"/>
+      <c r="T15" s="44"/>
     </row>
     <row r="16" spans="2:20" x14ac:dyDescent="0.35">
       <c r="C16" s="24"/>
@@ -5661,14 +5679,14 @@
       <c r="M16" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="O16" s="42" t="s">
+      <c r="O16" s="44" t="s">
         <v>113</v>
       </c>
-      <c r="P16" s="42"/>
-      <c r="Q16" s="42"/>
-      <c r="R16" s="42"/>
-      <c r="S16" s="42"/>
-      <c r="T16" s="42"/>
+      <c r="P16" s="44"/>
+      <c r="Q16" s="44"/>
+      <c r="R16" s="44"/>
+      <c r="S16" s="44"/>
+      <c r="T16" s="44"/>
     </row>
     <row r="17" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C17" s="24"/>
@@ -5687,12 +5705,12 @@
       <c r="M17" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="O17" s="42"/>
-      <c r="P17" s="42"/>
-      <c r="Q17" s="42"/>
-      <c r="R17" s="42"/>
-      <c r="S17" s="42"/>
-      <c r="T17" s="42"/>
+      <c r="O17" s="44"/>
+      <c r="P17" s="44"/>
+      <c r="Q17" s="44"/>
+      <c r="R17" s="44"/>
+      <c r="S17" s="44"/>
+      <c r="T17" s="44"/>
     </row>
     <row r="18" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C18" s="24"/>
@@ -5709,12 +5727,12 @@
         <v>154</v>
       </c>
       <c r="M18" s="2"/>
-      <c r="O18" s="42"/>
-      <c r="P18" s="42"/>
-      <c r="Q18" s="42"/>
-      <c r="R18" s="42"/>
-      <c r="S18" s="42"/>
-      <c r="T18" s="42"/>
+      <c r="O18" s="44"/>
+      <c r="P18" s="44"/>
+      <c r="Q18" s="44"/>
+      <c r="R18" s="44"/>
+      <c r="S18" s="44"/>
+      <c r="T18" s="44"/>
     </row>
     <row r="19" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C19" s="24"/>
@@ -5725,12 +5743,12 @@
       <c r="K19" s="9"/>
       <c r="L19" s="6"/>
       <c r="M19" s="2"/>
-      <c r="O19" s="42"/>
-      <c r="P19" s="42"/>
-      <c r="Q19" s="42"/>
-      <c r="R19" s="42"/>
-      <c r="S19" s="42"/>
-      <c r="T19" s="42"/>
+      <c r="O19" s="44"/>
+      <c r="P19" s="44"/>
+      <c r="Q19" s="44"/>
+      <c r="R19" s="44"/>
+      <c r="S19" s="44"/>
+      <c r="T19" s="44"/>
     </row>
     <row r="20" spans="3:20" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C20" s="24"/>
@@ -5751,14 +5769,14 @@
       <c r="K21" s="9"/>
       <c r="L21" s="6"/>
       <c r="M21" s="2"/>
-      <c r="O21" s="43" t="s">
+      <c r="O21" s="45" t="s">
         <v>153</v>
       </c>
-      <c r="P21" s="43"/>
-      <c r="Q21" s="43"/>
-      <c r="R21" s="43"/>
-      <c r="S21" s="43"/>
-      <c r="T21" s="43"/>
+      <c r="P21" s="45"/>
+      <c r="Q21" s="45"/>
+      <c r="R21" s="45"/>
+      <c r="S21" s="45"/>
+      <c r="T21" s="45"/>
     </row>
     <row r="22" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C22" s="24"/>
@@ -5779,14 +5797,14 @@
       <c r="K23" s="9"/>
       <c r="L23" s="6"/>
       <c r="M23" s="2"/>
-      <c r="O23" s="42" t="s">
+      <c r="O23" s="44" t="s">
         <v>159</v>
       </c>
-      <c r="P23" s="42"/>
-      <c r="Q23" s="42"/>
-      <c r="R23" s="42"/>
-      <c r="S23" s="42"/>
-      <c r="T23" s="42"/>
+      <c r="P23" s="44"/>
+      <c r="Q23" s="44"/>
+      <c r="R23" s="44"/>
+      <c r="S23" s="44"/>
+      <c r="T23" s="44"/>
     </row>
     <row r="24" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C24" s="24"/>
@@ -5797,12 +5815,12 @@
       <c r="K24" s="9"/>
       <c r="L24" s="6"/>
       <c r="M24" s="2"/>
-      <c r="O24" s="42"/>
-      <c r="P24" s="42"/>
-      <c r="Q24" s="42"/>
-      <c r="R24" s="42"/>
-      <c r="S24" s="42"/>
-      <c r="T24" s="42"/>
+      <c r="O24" s="44"/>
+      <c r="P24" s="44"/>
+      <c r="Q24" s="44"/>
+      <c r="R24" s="44"/>
+      <c r="S24" s="44"/>
+      <c r="T24" s="44"/>
     </row>
     <row r="25" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C25" s="24"/>
@@ -5813,12 +5831,12 @@
       <c r="K25" s="9"/>
       <c r="L25" s="6"/>
       <c r="M25" s="2"/>
-      <c r="O25" s="42"/>
-      <c r="P25" s="42"/>
-      <c r="Q25" s="42"/>
-      <c r="R25" s="42"/>
-      <c r="S25" s="42"/>
-      <c r="T25" s="42"/>
+      <c r="O25" s="44"/>
+      <c r="P25" s="44"/>
+      <c r="Q25" s="44"/>
+      <c r="R25" s="44"/>
+      <c r="S25" s="44"/>
+      <c r="T25" s="44"/>
     </row>
     <row r="26" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C26" s="24"/>
@@ -5829,12 +5847,12 @@
       <c r="K26" s="9"/>
       <c r="L26" s="6"/>
       <c r="M26" s="2"/>
-      <c r="O26" s="42"/>
-      <c r="P26" s="42"/>
-      <c r="Q26" s="42"/>
-      <c r="R26" s="42"/>
-      <c r="S26" s="42"/>
-      <c r="T26" s="42"/>
+      <c r="O26" s="44"/>
+      <c r="P26" s="44"/>
+      <c r="Q26" s="44"/>
+      <c r="R26" s="44"/>
+      <c r="S26" s="44"/>
+      <c r="T26" s="44"/>
     </row>
     <row r="27" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C27" s="24"/>
@@ -5845,14 +5863,14 @@
       <c r="K27" s="9"/>
       <c r="L27" s="6"/>
       <c r="M27" s="2"/>
-      <c r="O27" s="42" t="s">
+      <c r="O27" s="44" t="s">
         <v>160</v>
       </c>
-      <c r="P27" s="42"/>
-      <c r="Q27" s="42"/>
-      <c r="R27" s="42"/>
-      <c r="S27" s="42"/>
-      <c r="T27" s="42"/>
+      <c r="P27" s="44"/>
+      <c r="Q27" s="44"/>
+      <c r="R27" s="44"/>
+      <c r="S27" s="44"/>
+      <c r="T27" s="44"/>
     </row>
     <row r="28" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C28" s="24"/>
@@ -5863,12 +5881,12 @@
       <c r="K28" s="9"/>
       <c r="L28" s="6"/>
       <c r="M28" s="2"/>
-      <c r="O28" s="42"/>
-      <c r="P28" s="42"/>
-      <c r="Q28" s="42"/>
-      <c r="R28" s="42"/>
-      <c r="S28" s="42"/>
-      <c r="T28" s="42"/>
+      <c r="O28" s="44"/>
+      <c r="P28" s="44"/>
+      <c r="Q28" s="44"/>
+      <c r="R28" s="44"/>
+      <c r="S28" s="44"/>
+      <c r="T28" s="44"/>
     </row>
     <row r="29" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C29" s="24"/>
@@ -5879,12 +5897,12 @@
       <c r="K29" s="9"/>
       <c r="L29" s="6"/>
       <c r="M29" s="2"/>
-      <c r="O29" s="42"/>
-      <c r="P29" s="42"/>
-      <c r="Q29" s="42"/>
-      <c r="R29" s="42"/>
-      <c r="S29" s="42"/>
-      <c r="T29" s="42"/>
+      <c r="O29" s="44"/>
+      <c r="P29" s="44"/>
+      <c r="Q29" s="44"/>
+      <c r="R29" s="44"/>
+      <c r="S29" s="44"/>
+      <c r="T29" s="44"/>
     </row>
     <row r="30" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C30" s="24"/>
@@ -5895,12 +5913,12 @@
       <c r="K30" s="9"/>
       <c r="L30" s="6"/>
       <c r="M30" s="2"/>
-      <c r="O30" s="42"/>
-      <c r="P30" s="42"/>
-      <c r="Q30" s="42"/>
-      <c r="R30" s="42"/>
-      <c r="S30" s="42"/>
-      <c r="T30" s="42"/>
+      <c r="O30" s="44"/>
+      <c r="P30" s="44"/>
+      <c r="Q30" s="44"/>
+      <c r="R30" s="44"/>
+      <c r="S30" s="44"/>
+      <c r="T30" s="44"/>
     </row>
     <row r="31" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C31" s="24"/>
@@ -5911,14 +5929,14 @@
       <c r="K31" s="9"/>
       <c r="L31" s="6"/>
       <c r="M31" s="2"/>
-      <c r="O31" s="42" t="s">
+      <c r="O31" s="44" t="s">
         <v>161</v>
       </c>
-      <c r="P31" s="42"/>
-      <c r="Q31" s="42"/>
-      <c r="R31" s="42"/>
-      <c r="S31" s="42"/>
-      <c r="T31" s="42"/>
+      <c r="P31" s="44"/>
+      <c r="Q31" s="44"/>
+      <c r="R31" s="44"/>
+      <c r="S31" s="44"/>
+      <c r="T31" s="44"/>
     </row>
     <row r="32" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C32" s="24"/>
@@ -5929,12 +5947,12 @@
       <c r="K32" s="9"/>
       <c r="L32" s="6"/>
       <c r="M32" s="2"/>
-      <c r="O32" s="42"/>
-      <c r="P32" s="42"/>
-      <c r="Q32" s="42"/>
-      <c r="R32" s="42"/>
-      <c r="S32" s="42"/>
-      <c r="T32" s="42"/>
+      <c r="O32" s="44"/>
+      <c r="P32" s="44"/>
+      <c r="Q32" s="44"/>
+      <c r="R32" s="44"/>
+      <c r="S32" s="44"/>
+      <c r="T32" s="44"/>
     </row>
     <row r="33" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C33" s="24"/>
@@ -5945,12 +5963,12 @@
       <c r="K33" s="9"/>
       <c r="L33" s="6"/>
       <c r="M33" s="2"/>
-      <c r="O33" s="42"/>
-      <c r="P33" s="42"/>
-      <c r="Q33" s="42"/>
-      <c r="R33" s="42"/>
-      <c r="S33" s="42"/>
-      <c r="T33" s="42"/>
+      <c r="O33" s="44"/>
+      <c r="P33" s="44"/>
+      <c r="Q33" s="44"/>
+      <c r="R33" s="44"/>
+      <c r="S33" s="44"/>
+      <c r="T33" s="44"/>
     </row>
     <row r="34" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C34" s="24"/>
@@ -5961,12 +5979,12 @@
       <c r="K34" s="9"/>
       <c r="L34" s="6"/>
       <c r="M34" s="2"/>
-      <c r="O34" s="42"/>
-      <c r="P34" s="42"/>
-      <c r="Q34" s="42"/>
-      <c r="R34" s="42"/>
-      <c r="S34" s="42"/>
-      <c r="T34" s="42"/>
+      <c r="O34" s="44"/>
+      <c r="P34" s="44"/>
+      <c r="Q34" s="44"/>
+      <c r="R34" s="44"/>
+      <c r="S34" s="44"/>
+      <c r="T34" s="44"/>
     </row>
     <row r="35" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C35" s="24"/>
@@ -6107,16 +6125,16 @@
       <c r="C2" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="E2" s="39" t="s">
+      <c r="E2" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="40"/>
-      <c r="G2" s="41"/>
-      <c r="J2" s="39" t="s">
+      <c r="F2" s="42"/>
+      <c r="G2" s="43"/>
+      <c r="J2" s="41" t="s">
         <v>16</v>
       </c>
-      <c r="K2" s="40"/>
-      <c r="L2" s="41"/>
+      <c r="K2" s="42"/>
+      <c r="L2" s="43"/>
     </row>
     <row r="3" spans="2:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B3" s="22" t="s">
@@ -6143,14 +6161,14 @@
       <c r="L3" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="N3" s="42" t="s">
+      <c r="N3" s="44" t="s">
         <v>87</v>
       </c>
-      <c r="O3" s="42"/>
-      <c r="P3" s="42"/>
-      <c r="Q3" s="42"/>
-      <c r="R3" s="42"/>
-      <c r="S3" s="42"/>
+      <c r="O3" s="44"/>
+      <c r="P3" s="44"/>
+      <c r="Q3" s="44"/>
+      <c r="R3" s="44"/>
+      <c r="S3" s="44"/>
     </row>
     <row r="4" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B4" s="22" t="s">
@@ -6177,12 +6195,12 @@
       <c r="L4" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="N4" s="42"/>
-      <c r="O4" s="42"/>
-      <c r="P4" s="42"/>
-      <c r="Q4" s="42"/>
-      <c r="R4" s="42"/>
-      <c r="S4" s="42"/>
+      <c r="N4" s="44"/>
+      <c r="O4" s="44"/>
+      <c r="P4" s="44"/>
+      <c r="Q4" s="44"/>
+      <c r="R4" s="44"/>
+      <c r="S4" s="44"/>
     </row>
     <row r="5" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B5" s="22" t="s">
@@ -6209,12 +6227,12 @@
       <c r="L5" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="N5" s="42"/>
-      <c r="O5" s="42"/>
-      <c r="P5" s="42"/>
-      <c r="Q5" s="42"/>
-      <c r="R5" s="42"/>
-      <c r="S5" s="42"/>
+      <c r="N5" s="44"/>
+      <c r="O5" s="44"/>
+      <c r="P5" s="44"/>
+      <c r="Q5" s="44"/>
+      <c r="R5" s="44"/>
+      <c r="S5" s="44"/>
     </row>
     <row r="6" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B6" s="22" t="s">
@@ -6229,12 +6247,12 @@
       <c r="J6" s="4"/>
       <c r="K6" s="9"/>
       <c r="L6" s="2"/>
-      <c r="N6" s="42"/>
-      <c r="O6" s="42"/>
-      <c r="P6" s="42"/>
-      <c r="Q6" s="42"/>
-      <c r="R6" s="42"/>
-      <c r="S6" s="42"/>
+      <c r="N6" s="44"/>
+      <c r="O6" s="44"/>
+      <c r="P6" s="44"/>
+      <c r="Q6" s="44"/>
+      <c r="R6" s="44"/>
+      <c r="S6" s="44"/>
     </row>
     <row r="7" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B7" s="22" t="s">
@@ -6613,16 +6631,16 @@
     </row>
     <row r="10" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C10" s="24"/>
-      <c r="E10" s="39" t="s">
+      <c r="E10" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="40"/>
-      <c r="G10" s="41"/>
-      <c r="J10" s="39" t="s">
+      <c r="F10" s="42"/>
+      <c r="G10" s="43"/>
+      <c r="J10" s="41" t="s">
         <v>16</v>
       </c>
-      <c r="K10" s="40"/>
-      <c r="L10" s="41"/>
+      <c r="K10" s="42"/>
+      <c r="L10" s="43"/>
     </row>
     <row r="11" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C11" s="24"/>
@@ -7128,7 +7146,7 @@
       <c r="B4" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="44" t="s">
+      <c r="C4" s="39" t="s">
         <v>163</v>
       </c>
     </row>
@@ -7174,16 +7192,16 @@
     </row>
     <row r="10" spans="2:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C10" s="24"/>
-      <c r="E10" s="39" t="s">
+      <c r="E10" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="40"/>
-      <c r="G10" s="41"/>
-      <c r="J10" s="39" t="s">
+      <c r="F10" s="42"/>
+      <c r="G10" s="43"/>
+      <c r="J10" s="41" t="s">
         <v>16</v>
       </c>
-      <c r="K10" s="40"/>
-      <c r="L10" s="41"/>
+      <c r="K10" s="42"/>
+      <c r="L10" s="43"/>
     </row>
     <row r="11" spans="2:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C11" s="24"/>
@@ -7247,14 +7265,14 @@
       <c r="L13" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="N13" s="42" t="s">
+      <c r="N13" s="44" t="s">
         <v>94</v>
       </c>
-      <c r="O13" s="42"/>
-      <c r="P13" s="42"/>
-      <c r="Q13" s="42"/>
-      <c r="R13" s="42"/>
-      <c r="S13" s="42"/>
+      <c r="O13" s="44"/>
+      <c r="P13" s="44"/>
+      <c r="Q13" s="44"/>
+      <c r="R13" s="44"/>
+      <c r="S13" s="44"/>
     </row>
     <row r="14" spans="2:19" x14ac:dyDescent="0.35">
       <c r="C14" s="24"/>
@@ -7276,12 +7294,12 @@
       <c r="L14" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="N14" s="42"/>
-      <c r="O14" s="42"/>
-      <c r="P14" s="42"/>
-      <c r="Q14" s="42"/>
-      <c r="R14" s="42"/>
-      <c r="S14" s="42"/>
+      <c r="N14" s="44"/>
+      <c r="O14" s="44"/>
+      <c r="P14" s="44"/>
+      <c r="Q14" s="44"/>
+      <c r="R14" s="44"/>
+      <c r="S14" s="44"/>
     </row>
     <row r="15" spans="2:19" x14ac:dyDescent="0.35">
       <c r="C15" s="24"/>
@@ -7297,12 +7315,12 @@
       <c r="L15" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="N15" s="42"/>
-      <c r="O15" s="42"/>
-      <c r="P15" s="42"/>
-      <c r="Q15" s="42"/>
-      <c r="R15" s="42"/>
-      <c r="S15" s="42"/>
+      <c r="N15" s="44"/>
+      <c r="O15" s="44"/>
+      <c r="P15" s="44"/>
+      <c r="Q15" s="44"/>
+      <c r="R15" s="44"/>
+      <c r="S15" s="44"/>
     </row>
     <row r="16" spans="2:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C16" s="24"/>
@@ -7318,12 +7336,12 @@
       <c r="L16" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="N16" s="42"/>
-      <c r="O16" s="42"/>
-      <c r="P16" s="42"/>
-      <c r="Q16" s="42"/>
-      <c r="R16" s="42"/>
-      <c r="S16" s="42"/>
+      <c r="N16" s="44"/>
+      <c r="O16" s="44"/>
+      <c r="P16" s="44"/>
+      <c r="Q16" s="44"/>
+      <c r="R16" s="44"/>
+      <c r="S16" s="44"/>
     </row>
     <row r="17" spans="3:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C17" s="24"/>
@@ -7339,14 +7357,14 @@
       <c r="L17" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="N17" s="42" t="s">
+      <c r="N17" s="44" t="s">
         <v>95</v>
       </c>
-      <c r="O17" s="42"/>
-      <c r="P17" s="42"/>
-      <c r="Q17" s="42"/>
-      <c r="R17" s="42"/>
-      <c r="S17" s="42"/>
+      <c r="O17" s="44"/>
+      <c r="P17" s="44"/>
+      <c r="Q17" s="44"/>
+      <c r="R17" s="44"/>
+      <c r="S17" s="44"/>
     </row>
     <row r="18" spans="3:19" x14ac:dyDescent="0.35">
       <c r="C18" s="24"/>
@@ -7362,12 +7380,12 @@
       <c r="L18" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="N18" s="42"/>
-      <c r="O18" s="42"/>
-      <c r="P18" s="42"/>
-      <c r="Q18" s="42"/>
-      <c r="R18" s="42"/>
-      <c r="S18" s="42"/>
+      <c r="N18" s="44"/>
+      <c r="O18" s="44"/>
+      <c r="P18" s="44"/>
+      <c r="Q18" s="44"/>
+      <c r="R18" s="44"/>
+      <c r="S18" s="44"/>
     </row>
     <row r="19" spans="3:19" x14ac:dyDescent="0.35">
       <c r="C19" s="24"/>
@@ -7383,12 +7401,12 @@
       <c r="L19" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="N19" s="42"/>
-      <c r="O19" s="42"/>
-      <c r="P19" s="42"/>
-      <c r="Q19" s="42"/>
-      <c r="R19" s="42"/>
-      <c r="S19" s="42"/>
+      <c r="N19" s="44"/>
+      <c r="O19" s="44"/>
+      <c r="P19" s="44"/>
+      <c r="Q19" s="44"/>
+      <c r="R19" s="44"/>
+      <c r="S19" s="44"/>
     </row>
     <row r="20" spans="3:19" x14ac:dyDescent="0.35">
       <c r="C20" s="24"/>
@@ -7398,12 +7416,12 @@
       <c r="J20" s="2"/>
       <c r="K20" s="9"/>
       <c r="L20" s="4"/>
-      <c r="N20" s="42"/>
-      <c r="O20" s="42"/>
-      <c r="P20" s="42"/>
-      <c r="Q20" s="42"/>
-      <c r="R20" s="42"/>
-      <c r="S20" s="42"/>
+      <c r="N20" s="44"/>
+      <c r="O20" s="44"/>
+      <c r="P20" s="44"/>
+      <c r="Q20" s="44"/>
+      <c r="R20" s="44"/>
+      <c r="S20" s="44"/>
     </row>
     <row r="21" spans="3:19" x14ac:dyDescent="0.35">
       <c r="C21" s="24"/>
@@ -7422,14 +7440,14 @@
       <c r="J22" s="2"/>
       <c r="K22" s="9"/>
       <c r="L22" s="4"/>
-      <c r="N22" s="43" t="s">
+      <c r="N22" s="45" t="s">
         <v>153</v>
       </c>
-      <c r="O22" s="43"/>
-      <c r="P22" s="43"/>
-      <c r="Q22" s="43"/>
-      <c r="R22" s="43"/>
-      <c r="S22" s="43"/>
+      <c r="O22" s="45"/>
+      <c r="P22" s="45"/>
+      <c r="Q22" s="45"/>
+      <c r="R22" s="45"/>
+      <c r="S22" s="45"/>
     </row>
     <row r="23" spans="3:19" x14ac:dyDescent="0.35">
       <c r="C23" s="24"/>
@@ -7448,14 +7466,14 @@
       <c r="J24" s="2"/>
       <c r="K24" s="9"/>
       <c r="L24" s="4"/>
-      <c r="N24" s="42" t="s">
+      <c r="N24" s="44" t="s">
         <v>155</v>
       </c>
-      <c r="O24" s="42"/>
-      <c r="P24" s="42"/>
-      <c r="Q24" s="42"/>
-      <c r="R24" s="42"/>
-      <c r="S24" s="42"/>
+      <c r="O24" s="44"/>
+      <c r="P24" s="44"/>
+      <c r="Q24" s="44"/>
+      <c r="R24" s="44"/>
+      <c r="S24" s="44"/>
     </row>
     <row r="25" spans="3:19" x14ac:dyDescent="0.35">
       <c r="C25" s="24"/>
@@ -7465,12 +7483,12 @@
       <c r="J25" s="2"/>
       <c r="K25" s="9"/>
       <c r="L25" s="4"/>
-      <c r="N25" s="42"/>
-      <c r="O25" s="42"/>
-      <c r="P25" s="42"/>
-      <c r="Q25" s="42"/>
-      <c r="R25" s="42"/>
-      <c r="S25" s="42"/>
+      <c r="N25" s="44"/>
+      <c r="O25" s="44"/>
+      <c r="P25" s="44"/>
+      <c r="Q25" s="44"/>
+      <c r="R25" s="44"/>
+      <c r="S25" s="44"/>
     </row>
     <row r="26" spans="3:19" x14ac:dyDescent="0.35">
       <c r="C26" s="24"/>
@@ -7480,12 +7498,12 @@
       <c r="J26" s="2"/>
       <c r="K26" s="9"/>
       <c r="L26" s="4"/>
-      <c r="N26" s="42"/>
-      <c r="O26" s="42"/>
-      <c r="P26" s="42"/>
-      <c r="Q26" s="42"/>
-      <c r="R26" s="42"/>
-      <c r="S26" s="42"/>
+      <c r="N26" s="44"/>
+      <c r="O26" s="44"/>
+      <c r="P26" s="44"/>
+      <c r="Q26" s="44"/>
+      <c r="R26" s="44"/>
+      <c r="S26" s="44"/>
     </row>
     <row r="27" spans="3:19" x14ac:dyDescent="0.35">
       <c r="C27" s="24"/>
@@ -7495,12 +7513,12 @@
       <c r="J27" s="2"/>
       <c r="K27" s="9"/>
       <c r="L27" s="4"/>
-      <c r="N27" s="42"/>
-      <c r="O27" s="42"/>
-      <c r="P27" s="42"/>
-      <c r="Q27" s="42"/>
-      <c r="R27" s="42"/>
-      <c r="S27" s="42"/>
+      <c r="N27" s="44"/>
+      <c r="O27" s="44"/>
+      <c r="P27" s="44"/>
+      <c r="Q27" s="44"/>
+      <c r="R27" s="44"/>
+      <c r="S27" s="44"/>
     </row>
     <row r="28" spans="3:19" x14ac:dyDescent="0.35">
       <c r="C28" s="24"/>
@@ -7510,14 +7528,14 @@
       <c r="J28" s="2"/>
       <c r="K28" s="9"/>
       <c r="L28" s="4"/>
-      <c r="N28" s="42" t="s">
+      <c r="N28" s="44" t="s">
         <v>158</v>
       </c>
-      <c r="O28" s="42"/>
-      <c r="P28" s="42"/>
-      <c r="Q28" s="42"/>
-      <c r="R28" s="42"/>
-      <c r="S28" s="42"/>
+      <c r="O28" s="44"/>
+      <c r="P28" s="44"/>
+      <c r="Q28" s="44"/>
+      <c r="R28" s="44"/>
+      <c r="S28" s="44"/>
     </row>
     <row r="29" spans="3:19" x14ac:dyDescent="0.35">
       <c r="C29" s="24"/>
@@ -7527,12 +7545,12 @@
       <c r="J29" s="2"/>
       <c r="K29" s="9"/>
       <c r="L29" s="4"/>
-      <c r="N29" s="42"/>
-      <c r="O29" s="42"/>
-      <c r="P29" s="42"/>
-      <c r="Q29" s="42"/>
-      <c r="R29" s="42"/>
-      <c r="S29" s="42"/>
+      <c r="N29" s="44"/>
+      <c r="O29" s="44"/>
+      <c r="P29" s="44"/>
+      <c r="Q29" s="44"/>
+      <c r="R29" s="44"/>
+      <c r="S29" s="44"/>
     </row>
     <row r="30" spans="3:19" x14ac:dyDescent="0.35">
       <c r="C30" s="24"/>
@@ -7542,12 +7560,12 @@
       <c r="J30" s="2"/>
       <c r="K30" s="9"/>
       <c r="L30" s="2"/>
-      <c r="N30" s="42"/>
-      <c r="O30" s="42"/>
-      <c r="P30" s="42"/>
-      <c r="Q30" s="42"/>
-      <c r="R30" s="42"/>
-      <c r="S30" s="42"/>
+      <c r="N30" s="44"/>
+      <c r="O30" s="44"/>
+      <c r="P30" s="44"/>
+      <c r="Q30" s="44"/>
+      <c r="R30" s="44"/>
+      <c r="S30" s="44"/>
     </row>
     <row r="31" spans="3:19" x14ac:dyDescent="0.35">
       <c r="C31" s="24"/>
@@ -7557,12 +7575,12 @@
       <c r="J31" s="2"/>
       <c r="K31" s="9"/>
       <c r="L31" s="2"/>
-      <c r="N31" s="42"/>
-      <c r="O31" s="42"/>
-      <c r="P31" s="42"/>
-      <c r="Q31" s="42"/>
-      <c r="R31" s="42"/>
-      <c r="S31" s="42"/>
+      <c r="N31" s="44"/>
+      <c r="O31" s="44"/>
+      <c r="P31" s="44"/>
+      <c r="Q31" s="44"/>
+      <c r="R31" s="44"/>
+      <c r="S31" s="44"/>
     </row>
     <row r="32" spans="3:19" x14ac:dyDescent="0.35">
       <c r="C32" s="24"/>
@@ -7769,16 +7787,16 @@
     </row>
     <row r="10" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C10" s="24"/>
-      <c r="E10" s="39" t="s">
+      <c r="E10" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="40"/>
-      <c r="G10" s="41"/>
-      <c r="J10" s="39" t="s">
+      <c r="F10" s="42"/>
+      <c r="G10" s="43"/>
+      <c r="J10" s="41" t="s">
         <v>16</v>
       </c>
-      <c r="K10" s="40"/>
-      <c r="L10" s="41"/>
+      <c r="K10" s="42"/>
+      <c r="L10" s="43"/>
     </row>
     <row r="11" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C11" s="24"/>

</xml_diff>

<commit_message>
Addesd stuff. Yeah, im not specific but nobody reads this. Have you read it? Let me know in a youtube comment, ill think of a price
</commit_message>
<xml_diff>
--- a/Game Stuff/Spreadsheet.xlsx
+++ b/Game Stuff/Spreadsheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Thassa's Pulse\Game Stuff\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4CDCE38-96CB-42A8-9597-DCEB445A8937}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CCFC74F-315E-4114-B8C5-9C10256A9ED2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{E9D95B66-7EA4-4203-9BE9-B35EAC251241}"/>
+    <workbookView xWindow="45972" yWindow="-4944" windowWidth="17496" windowHeight="30216" firstSheet="3" activeTab="4" xr2:uid="{E9D95B66-7EA4-4203-9BE9-B35EAC251241}"/>
   </bookViews>
   <sheets>
     <sheet name="Material Summary" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1104" uniqueCount="278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1123" uniqueCount="282">
   <si>
     <t>Item</t>
   </si>
@@ -566,9 +566,6 @@
     <t>18917.3 Mw</t>
   </si>
   <si>
-    <t>1875.2 MW</t>
-  </si>
-  <si>
     <t>Nitrogen Gas</t>
   </si>
   <si>
@@ -710,9 +707,6 @@
     <t>Rubber Line going to Phyrexian Datavaul, Keldon Armory and Obelisk of Alara  has an extra 145.2 available</t>
   </si>
   <si>
-    <t>C</t>
-  </si>
-  <si>
     <t>Oran Rief Mines</t>
   </si>
   <si>
@@ -773,21 +767,12 @@
     <t>Karn's Conduit</t>
   </si>
   <si>
-    <t>Neko's Nexus, Ghirapur Gridworks, Phyrexian Datavault, Keldon Armory , Obelisks of Alara, Karn's Conduit</t>
-  </si>
-  <si>
     <t>Phyrexian Datavault, Keldon Armory, Jund Pyroclast, Urabrask's Refinery, Obelisks of Alara, Karn's Conduit</t>
   </si>
   <si>
-    <t>Thran Foundy, Neko's Nexus, Ghirapur Gridworks, The Abyssal Chains of Shandalar, Keldon Armory, Karn's Conduit</t>
-  </si>
-  <si>
     <t>Obelisks of Alara, Keldon Armory, Riveteers District, Phyrexian Datavault, Thran Foundry , Darksteel Forge</t>
   </si>
   <si>
-    <t>Bottom belt going to Keldon Armory and Karn's Conduit has an extra 277.835 Iron Ingots</t>
-  </si>
-  <si>
     <t>738.9 MW</t>
   </si>
   <si>
@@ -888,6 +873,33 @@
   </si>
   <si>
     <t xml:space="preserve">2.84 Hours </t>
+  </si>
+  <si>
+    <t>Bottom belt going to Keldon Armory, Karn's Conduit And Jund PYroclast has an extra 268.457 Iron Ingots</t>
+  </si>
+  <si>
+    <t>Neko's Nexus, Ghirapur Gridworks, Phyrexian Datavault, Keldon Armory , Obelisks of Alara, Karn's Conduit, Jund Pyroclast</t>
+  </si>
+  <si>
+    <t>Jund Pytoclast</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Riveteers District, Darksteel Forge, Oran-Rief Mines </t>
+  </si>
+  <si>
+    <t>Thran Foundy, Neko's Nexus, Ghirapur Gridworks, The Abyssal Chains of Shandalar, Keldon Armory, Karn's Conduit, Jund Pyroclast</t>
+  </si>
+  <si>
+    <t>Gas Filter</t>
+  </si>
+  <si>
+    <t>Iodine-Infused Filter</t>
+  </si>
+  <si>
+    <t>3000 MWh</t>
+  </si>
+  <si>
+    <t>1977.3 MW</t>
   </si>
 </sst>
 </file>
@@ -1362,7 +1374,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1492,9 +1504,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1921,18 +1930,18 @@
     </row>
     <row r="3" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="4" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C4" s="72" t="s">
+      <c r="C4" s="71" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="73"/>
-      <c r="E4" s="74"/>
+      <c r="D4" s="72"/>
+      <c r="E4" s="73"/>
       <c r="F4" s="13"/>
       <c r="G4" s="13"/>
-      <c r="H4" s="72" t="s">
+      <c r="H4" s="71" t="s">
         <v>8</v>
       </c>
-      <c r="I4" s="73"/>
-      <c r="J4" s="74"/>
+      <c r="I4" s="72"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C5" s="35" t="s">
@@ -2001,7 +2010,7 @@
         <v>41</v>
       </c>
       <c r="D8" s="11">
-        <v>1837.835</v>
+        <v>1828.46</v>
       </c>
       <c r="E8" s="41" t="s">
         <v>42</v>
@@ -2084,7 +2093,7 @@
         <v>345.64157</v>
       </c>
       <c r="E12" s="41" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="H12" s="2" t="s">
         <v>67</v>
@@ -2204,7 +2213,7 @@
         <v>1898.3330000000001</v>
       </c>
       <c r="E18" s="41" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="H18" s="2" t="s">
         <v>73</v>
@@ -2512,7 +2521,7 @@
         <v>138</v>
       </c>
       <c r="I40" s="57">
-        <v>61.7</v>
+        <v>60.4375</v>
       </c>
       <c r="J40" s="41" t="s">
         <v>131</v>
@@ -2564,10 +2573,10 @@
     </row>
     <row r="45" spans="3:10" x14ac:dyDescent="0.35">
       <c r="H45" s="39" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I45" s="58">
-        <v>12.5</v>
+        <v>6.25</v>
       </c>
       <c r="J45" s="42" t="s">
         <v>165</v>
@@ -2575,7 +2584,7 @@
     </row>
     <row r="46" spans="3:10" x14ac:dyDescent="0.35">
       <c r="H46" s="39" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I46" s="58">
         <v>12.5</v>
@@ -2586,7 +2595,7 @@
     </row>
     <row r="47" spans="3:10" x14ac:dyDescent="0.35">
       <c r="H47" s="39" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="I47" s="58">
         <v>148.44999999999999</v>
@@ -2597,156 +2606,156 @@
     </row>
     <row r="48" spans="3:10" x14ac:dyDescent="0.35">
       <c r="H48" s="39" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I48" s="58">
         <v>2</v>
       </c>
       <c r="J48" s="41" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="49" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H49" s="39" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I49" s="58">
         <v>2</v>
       </c>
       <c r="J49" s="41" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="50" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H50" s="39" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I50" s="58">
         <v>2</v>
       </c>
       <c r="J50" s="41" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="51" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H51" s="39" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="I51" s="58">
         <v>5</v>
       </c>
       <c r="J51" s="41" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="52" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H52" s="39" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="I52" s="58">
         <v>5</v>
       </c>
       <c r="J52" s="41" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="53" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H53" s="39" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="I53" s="58">
         <v>5</v>
       </c>
       <c r="J53" s="41" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="54" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H54" s="39" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="I54" s="58">
         <v>5</v>
       </c>
       <c r="J54" s="41" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="55" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H55" s="39" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I55" s="57">
         <v>5</v>
       </c>
       <c r="J55" s="41" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="56" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H56" s="39" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="I56" s="57">
         <v>5</v>
       </c>
       <c r="J56" s="41" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="57" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H57" s="39" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="I57" s="57">
         <v>5</v>
       </c>
       <c r="J57" s="41" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="58" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H58" s="39" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="I58" s="57">
         <v>5</v>
       </c>
       <c r="J58" s="41" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="59" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H59" s="39" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I59" s="57">
         <v>5</v>
       </c>
       <c r="J59" s="41" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="60" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H60" s="39" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="I60" s="57">
         <v>5</v>
       </c>
       <c r="J60" s="41" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="61" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H61" s="39" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="I61" s="57">
         <v>11.41666</v>
       </c>
       <c r="J61" s="41" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="62" spans="8:10" x14ac:dyDescent="0.35">
@@ -2754,181 +2763,193 @@
         <v>53</v>
       </c>
       <c r="I62" s="57">
-        <v>7.0670000000000002</v>
+        <v>4.5670000000000002</v>
       </c>
       <c r="J62" s="41" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
     </row>
     <row r="63" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H63" s="39" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="I63" s="58">
         <v>5</v>
       </c>
       <c r="J63" s="41" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="64" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H64" s="39" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="I64" s="58">
         <v>2.5</v>
       </c>
       <c r="J64" s="41" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="65" spans="3:10" x14ac:dyDescent="0.35">
       <c r="H65" s="39" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="I65" s="58">
         <v>2</v>
       </c>
       <c r="J65" s="41" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="66" spans="3:10" x14ac:dyDescent="0.35">
       <c r="H66" s="39" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="I66" s="58">
         <v>2</v>
       </c>
       <c r="J66" s="41" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="67" spans="3:10" x14ac:dyDescent="0.35">
       <c r="H67" s="39" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="I67" s="58">
         <v>2</v>
       </c>
       <c r="J67" s="41" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="68" spans="3:10" x14ac:dyDescent="0.35">
       <c r="C68" s="1"/>
       <c r="H68" s="39" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="I68" s="58">
         <v>1</v>
       </c>
       <c r="J68" s="41" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="69" spans="3:10" x14ac:dyDescent="0.35">
       <c r="C69" s="1"/>
-      <c r="H69" s="63" t="s">
-        <v>250</v>
+      <c r="H69" s="39" t="s">
+        <v>245</v>
       </c>
       <c r="I69" s="8">
         <f>5/8</f>
         <v>0.625</v>
       </c>
       <c r="J69" s="4" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="70" spans="3:10" x14ac:dyDescent="0.35">
       <c r="C70" s="1"/>
-      <c r="H70" s="63" t="s">
-        <v>251</v>
+      <c r="H70" s="39" t="s">
+        <v>246</v>
       </c>
       <c r="I70" s="9">
         <v>1</v>
       </c>
       <c r="J70" s="4" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="71" spans="3:10" x14ac:dyDescent="0.35">
-      <c r="H71" s="63" t="s">
-        <v>252</v>
+      <c r="H71" s="39" t="s">
+        <v>247</v>
       </c>
       <c r="I71" s="9">
         <v>0.5</v>
       </c>
       <c r="J71" s="4" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="72" spans="3:10" x14ac:dyDescent="0.35">
-      <c r="H72" s="63" t="s">
-        <v>253</v>
+      <c r="H72" s="39" t="s">
+        <v>248</v>
       </c>
       <c r="I72" s="9">
         <v>3.5</v>
       </c>
       <c r="J72" s="4" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="73" spans="3:10" x14ac:dyDescent="0.35">
-      <c r="H73" s="63" t="s">
-        <v>254</v>
+      <c r="H73" s="39" t="s">
+        <v>249</v>
       </c>
       <c r="I73" s="9">
         <v>0.5</v>
       </c>
       <c r="J73" s="4" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="74" spans="3:10" x14ac:dyDescent="0.35">
-      <c r="H74" s="63" t="s">
-        <v>263</v>
+      <c r="H74" s="39" t="s">
+        <v>258</v>
       </c>
       <c r="I74" s="8">
         <v>20</v>
       </c>
       <c r="J74" s="4" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
     </row>
     <row r="75" spans="3:10" x14ac:dyDescent="0.35">
-      <c r="H75" s="63" t="s">
-        <v>264</v>
+      <c r="H75" s="39" t="s">
+        <v>259</v>
       </c>
       <c r="I75" s="9">
         <v>0.5</v>
       </c>
       <c r="J75" s="4" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
     </row>
     <row r="76" spans="3:10" x14ac:dyDescent="0.35">
-      <c r="H76" s="63" t="s">
-        <v>265</v>
+      <c r="H76" s="39" t="s">
+        <v>260</v>
       </c>
       <c r="I76" s="9">
         <v>0.5</v>
       </c>
       <c r="J76" s="4" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
     </row>
     <row r="77" spans="3:10" x14ac:dyDescent="0.35">
       <c r="C77" s="1"/>
-      <c r="H77" s="2"/>
-      <c r="I77" s="57"/>
-      <c r="J77" s="41"/>
+      <c r="H77" s="39" t="s">
+        <v>278</v>
+      </c>
+      <c r="I77" s="9">
+        <v>1.5625</v>
+      </c>
+      <c r="J77" s="4" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="78" spans="3:10" x14ac:dyDescent="0.35">
       <c r="C78" s="1"/>
-      <c r="H78" s="2"/>
-      <c r="I78" s="57"/>
-      <c r="J78" s="41"/>
+      <c r="H78" s="39" t="s">
+        <v>279</v>
+      </c>
+      <c r="I78" s="9">
+        <v>1.5625</v>
+      </c>
+      <c r="J78" s="4" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="79" spans="3:10" x14ac:dyDescent="0.35">
       <c r="C79" s="1"/>
@@ -3118,16 +3139,16 @@
     </row>
     <row r="10" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C10" s="23"/>
-      <c r="E10" s="72" t="s">
+      <c r="E10" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="73"/>
-      <c r="G10" s="74"/>
-      <c r="J10" s="72" t="s">
+      <c r="F10" s="72"/>
+      <c r="G10" s="73"/>
+      <c r="J10" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="K10" s="73"/>
-      <c r="L10" s="74"/>
+      <c r="K10" s="72"/>
+      <c r="L10" s="73"/>
     </row>
     <row r="11" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C11" s="23"/>
@@ -3534,7 +3555,7 @@
         <v>11</v>
       </c>
       <c r="C4" s="37" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="5" spans="2:20" x14ac:dyDescent="0.35">
@@ -3579,17 +3600,17 @@
     </row>
     <row r="10" spans="2:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C10" s="23"/>
-      <c r="E10" s="72" t="s">
+      <c r="E10" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="73"/>
-      <c r="G10" s="74"/>
-      <c r="J10" s="72" t="s">
+      <c r="F10" s="72"/>
+      <c r="G10" s="73"/>
+      <c r="J10" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="K10" s="73"/>
-      <c r="L10" s="73"/>
-      <c r="M10" s="74"/>
+      <c r="K10" s="72"/>
+      <c r="L10" s="72"/>
+      <c r="M10" s="73"/>
     </row>
     <row r="11" spans="2:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C11" s="23"/>
@@ -3636,14 +3657,14 @@
         <v>8</v>
       </c>
       <c r="M12" s="19"/>
-      <c r="O12" s="75" t="s">
+      <c r="O12" s="74" t="s">
         <v>121</v>
       </c>
-      <c r="P12" s="75"/>
-      <c r="Q12" s="75"/>
-      <c r="R12" s="75"/>
-      <c r="S12" s="75"/>
-      <c r="T12" s="75"/>
+      <c r="P12" s="74"/>
+      <c r="Q12" s="74"/>
+      <c r="R12" s="74"/>
+      <c r="S12" s="74"/>
+      <c r="T12" s="74"/>
     </row>
     <row r="13" spans="2:20" x14ac:dyDescent="0.35">
       <c r="C13" s="23"/>
@@ -3666,12 +3687,12 @@
         <v>25</v>
       </c>
       <c r="M13" s="2"/>
-      <c r="O13" s="75"/>
-      <c r="P13" s="75"/>
-      <c r="Q13" s="75"/>
-      <c r="R13" s="75"/>
-      <c r="S13" s="75"/>
-      <c r="T13" s="75"/>
+      <c r="O13" s="74"/>
+      <c r="P13" s="74"/>
+      <c r="Q13" s="74"/>
+      <c r="R13" s="74"/>
+      <c r="S13" s="74"/>
+      <c r="T13" s="74"/>
     </row>
     <row r="14" spans="2:20" x14ac:dyDescent="0.35">
       <c r="C14" s="23"/>
@@ -3688,12 +3709,12 @@
         <v>25</v>
       </c>
       <c r="M14" s="2"/>
-      <c r="O14" s="75"/>
-      <c r="P14" s="75"/>
-      <c r="Q14" s="75"/>
-      <c r="R14" s="75"/>
-      <c r="S14" s="75"/>
-      <c r="T14" s="75"/>
+      <c r="O14" s="74"/>
+      <c r="P14" s="74"/>
+      <c r="Q14" s="74"/>
+      <c r="R14" s="74"/>
+      <c r="S14" s="74"/>
+      <c r="T14" s="74"/>
     </row>
     <row r="15" spans="2:20" x14ac:dyDescent="0.35">
       <c r="C15" s="23"/>
@@ -3710,12 +3731,12 @@
         <v>8</v>
       </c>
       <c r="M15" s="2"/>
-      <c r="O15" s="75"/>
-      <c r="P15" s="75"/>
-      <c r="Q15" s="75"/>
-      <c r="R15" s="75"/>
-      <c r="S15" s="75"/>
-      <c r="T15" s="75"/>
+      <c r="O15" s="74"/>
+      <c r="P15" s="74"/>
+      <c r="Q15" s="74"/>
+      <c r="R15" s="74"/>
+      <c r="S15" s="74"/>
+      <c r="T15" s="74"/>
     </row>
     <row r="16" spans="2:20" x14ac:dyDescent="0.35">
       <c r="C16" s="23"/>
@@ -3732,14 +3753,14 @@
         <v>111</v>
       </c>
       <c r="M16" s="2"/>
-      <c r="O16" s="75" t="s">
+      <c r="O16" s="74" t="s">
         <v>120</v>
       </c>
-      <c r="P16" s="75"/>
-      <c r="Q16" s="75"/>
-      <c r="R16" s="75"/>
-      <c r="S16" s="75"/>
-      <c r="T16" s="75"/>
+      <c r="P16" s="74"/>
+      <c r="Q16" s="74"/>
+      <c r="R16" s="74"/>
+      <c r="S16" s="74"/>
+      <c r="T16" s="74"/>
     </row>
     <row r="17" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C17" s="23"/>
@@ -3756,12 +3777,12 @@
         <v>111</v>
       </c>
       <c r="M17" s="2"/>
-      <c r="O17" s="75"/>
-      <c r="P17" s="75"/>
-      <c r="Q17" s="75"/>
-      <c r="R17" s="75"/>
-      <c r="S17" s="75"/>
-      <c r="T17" s="75"/>
+      <c r="O17" s="74"/>
+      <c r="P17" s="74"/>
+      <c r="Q17" s="74"/>
+      <c r="R17" s="74"/>
+      <c r="S17" s="74"/>
+      <c r="T17" s="74"/>
     </row>
     <row r="18" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C18" s="23"/>
@@ -3778,12 +3799,12 @@
         <v>151</v>
       </c>
       <c r="M18" s="2"/>
-      <c r="O18" s="75"/>
-      <c r="P18" s="75"/>
-      <c r="Q18" s="75"/>
-      <c r="R18" s="75"/>
-      <c r="S18" s="75"/>
-      <c r="T18" s="75"/>
+      <c r="O18" s="74"/>
+      <c r="P18" s="74"/>
+      <c r="Q18" s="74"/>
+      <c r="R18" s="74"/>
+      <c r="S18" s="74"/>
+      <c r="T18" s="74"/>
     </row>
     <row r="19" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C19" s="23"/>
@@ -3800,12 +3821,12 @@
         <v>151</v>
       </c>
       <c r="M19" s="2"/>
-      <c r="O19" s="75"/>
-      <c r="P19" s="75"/>
-      <c r="Q19" s="75"/>
-      <c r="R19" s="75"/>
-      <c r="S19" s="75"/>
-      <c r="T19" s="75"/>
+      <c r="O19" s="74"/>
+      <c r="P19" s="74"/>
+      <c r="Q19" s="74"/>
+      <c r="R19" s="74"/>
+      <c r="S19" s="74"/>
+      <c r="T19" s="74"/>
     </row>
     <row r="20" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C20" s="23"/>
@@ -3819,7 +3840,7 @@
         <v>2.8</v>
       </c>
       <c r="L20" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="M20" s="2"/>
     </row>
@@ -3835,17 +3856,17 @@
         <v>109.5</v>
       </c>
       <c r="L21" s="4" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="M21" s="2"/>
-      <c r="O21" s="76" t="s">
+      <c r="O21" s="75" t="s">
         <v>150</v>
       </c>
-      <c r="P21" s="76"/>
-      <c r="Q21" s="76"/>
-      <c r="R21" s="76"/>
-      <c r="S21" s="76"/>
-      <c r="T21" s="76"/>
+      <c r="P21" s="75"/>
+      <c r="Q21" s="75"/>
+      <c r="R21" s="75"/>
+      <c r="S21" s="75"/>
+      <c r="T21" s="75"/>
     </row>
     <row r="22" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C22" s="23"/>
@@ -3866,14 +3887,14 @@
       <c r="K23" s="9"/>
       <c r="L23" s="4"/>
       <c r="M23" s="2"/>
-      <c r="O23" s="75" t="s">
-        <v>217</v>
-      </c>
-      <c r="P23" s="75"/>
-      <c r="Q23" s="75"/>
-      <c r="R23" s="75"/>
-      <c r="S23" s="75"/>
-      <c r="T23" s="75"/>
+      <c r="O23" s="74" t="s">
+        <v>216</v>
+      </c>
+      <c r="P23" s="74"/>
+      <c r="Q23" s="74"/>
+      <c r="R23" s="74"/>
+      <c r="S23" s="74"/>
+      <c r="T23" s="74"/>
     </row>
     <row r="24" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C24" s="23"/>
@@ -3884,12 +3905,12 @@
       <c r="K24" s="9"/>
       <c r="L24" s="4"/>
       <c r="M24" s="2"/>
-      <c r="O24" s="75"/>
-      <c r="P24" s="75"/>
-      <c r="Q24" s="75"/>
-      <c r="R24" s="75"/>
-      <c r="S24" s="75"/>
-      <c r="T24" s="75"/>
+      <c r="O24" s="74"/>
+      <c r="P24" s="74"/>
+      <c r="Q24" s="74"/>
+      <c r="R24" s="74"/>
+      <c r="S24" s="74"/>
+      <c r="T24" s="74"/>
     </row>
     <row r="25" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C25" s="23"/>
@@ -3900,12 +3921,12 @@
       <c r="K25" s="9"/>
       <c r="L25" s="4"/>
       <c r="M25" s="2"/>
-      <c r="O25" s="75"/>
-      <c r="P25" s="75"/>
-      <c r="Q25" s="75"/>
-      <c r="R25" s="75"/>
-      <c r="S25" s="75"/>
-      <c r="T25" s="75"/>
+      <c r="O25" s="74"/>
+      <c r="P25" s="74"/>
+      <c r="Q25" s="74"/>
+      <c r="R25" s="74"/>
+      <c r="S25" s="74"/>
+      <c r="T25" s="74"/>
     </row>
     <row r="26" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C26" s="23"/>
@@ -3916,12 +3937,12 @@
       <c r="K26" s="9"/>
       <c r="L26" s="4"/>
       <c r="M26" s="2"/>
-      <c r="O26" s="75"/>
-      <c r="P26" s="75"/>
-      <c r="Q26" s="75"/>
-      <c r="R26" s="75"/>
-      <c r="S26" s="75"/>
-      <c r="T26" s="75"/>
+      <c r="O26" s="74"/>
+      <c r="P26" s="74"/>
+      <c r="Q26" s="74"/>
+      <c r="R26" s="74"/>
+      <c r="S26" s="74"/>
+      <c r="T26" s="74"/>
     </row>
     <row r="27" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C27" s="23"/>
@@ -3932,14 +3953,14 @@
       <c r="K27" s="9"/>
       <c r="L27" s="4"/>
       <c r="M27" s="2"/>
-      <c r="O27" s="75" t="s">
+      <c r="O27" s="74" t="s">
         <v>152</v>
       </c>
-      <c r="P27" s="75"/>
-      <c r="Q27" s="75"/>
-      <c r="R27" s="75"/>
-      <c r="S27" s="75"/>
-      <c r="T27" s="75"/>
+      <c r="P27" s="74"/>
+      <c r="Q27" s="74"/>
+      <c r="R27" s="74"/>
+      <c r="S27" s="74"/>
+      <c r="T27" s="74"/>
     </row>
     <row r="28" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C28" s="23"/>
@@ -3950,12 +3971,12 @@
       <c r="K28" s="9"/>
       <c r="L28" s="4"/>
       <c r="M28" s="2"/>
-      <c r="O28" s="75"/>
-      <c r="P28" s="75"/>
-      <c r="Q28" s="75"/>
-      <c r="R28" s="75"/>
-      <c r="S28" s="75"/>
-      <c r="T28" s="75"/>
+      <c r="O28" s="74"/>
+      <c r="P28" s="74"/>
+      <c r="Q28" s="74"/>
+      <c r="R28" s="74"/>
+      <c r="S28" s="74"/>
+      <c r="T28" s="74"/>
     </row>
     <row r="29" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C29" s="23"/>
@@ -3966,12 +3987,12 @@
       <c r="K29" s="9"/>
       <c r="L29" s="4"/>
       <c r="M29" s="2"/>
-      <c r="O29" s="75"/>
-      <c r="P29" s="75"/>
-      <c r="Q29" s="75"/>
-      <c r="R29" s="75"/>
-      <c r="S29" s="75"/>
-      <c r="T29" s="75"/>
+      <c r="O29" s="74"/>
+      <c r="P29" s="74"/>
+      <c r="Q29" s="74"/>
+      <c r="R29" s="74"/>
+      <c r="S29" s="74"/>
+      <c r="T29" s="74"/>
     </row>
     <row r="30" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C30" s="23"/>
@@ -3982,12 +4003,12 @@
       <c r="K30" s="9"/>
       <c r="L30" s="2"/>
       <c r="M30" s="2"/>
-      <c r="O30" s="75"/>
-      <c r="P30" s="75"/>
-      <c r="Q30" s="75"/>
-      <c r="R30" s="75"/>
-      <c r="S30" s="75"/>
-      <c r="T30" s="75"/>
+      <c r="O30" s="74"/>
+      <c r="P30" s="74"/>
+      <c r="Q30" s="74"/>
+      <c r="R30" s="74"/>
+      <c r="S30" s="74"/>
+      <c r="T30" s="74"/>
     </row>
     <row r="31" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C31" s="23"/>
@@ -4146,7 +4167,7 @@
     <col min="6" max="6" width="7.36328125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="16.36328125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="20.453125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9" customWidth="1"/>
     <col min="12" max="12" width="17" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="9.81640625" bestFit="1" customWidth="1"/>
   </cols>
@@ -4168,12 +4189,12 @@
         <v>44</v>
       </c>
     </row>
-    <row r="4" spans="2:12" ht="56" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:12" ht="64" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B4" s="27" t="s">
         <v>11</v>
       </c>
       <c r="C4" s="30" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.35">
@@ -4218,16 +4239,16 @@
     </row>
     <row r="10" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C10" s="23"/>
-      <c r="E10" s="72" t="s">
+      <c r="E10" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="73"/>
-      <c r="G10" s="74"/>
-      <c r="J10" s="72" t="s">
+      <c r="F10" s="72"/>
+      <c r="G10" s="73"/>
+      <c r="J10" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="K10" s="73"/>
-      <c r="L10" s="74"/>
+      <c r="K10" s="72"/>
+      <c r="L10" s="73"/>
     </row>
     <row r="11" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C11" s="23"/>
@@ -4349,7 +4370,8 @@
         <v>138</v>
       </c>
       <c r="K16" s="11">
-        <v>62</v>
+        <f>62-1-9/16</f>
+        <v>60.4375</v>
       </c>
       <c r="L16" s="42" t="s">
         <v>8</v>
@@ -4373,7 +4395,7 @@
         <v>7.35</v>
       </c>
       <c r="L17" s="42" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="18" spans="3:12" x14ac:dyDescent="0.35">
@@ -4448,7 +4470,7 @@
         <v>0.3</v>
       </c>
       <c r="L22" s="42" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="23" spans="3:12" x14ac:dyDescent="0.35">
@@ -4463,7 +4485,7 @@
         <v>176.4</v>
       </c>
       <c r="L23" s="42" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="24" spans="3:12" x14ac:dyDescent="0.35">
@@ -4478,7 +4500,7 @@
         <v>28.6</v>
       </c>
       <c r="L24" s="42" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="25" spans="3:12" x14ac:dyDescent="0.35">
@@ -4486,9 +4508,16 @@
       <c r="E25" s="2"/>
       <c r="F25" s="9"/>
       <c r="G25" s="2"/>
-      <c r="J25" s="2"/>
-      <c r="K25" s="11"/>
-      <c r="L25" s="42"/>
+      <c r="J25" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="K25" s="11">
+        <f>1+9/16</f>
+        <v>1.5625</v>
+      </c>
+      <c r="L25" s="42" t="s">
+        <v>165</v>
+      </c>
     </row>
     <row r="26" spans="3:12" x14ac:dyDescent="0.35">
       <c r="C26" s="23"/>
@@ -4699,7 +4728,7 @@
         <v>11</v>
       </c>
       <c r="C4" s="37" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.35">
@@ -4744,16 +4773,16 @@
     </row>
     <row r="10" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C10" s="23"/>
-      <c r="E10" s="72" t="s">
+      <c r="E10" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="73"/>
-      <c r="G10" s="74"/>
-      <c r="J10" s="72" t="s">
+      <c r="F10" s="72"/>
+      <c r="G10" s="73"/>
+      <c r="J10" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="K10" s="73"/>
-      <c r="L10" s="74"/>
+      <c r="K10" s="72"/>
+      <c r="L10" s="73"/>
     </row>
     <row r="11" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C11" s="23"/>
@@ -4836,7 +4865,7 @@
         <v>158</v>
       </c>
       <c r="L14" s="4" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.35">
@@ -4857,7 +4886,7 @@
         <v>159</v>
       </c>
       <c r="L15" s="4" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.35">
@@ -5152,7 +5181,7 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="17.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
     <col min="5" max="5" width="14.90625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="7.81640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="16.36328125" bestFit="1" customWidth="1"/>
@@ -5170,12 +5199,12 @@
         <v>165</v>
       </c>
     </row>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:12" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B3" s="27" t="s">
         <v>10</v>
       </c>
       <c r="C3" s="28" t="s">
-        <v>131</v>
+        <v>276</v>
       </c>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.35">
@@ -5183,7 +5212,7 @@
         <v>11</v>
       </c>
       <c r="C4" s="25" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.35">
@@ -5199,7 +5228,7 @@
         <v>13</v>
       </c>
       <c r="C6" s="25" t="s">
-        <v>170</v>
+        <v>281</v>
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.35">
@@ -5215,7 +5244,7 @@
         <v>31</v>
       </c>
       <c r="C8" s="25" t="s">
-        <v>166</v>
+        <v>280</v>
       </c>
     </row>
     <row r="9" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -5228,16 +5257,16 @@
     </row>
     <row r="10" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C10" s="23"/>
-      <c r="E10" s="72" t="s">
+      <c r="E10" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="73"/>
-      <c r="G10" s="74"/>
-      <c r="J10" s="72" t="s">
+      <c r="F10" s="72"/>
+      <c r="G10" s="73"/>
+      <c r="J10" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="K10" s="73"/>
-      <c r="L10" s="74"/>
+      <c r="K10" s="72"/>
+      <c r="L10" s="73"/>
     </row>
     <row r="11" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C11" s="23"/>
@@ -5266,7 +5295,7 @@
         <v>19</v>
       </c>
       <c r="F12" s="8">
-        <v>980.42</v>
+        <v>986.67</v>
       </c>
       <c r="G12" s="4" t="s">
         <v>62</v>
@@ -5284,19 +5313,19 @@
     <row r="13" spans="2:12" x14ac:dyDescent="0.35">
       <c r="C13" s="23"/>
       <c r="E13" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F13" s="9">
         <v>300</v>
       </c>
       <c r="G13" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="J13" s="38">
+        <v>6.25</v>
+      </c>
+      <c r="K13" s="9" t="s">
         <v>172</v>
-      </c>
-      <c r="J13" s="38">
-        <v>12.5</v>
-      </c>
-      <c r="K13" s="9" t="s">
-        <v>173</v>
       </c>
       <c r="L13" s="4" t="s">
         <v>8</v>
@@ -5317,7 +5346,7 @@
         <v>12.5</v>
       </c>
       <c r="K14" s="9" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="L14" s="4" t="s">
         <v>8</v>
@@ -5338,7 +5367,7 @@
         <v>148.44999999999999</v>
       </c>
       <c r="K15" s="9" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L15" s="4" t="s">
         <v>8</v>
@@ -5359,10 +5388,10 @@
         <v>1.55</v>
       </c>
       <c r="K16" s="9" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L16" s="4" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="17" spans="3:12" x14ac:dyDescent="0.35">
@@ -5371,38 +5400,72 @@
         <v>17</v>
       </c>
       <c r="F17" s="9">
-        <v>200</v>
+        <v>212.5</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="J17" s="38"/>
-      <c r="K17" s="9"/>
-      <c r="L17" s="4"/>
+      <c r="J17" s="38">
+        <f>1+9/16</f>
+        <v>1.5625</v>
+      </c>
+      <c r="K17" s="9" t="s">
+        <v>278</v>
+      </c>
+      <c r="L17" s="4" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="18" spans="3:12" x14ac:dyDescent="0.35">
       <c r="C18" s="23"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="9"/>
-      <c r="G18" s="2"/>
-      <c r="J18" s="38"/>
-      <c r="K18" s="9"/>
-      <c r="L18" s="4"/>
+      <c r="E18" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F18" s="9">
+        <f>9+3/8</f>
+        <v>9.375</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J18" s="38">
+        <f>1+9/16</f>
+        <v>1.5625</v>
+      </c>
+      <c r="K18" s="9" t="s">
+        <v>279</v>
+      </c>
+      <c r="L18" s="4" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="19" spans="3:12" x14ac:dyDescent="0.35">
       <c r="C19" s="23"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="2"/>
+      <c r="E19" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F19" s="9">
+        <v>2.5</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>50</v>
+      </c>
       <c r="J19" s="11"/>
       <c r="K19" s="9"/>
       <c r="L19" s="4"/>
     </row>
     <row r="20" spans="3:12" x14ac:dyDescent="0.35">
       <c r="C20" s="23"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="9"/>
-      <c r="G20" s="2"/>
+      <c r="E20" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="F20" s="9">
+        <f>1+9/16</f>
+        <v>1.5625</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>131</v>
+      </c>
       <c r="J20" s="11"/>
       <c r="K20" s="9"/>
       <c r="L20" s="4"/>
@@ -5645,7 +5708,7 @@
         <v>9</v>
       </c>
       <c r="E4" s="40" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="5" spans="4:14" ht="59.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -5653,7 +5716,7 @@
         <v>10</v>
       </c>
       <c r="E5" s="52" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="6" spans="4:14" x14ac:dyDescent="0.35">
@@ -5661,7 +5724,7 @@
         <v>11</v>
       </c>
       <c r="E6" s="41" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="7" spans="4:14" x14ac:dyDescent="0.35">
@@ -5675,7 +5738,7 @@
         <v>13</v>
       </c>
       <c r="E8" s="41" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="9" spans="4:14" x14ac:dyDescent="0.35">
@@ -5683,7 +5746,7 @@
         <v>14</v>
       </c>
       <c r="E9" s="41" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="10" spans="4:14" x14ac:dyDescent="0.35">
@@ -5703,16 +5766,16 @@
       </c>
     </row>
     <row r="12" spans="4:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="G12" s="89" t="s">
+      <c r="G12" s="88" t="s">
         <v>15</v>
       </c>
-      <c r="H12" s="90"/>
-      <c r="I12" s="91"/>
-      <c r="L12" s="89" t="s">
+      <c r="H12" s="89"/>
+      <c r="I12" s="90"/>
+      <c r="L12" s="88" t="s">
         <v>16</v>
       </c>
-      <c r="M12" s="90"/>
-      <c r="N12" s="91"/>
+      <c r="M12" s="89"/>
+      <c r="N12" s="90"/>
     </row>
     <row r="13" spans="4:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="G13" s="53" t="s">
@@ -5748,7 +5811,7 @@
         <v>2</v>
       </c>
       <c r="M14" s="19" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N14" s="40" t="s">
         <v>8</v>
@@ -5768,7 +5831,7 @@
         <v>2</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="N15" s="41" t="s">
         <v>8</v>
@@ -5788,7 +5851,7 @@
         <v>2</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="N16" s="41" t="s">
         <v>8</v>
@@ -5808,7 +5871,7 @@
         <v>5</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="N17" s="41" t="s">
         <v>8</v>
@@ -5828,7 +5891,7 @@
         <v>5</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="N18" s="41" t="s">
         <v>8</v>
@@ -5848,7 +5911,7 @@
         <v>5</v>
       </c>
       <c r="M19" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="N19" s="41" t="s">
         <v>8</v>
@@ -5862,13 +5925,13 @@
         <v>30.4666</v>
       </c>
       <c r="I20" s="41" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="L20" s="6">
         <v>5</v>
       </c>
       <c r="M20" s="2" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="N20" s="41" t="s">
         <v>8</v>
@@ -5882,13 +5945,13 @@
         <v>30.4666</v>
       </c>
       <c r="I21" s="41" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="L21" s="6">
         <v>5</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="N21" s="41" t="s">
         <v>8</v>
@@ -5908,7 +5971,7 @@
         <v>5</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="N22" s="41" t="s">
         <v>8</v>
@@ -5928,7 +5991,7 @@
         <v>5</v>
       </c>
       <c r="M23" s="2" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="N23" s="41" t="s">
         <v>8</v>
@@ -5948,7 +6011,7 @@
         <v>5</v>
       </c>
       <c r="M24" s="2" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="N24" s="41" t="s">
         <v>8</v>
@@ -5959,7 +6022,7 @@
         <v>5</v>
       </c>
       <c r="M25" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="N25" s="41" t="s">
         <v>8</v>
@@ -5970,7 +6033,7 @@
         <v>5</v>
       </c>
       <c r="M26" s="2" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="N26" s="41" t="s">
         <v>8</v>
@@ -5981,7 +6044,7 @@
         <v>11.41666</v>
       </c>
       <c r="M27" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="N27" s="41" t="s">
         <v>8</v>
@@ -5995,7 +6058,7 @@
         <v>5</v>
       </c>
       <c r="N28" s="41" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="29" spans="7:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -6041,7 +6104,7 @@
         <v>9</v>
       </c>
       <c r="C2" s="24" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="3" spans="2:15" x14ac:dyDescent="0.35">
@@ -6056,8 +6119,8 @@
       <c r="B4" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="64" t="s">
-        <v>257</v>
+      <c r="C4" s="63" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="5" spans="2:15" x14ac:dyDescent="0.35">
@@ -6065,7 +6128,7 @@
         <v>12</v>
       </c>
       <c r="C5" s="25" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="6" spans="2:15" x14ac:dyDescent="0.35">
@@ -6073,7 +6136,7 @@
         <v>13</v>
       </c>
       <c r="C6" s="25" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="7" spans="2:15" x14ac:dyDescent="0.35">
@@ -6081,7 +6144,7 @@
         <v>14</v>
       </c>
       <c r="C7" s="25" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="8" spans="2:15" x14ac:dyDescent="0.35">
@@ -6089,7 +6152,7 @@
         <v>31</v>
       </c>
       <c r="C8" s="25" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="9" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -6097,21 +6160,21 @@
         <v>32</v>
       </c>
       <c r="C9" s="26" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="10" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C10" s="23"/>
-      <c r="E10" s="72" t="s">
+      <c r="E10" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="73"/>
-      <c r="G10" s="74"/>
-      <c r="J10" s="72" t="s">
+      <c r="F10" s="72"/>
+      <c r="G10" s="73"/>
+      <c r="J10" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="K10" s="73"/>
-      <c r="L10" s="74"/>
+      <c r="K10" s="72"/>
+      <c r="L10" s="73"/>
     </row>
     <row r="11" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C11" s="23"/>
@@ -6173,10 +6236,10 @@
         <v>137</v>
       </c>
       <c r="L13" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="N13" s="49" t="s">
         <v>213</v>
-      </c>
-      <c r="N13" s="49" t="s">
-        <v>214</v>
       </c>
       <c r="O13" s="14" t="s">
         <v>25</v>
@@ -6200,7 +6263,7 @@
         <v>137</v>
       </c>
       <c r="L14" s="4" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="N14" s="5">
         <v>1</v>
@@ -6218,7 +6281,7 @@
         <v>180</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="J15" s="38"/>
       <c r="K15" s="9"/>
@@ -6296,7 +6359,7 @@
         <v>180</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="J19" s="11"/>
       <c r="K19" s="9"/>
@@ -6549,7 +6612,7 @@
         <v>9</v>
       </c>
       <c r="C2" s="24" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="3" spans="2:12" ht="101.5" x14ac:dyDescent="0.35">
@@ -6557,7 +6620,7 @@
         <v>10</v>
       </c>
       <c r="C3" s="28" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.35">
@@ -6577,7 +6640,7 @@
         <v>13</v>
       </c>
       <c r="C6" s="25" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.35">
@@ -6585,7 +6648,7 @@
         <v>14</v>
       </c>
       <c r="C7" s="25" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.35">
@@ -6593,7 +6656,7 @@
         <v>31</v>
       </c>
       <c r="C8" s="25" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
     </row>
     <row r="9" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -6601,21 +6664,21 @@
         <v>32</v>
       </c>
       <c r="C9" s="26" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
     </row>
     <row r="10" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C10" s="23"/>
-      <c r="E10" s="72" t="s">
+      <c r="E10" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="73"/>
-      <c r="G10" s="74"/>
-      <c r="J10" s="72" t="s">
+      <c r="F10" s="72"/>
+      <c r="G10" s="73"/>
+      <c r="J10" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="K10" s="73"/>
-      <c r="L10" s="74"/>
+      <c r="K10" s="72"/>
+      <c r="L10" s="73"/>
     </row>
     <row r="11" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C11" s="23"/>
@@ -6641,7 +6704,7 @@
     <row r="12" spans="2:12" x14ac:dyDescent="0.35">
       <c r="C12" s="23"/>
       <c r="E12" s="4" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="F12" s="8">
         <v>485.50555000000003</v>
@@ -6653,7 +6716,7 @@
         <v>5</v>
       </c>
       <c r="K12" s="8" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="L12" s="4" t="s">
         <v>8</v>
@@ -6674,7 +6737,7 @@
         <v>2.5</v>
       </c>
       <c r="K13" s="9" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="L13" s="4" t="s">
         <v>8</v>
@@ -6695,7 +6758,7 @@
         <v>2</v>
       </c>
       <c r="K14" s="9" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="L14" s="4" t="s">
         <v>8</v>
@@ -6716,7 +6779,7 @@
         <v>2</v>
       </c>
       <c r="K15" s="9" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="L15" s="4" t="s">
         <v>8</v>
@@ -6725,7 +6788,7 @@
     <row r="16" spans="2:12" x14ac:dyDescent="0.35">
       <c r="C16" s="23"/>
       <c r="E16" s="2" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="F16" s="9">
         <v>72</v>
@@ -6737,7 +6800,7 @@
         <v>2</v>
       </c>
       <c r="K16" s="9" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="L16" s="4" t="s">
         <v>8</v>
@@ -6758,7 +6821,7 @@
         <v>1</v>
       </c>
       <c r="K17" s="9" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="L17" s="4" t="s">
         <v>8</v>
@@ -6767,13 +6830,13 @@
     <row r="18" spans="3:12" x14ac:dyDescent="0.35">
       <c r="C18" s="23"/>
       <c r="E18" s="2" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="F18" s="9">
         <v>392.66660000000002</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="J18" s="38"/>
       <c r="K18" s="9"/>
@@ -6797,7 +6860,7 @@
     <row r="20" spans="3:12" x14ac:dyDescent="0.35">
       <c r="C20" s="23"/>
       <c r="E20" s="2" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="F20" s="9">
         <v>72</v>
@@ -6812,13 +6875,13 @@
     <row r="21" spans="3:12" x14ac:dyDescent="0.35">
       <c r="C21" s="23"/>
       <c r="E21" s="2" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="F21" s="9">
         <v>515</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="J21" s="11"/>
       <c r="K21" s="9"/>
@@ -6827,7 +6890,7 @@
     <row r="22" spans="3:12" x14ac:dyDescent="0.35">
       <c r="C22" s="23"/>
       <c r="E22" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F22" s="9">
         <v>1.55</v>
@@ -7059,7 +7122,7 @@
         <v>9</v>
       </c>
       <c r="C2" s="24" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="3" spans="2:12" ht="58" x14ac:dyDescent="0.35">
@@ -7067,7 +7130,7 @@
         <v>10</v>
       </c>
       <c r="C3" s="31" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.35">
@@ -7087,7 +7150,7 @@
         <v>13</v>
       </c>
       <c r="C6" s="25" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.35">
@@ -7095,7 +7158,7 @@
         <v>14</v>
       </c>
       <c r="C7" s="25" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.35">
@@ -7111,21 +7174,21 @@
         <v>32</v>
       </c>
       <c r="C9" s="26" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
     </row>
     <row r="10" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C10" s="23"/>
-      <c r="E10" s="72" t="s">
+      <c r="E10" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="73"/>
-      <c r="G10" s="74"/>
-      <c r="J10" s="72" t="s">
+      <c r="F10" s="72"/>
+      <c r="G10" s="73"/>
+      <c r="J10" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="K10" s="73"/>
-      <c r="L10" s="74"/>
+      <c r="K10" s="72"/>
+      <c r="L10" s="73"/>
     </row>
     <row r="11" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C11" s="23"/>
@@ -7160,7 +7223,7 @@
         <v>33</v>
       </c>
       <c r="J12" s="38" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="K12" s="8">
         <f>5/8</f>
@@ -7179,10 +7242,10 @@
         <v>138.01249999999999</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="J13" s="38" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="K13" s="9">
         <v>1</v>
@@ -7200,10 +7263,10 @@
         <v>98.243700000000004</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="J14" s="38" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="K14" s="9">
         <v>0.5</v>
@@ -7224,7 +7287,7 @@
         <v>131</v>
       </c>
       <c r="J15" s="38" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="K15" s="9">
         <v>3.5</v>
@@ -7245,7 +7308,7 @@
         <v>22</v>
       </c>
       <c r="J16" s="38" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="K16" s="9">
         <v>0.5</v>
@@ -7257,7 +7320,7 @@
     <row r="17" spans="3:12" x14ac:dyDescent="0.35">
       <c r="C17" s="23"/>
       <c r="E17" s="2" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="F17" s="9">
         <v>110.01</v>
@@ -7278,7 +7341,7 @@
         <v>46</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J18" s="38"/>
       <c r="K18" s="9"/>
@@ -7287,7 +7350,7 @@
     <row r="19" spans="3:12" x14ac:dyDescent="0.35">
       <c r="C19" s="23"/>
       <c r="E19" s="2" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="F19" s="9">
         <v>5</v>
@@ -7302,7 +7365,7 @@
     <row r="20" spans="3:12" x14ac:dyDescent="0.35">
       <c r="C20" s="23"/>
       <c r="E20" s="2" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="F20" s="9">
         <v>0.5</v>
@@ -7552,76 +7615,76 @@
       <c r="B2" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="66" t="s">
-        <v>255</v>
+      <c r="C2" s="65" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="3" spans="2:12" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B3" s="51" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="67" t="s">
-        <v>261</v>
+      <c r="C3" s="66" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="4" spans="2:12" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="71" t="s">
+      <c r="B4" s="70" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="70"/>
+      <c r="C4" s="69"/>
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B5" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="68"/>
+      <c r="C5" s="67"/>
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B6" s="17" t="s">
-        <v>266</v>
-      </c>
-      <c r="C6" s="68" t="s">
-        <v>272</v>
+        <v>261</v>
+      </c>
+      <c r="C6" s="67" t="s">
+        <v>267</v>
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B7" s="17" t="s">
-        <v>267</v>
-      </c>
-      <c r="C7" s="68" t="s">
-        <v>273</v>
+        <v>262</v>
+      </c>
+      <c r="C7" s="67" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B8" s="17" t="s">
-        <v>268</v>
-      </c>
-      <c r="C8" s="68" t="s">
-        <v>274</v>
+        <v>263</v>
+      </c>
+      <c r="C8" s="67" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B9" s="17" t="s">
-        <v>269</v>
-      </c>
-      <c r="C9" s="68" t="s">
-        <v>275</v>
+        <v>264</v>
+      </c>
+      <c r="C9" s="67" t="s">
+        <v>270</v>
       </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B10" s="17" t="s">
-        <v>270</v>
-      </c>
-      <c r="C10" s="68" t="s">
-        <v>276</v>
+        <v>265</v>
+      </c>
+      <c r="C10" s="67" t="s">
+        <v>271</v>
       </c>
     </row>
     <row r="11" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B11" s="18" t="s">
-        <v>271</v>
-      </c>
-      <c r="C11" s="69" t="s">
-        <v>277</v>
+        <v>266</v>
+      </c>
+      <c r="C11" s="68" t="s">
+        <v>272</v>
       </c>
     </row>
     <row r="12" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -7629,16 +7692,16 @@
     </row>
     <row r="13" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C13" s="23"/>
-      <c r="E13" s="72" t="s">
+      <c r="E13" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="F13" s="73"/>
-      <c r="G13" s="74"/>
-      <c r="J13" s="72" t="s">
+      <c r="F13" s="72"/>
+      <c r="G13" s="73"/>
+      <c r="J13" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="K13" s="73"/>
-      <c r="L13" s="74"/>
+      <c r="K13" s="72"/>
+      <c r="L13" s="73"/>
     </row>
     <row r="14" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C14" s="23"/>
@@ -7673,7 +7736,7 @@
         <v>151</v>
       </c>
       <c r="J15" s="38" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="K15" s="8">
         <v>20</v>
@@ -7694,7 +7757,7 @@
         <v>21</v>
       </c>
       <c r="J16" s="38" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="K16" s="9">
         <v>0.5</v>
@@ -7706,16 +7769,16 @@
     <row r="17" spans="3:12" x14ac:dyDescent="0.35">
       <c r="C17" s="23"/>
       <c r="E17" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F17" s="9">
         <v>25</v>
       </c>
       <c r="G17" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="J17" s="38" t="s">
         <v>260</v>
-      </c>
-      <c r="J17" s="38" t="s">
-        <v>265</v>
       </c>
       <c r="K17" s="9">
         <v>0.5</v>
@@ -7733,7 +7796,7 @@
         <v>40.888800000000003</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="J18" s="38"/>
       <c r="K18" s="9"/>
@@ -7748,7 +7811,7 @@
         <v>66.666600000000003</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="J19" s="38"/>
       <c r="K19" s="9"/>
@@ -7763,7 +7826,7 @@
         <v>72.8</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="J20" s="38"/>
       <c r="K20" s="9"/>
@@ -8045,16 +8108,16 @@
       <c r="D4" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="72" t="s">
+      <c r="F4" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="G4" s="73"/>
-      <c r="H4" s="74"/>
-      <c r="K4" s="72" t="s">
+      <c r="G4" s="72"/>
+      <c r="H4" s="73"/>
+      <c r="K4" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="L4" s="73"/>
-      <c r="M4" s="74"/>
+      <c r="L4" s="72"/>
+      <c r="M4" s="73"/>
     </row>
     <row r="5" spans="3:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C5" s="17" t="s">
@@ -8433,10 +8496,11 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="17.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.6328125" style="23" customWidth="1"/>
+    <col min="4" max="4" width="24.90625" style="23" customWidth="1"/>
     <col min="6" max="6" width="7.26953125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="7.81640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.453125" customWidth="1"/>
     <col min="11" max="11" width="8.26953125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="8.81640625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="27" bestFit="1" customWidth="1"/>
@@ -8466,7 +8530,7 @@
         <v>11</v>
       </c>
       <c r="D6" s="30" t="s">
-        <v>241</v>
+        <v>277</v>
       </c>
     </row>
     <row r="7" spans="3:21" x14ac:dyDescent="0.35">
@@ -8511,17 +8575,17 @@
     </row>
     <row r="12" spans="3:21" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="13" spans="3:21" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="F13" s="72" t="s">
+      <c r="F13" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="G13" s="73"/>
-      <c r="H13" s="74"/>
-      <c r="K13" s="72" t="s">
+      <c r="G13" s="72"/>
+      <c r="H13" s="73"/>
+      <c r="K13" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="L13" s="73"/>
-      <c r="M13" s="73"/>
-      <c r="N13" s="74"/>
+      <c r="L13" s="72"/>
+      <c r="M13" s="72"/>
+      <c r="N13" s="73"/>
     </row>
     <row r="14" spans="3:21" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="F14" s="14" t="s">
@@ -8545,14 +8609,14 @@
       <c r="N14" s="34" t="s">
         <v>112</v>
       </c>
-      <c r="P14" s="75" t="s">
+      <c r="P14" s="74" t="s">
         <v>115</v>
       </c>
-      <c r="Q14" s="75"/>
-      <c r="R14" s="75"/>
-      <c r="S14" s="75"/>
-      <c r="T14" s="75"/>
-      <c r="U14" s="75"/>
+      <c r="Q14" s="74"/>
+      <c r="R14" s="74"/>
+      <c r="S14" s="74"/>
+      <c r="T14" s="74"/>
+      <c r="U14" s="74"/>
     </row>
     <row r="15" spans="3:21" x14ac:dyDescent="0.35">
       <c r="F15" s="4" t="s">
@@ -8568,18 +8632,18 @@
         <v>35</v>
       </c>
       <c r="L15" s="8">
-        <v>1837.835</v>
+        <v>1828.46</v>
       </c>
       <c r="M15" s="4" t="s">
         <v>25</v>
       </c>
       <c r="N15" s="19"/>
-      <c r="P15" s="75"/>
-      <c r="Q15" s="75"/>
-      <c r="R15" s="75"/>
-      <c r="S15" s="75"/>
-      <c r="T15" s="75"/>
-      <c r="U15" s="75"/>
+      <c r="P15" s="74"/>
+      <c r="Q15" s="74"/>
+      <c r="R15" s="74"/>
+      <c r="S15" s="74"/>
+      <c r="T15" s="74"/>
+      <c r="U15" s="74"/>
     </row>
     <row r="16" spans="3:21" x14ac:dyDescent="0.35">
       <c r="F16" s="2" t="s">
@@ -8603,12 +8667,12 @@
       <c r="N16" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="P16" s="75"/>
-      <c r="Q16" s="75"/>
-      <c r="R16" s="75"/>
-      <c r="S16" s="75"/>
-      <c r="T16" s="75"/>
-      <c r="U16" s="75"/>
+      <c r="P16" s="74"/>
+      <c r="Q16" s="74"/>
+      <c r="R16" s="74"/>
+      <c r="S16" s="74"/>
+      <c r="T16" s="74"/>
+      <c r="U16" s="74"/>
     </row>
     <row r="17" spans="6:21" x14ac:dyDescent="0.35">
       <c r="F17" s="2"/>
@@ -8626,12 +8690,12 @@
       <c r="N17" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="P17" s="75"/>
-      <c r="Q17" s="75"/>
-      <c r="R17" s="75"/>
-      <c r="S17" s="75"/>
-      <c r="T17" s="75"/>
-      <c r="U17" s="75"/>
+      <c r="P17" s="74"/>
+      <c r="Q17" s="74"/>
+      <c r="R17" s="74"/>
+      <c r="S17" s="74"/>
+      <c r="T17" s="74"/>
+      <c r="U17" s="74"/>
     </row>
     <row r="18" spans="6:21" x14ac:dyDescent="0.35">
       <c r="F18" s="2"/>
@@ -8678,17 +8742,17 @@
         <v>150</v>
       </c>
       <c r="M20" s="2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="N20" s="2"/>
-      <c r="P20" s="76" t="s">
+      <c r="P20" s="75" t="s">
         <v>150</v>
       </c>
-      <c r="Q20" s="76"/>
-      <c r="R20" s="76"/>
-      <c r="S20" s="76"/>
-      <c r="T20" s="76"/>
-      <c r="U20" s="76"/>
+      <c r="Q20" s="75"/>
+      <c r="R20" s="75"/>
+      <c r="S20" s="75"/>
+      <c r="T20" s="75"/>
+      <c r="U20" s="75"/>
     </row>
     <row r="21" spans="6:21" x14ac:dyDescent="0.35">
       <c r="F21" s="2"/>
@@ -8701,7 +8765,7 @@
         <v>12.013</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="N21" s="2"/>
     </row>
@@ -8709,18 +8773,25 @@
       <c r="F22" s="2"/>
       <c r="G22" s="9"/>
       <c r="H22" s="2"/>
-      <c r="K22" s="2"/>
-      <c r="L22" s="9"/>
-      <c r="M22" s="2"/>
+      <c r="K22" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="L22" s="9">
+        <f>9+3/8</f>
+        <v>9.375</v>
+      </c>
+      <c r="M22" s="2" t="s">
+        <v>165</v>
+      </c>
       <c r="N22" s="2"/>
-      <c r="P22" s="75" t="s">
-        <v>180</v>
-      </c>
-      <c r="Q22" s="75"/>
-      <c r="R22" s="75"/>
-      <c r="S22" s="75"/>
-      <c r="T22" s="75"/>
-      <c r="U22" s="75"/>
+      <c r="P22" s="74" t="s">
+        <v>179</v>
+      </c>
+      <c r="Q22" s="74"/>
+      <c r="R22" s="74"/>
+      <c r="S22" s="74"/>
+      <c r="T22" s="74"/>
+      <c r="U22" s="74"/>
     </row>
     <row r="23" spans="6:21" x14ac:dyDescent="0.35">
       <c r="F23" s="2"/>
@@ -8730,12 +8801,12 @@
       <c r="L23" s="9"/>
       <c r="M23" s="2"/>
       <c r="N23" s="2"/>
-      <c r="P23" s="75"/>
-      <c r="Q23" s="75"/>
-      <c r="R23" s="75"/>
-      <c r="S23" s="75"/>
-      <c r="T23" s="75"/>
-      <c r="U23" s="75"/>
+      <c r="P23" s="74"/>
+      <c r="Q23" s="74"/>
+      <c r="R23" s="74"/>
+      <c r="S23" s="74"/>
+      <c r="T23" s="74"/>
+      <c r="U23" s="74"/>
     </row>
     <row r="24" spans="6:21" x14ac:dyDescent="0.35">
       <c r="F24" s="2"/>
@@ -8745,12 +8816,12 @@
       <c r="L24" s="9"/>
       <c r="M24" s="2"/>
       <c r="N24" s="2"/>
-      <c r="P24" s="75"/>
-      <c r="Q24" s="75"/>
-      <c r="R24" s="75"/>
-      <c r="S24" s="75"/>
-      <c r="T24" s="75"/>
-      <c r="U24" s="75"/>
+      <c r="P24" s="74"/>
+      <c r="Q24" s="74"/>
+      <c r="R24" s="74"/>
+      <c r="S24" s="74"/>
+      <c r="T24" s="74"/>
+      <c r="U24" s="74"/>
     </row>
     <row r="25" spans="6:21" x14ac:dyDescent="0.35">
       <c r="F25" s="2"/>
@@ -8760,12 +8831,12 @@
       <c r="L25" s="9"/>
       <c r="M25" s="2"/>
       <c r="N25" s="2"/>
-      <c r="P25" s="75"/>
-      <c r="Q25" s="75"/>
-      <c r="R25" s="75"/>
-      <c r="S25" s="75"/>
-      <c r="T25" s="75"/>
-      <c r="U25" s="75"/>
+      <c r="P25" s="74"/>
+      <c r="Q25" s="74"/>
+      <c r="R25" s="74"/>
+      <c r="S25" s="74"/>
+      <c r="T25" s="74"/>
+      <c r="U25" s="74"/>
     </row>
     <row r="26" spans="6:21" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="F26" s="2"/>
@@ -8775,14 +8846,14 @@
       <c r="L26" s="9"/>
       <c r="M26" s="2"/>
       <c r="N26" s="2"/>
-      <c r="P26" s="75" t="s">
-        <v>181</v>
-      </c>
-      <c r="Q26" s="75"/>
-      <c r="R26" s="75"/>
-      <c r="S26" s="75"/>
-      <c r="T26" s="75"/>
-      <c r="U26" s="75"/>
+      <c r="P26" s="74" t="s">
+        <v>180</v>
+      </c>
+      <c r="Q26" s="74"/>
+      <c r="R26" s="74"/>
+      <c r="S26" s="74"/>
+      <c r="T26" s="74"/>
+      <c r="U26" s="74"/>
     </row>
     <row r="27" spans="6:21" x14ac:dyDescent="0.35">
       <c r="F27" s="2"/>
@@ -8792,12 +8863,12 @@
       <c r="L27" s="9"/>
       <c r="M27" s="2"/>
       <c r="N27" s="2"/>
-      <c r="P27" s="75"/>
-      <c r="Q27" s="75"/>
-      <c r="R27" s="75"/>
-      <c r="S27" s="75"/>
-      <c r="T27" s="75"/>
-      <c r="U27" s="75"/>
+      <c r="P27" s="74"/>
+      <c r="Q27" s="74"/>
+      <c r="R27" s="74"/>
+      <c r="S27" s="74"/>
+      <c r="T27" s="74"/>
+      <c r="U27" s="74"/>
     </row>
     <row r="28" spans="6:21" x14ac:dyDescent="0.35">
       <c r="F28" s="2"/>
@@ -8807,12 +8878,12 @@
       <c r="L28" s="9"/>
       <c r="M28" s="2"/>
       <c r="N28" s="2"/>
-      <c r="P28" s="75"/>
-      <c r="Q28" s="75"/>
-      <c r="R28" s="75"/>
-      <c r="S28" s="75"/>
-      <c r="T28" s="75"/>
-      <c r="U28" s="75"/>
+      <c r="P28" s="74"/>
+      <c r="Q28" s="74"/>
+      <c r="R28" s="74"/>
+      <c r="S28" s="74"/>
+      <c r="T28" s="74"/>
+      <c r="U28" s="74"/>
     </row>
     <row r="29" spans="6:21" x14ac:dyDescent="0.35">
       <c r="F29" s="2"/>
@@ -8822,12 +8893,12 @@
       <c r="L29" s="9"/>
       <c r="M29" s="2"/>
       <c r="N29" s="2"/>
-      <c r="P29" s="75"/>
-      <c r="Q29" s="75"/>
-      <c r="R29" s="75"/>
-      <c r="S29" s="75"/>
-      <c r="T29" s="75"/>
-      <c r="U29" s="75"/>
+      <c r="P29" s="74"/>
+      <c r="Q29" s="74"/>
+      <c r="R29" s="74"/>
+      <c r="S29" s="74"/>
+      <c r="T29" s="74"/>
+      <c r="U29" s="74"/>
     </row>
     <row r="30" spans="6:21" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="F30" s="2"/>
@@ -8837,14 +8908,14 @@
       <c r="L30" s="9"/>
       <c r="M30" s="2"/>
       <c r="N30" s="2"/>
-      <c r="P30" s="75" t="s">
-        <v>243</v>
-      </c>
-      <c r="Q30" s="75"/>
-      <c r="R30" s="75"/>
-      <c r="S30" s="75"/>
-      <c r="T30" s="75"/>
-      <c r="U30" s="75"/>
+      <c r="P30" s="74" t="s">
+        <v>273</v>
+      </c>
+      <c r="Q30" s="74"/>
+      <c r="R30" s="74"/>
+      <c r="S30" s="74"/>
+      <c r="T30" s="74"/>
+      <c r="U30" s="74"/>
     </row>
     <row r="31" spans="6:21" x14ac:dyDescent="0.35">
       <c r="F31" s="2"/>
@@ -8854,12 +8925,12 @@
       <c r="L31" s="9"/>
       <c r="M31" s="2"/>
       <c r="N31" s="2"/>
-      <c r="P31" s="75"/>
-      <c r="Q31" s="75"/>
-      <c r="R31" s="75"/>
-      <c r="S31" s="75"/>
-      <c r="T31" s="75"/>
-      <c r="U31" s="75"/>
+      <c r="P31" s="74"/>
+      <c r="Q31" s="74"/>
+      <c r="R31" s="74"/>
+      <c r="S31" s="74"/>
+      <c r="T31" s="74"/>
+      <c r="U31" s="74"/>
     </row>
     <row r="32" spans="6:21" x14ac:dyDescent="0.35">
       <c r="F32" s="2"/>
@@ -8869,12 +8940,12 @@
       <c r="L32" s="9"/>
       <c r="M32" s="2"/>
       <c r="N32" s="2"/>
-      <c r="P32" s="75"/>
-      <c r="Q32" s="75"/>
-      <c r="R32" s="75"/>
-      <c r="S32" s="75"/>
-      <c r="T32" s="75"/>
-      <c r="U32" s="75"/>
+      <c r="P32" s="74"/>
+      <c r="Q32" s="74"/>
+      <c r="R32" s="74"/>
+      <c r="S32" s="74"/>
+      <c r="T32" s="74"/>
+      <c r="U32" s="74"/>
     </row>
     <row r="33" spans="6:21" x14ac:dyDescent="0.35">
       <c r="F33" s="2"/>
@@ -8884,12 +8955,12 @@
       <c r="L33" s="9"/>
       <c r="M33" s="2"/>
       <c r="N33" s="2"/>
-      <c r="P33" s="75"/>
-      <c r="Q33" s="75"/>
-      <c r="R33" s="75"/>
-      <c r="S33" s="75"/>
-      <c r="T33" s="75"/>
-      <c r="U33" s="75"/>
+      <c r="P33" s="74"/>
+      <c r="Q33" s="74"/>
+      <c r="R33" s="74"/>
+      <c r="S33" s="74"/>
+      <c r="T33" s="74"/>
+      <c r="U33" s="74"/>
     </row>
     <row r="34" spans="6:21" x14ac:dyDescent="0.35">
       <c r="F34" s="2"/>
@@ -8980,6 +9051,10 @@
       <c r="L43" s="9"/>
       <c r="M43" s="2"/>
       <c r="N43" s="2"/>
+      <c r="R43">
+        <f>277.832-9-3/8</f>
+        <v>268.45699999999999</v>
+      </c>
     </row>
     <row r="44" spans="6:21" x14ac:dyDescent="0.35">
       <c r="F44" s="2"/>
@@ -9036,7 +9111,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F1350C4-6C4D-4B59-A3BC-5B1F652DB40B}">
-  <dimension ref="B1:O48"/>
+  <dimension ref="B1:L45"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="17.81640625" bestFit="1" customWidth="1"/>
@@ -9067,12 +9142,12 @@
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="2:12" ht="58" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:12" ht="76.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B4" s="29" t="s">
         <v>11</v>
       </c>
       <c r="C4" s="31" t="s">
-        <v>239</v>
+        <v>274</v>
       </c>
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.35">
@@ -9120,16 +9195,16 @@
     </row>
     <row r="11" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C11" s="23"/>
-      <c r="E11" s="72" t="s">
+      <c r="E11" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="F11" s="73"/>
-      <c r="G11" s="74"/>
-      <c r="J11" s="72" t="s">
+      <c r="F11" s="72"/>
+      <c r="G11" s="73"/>
+      <c r="J11" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="K11" s="73"/>
-      <c r="L11" s="74"/>
+      <c r="K11" s="72"/>
+      <c r="L11" s="73"/>
     </row>
     <row r="12" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C12" s="23"/>
@@ -9167,7 +9242,7 @@
         <v>53</v>
       </c>
       <c r="K13" s="8">
-        <v>7.0670000000000002</v>
+        <v>4.5670000000000002</v>
       </c>
       <c r="L13" s="4" t="s">
         <v>8</v>
@@ -9236,7 +9311,7 @@
         <v>9.6</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="18" spans="3:12" x14ac:dyDescent="0.35">
@@ -9251,7 +9326,7 @@
         <v>72</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="19" spans="3:12" x14ac:dyDescent="0.35">
@@ -9266,7 +9341,7 @@
         <v>5</v>
       </c>
       <c r="L19" s="2" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="20" spans="3:12" x14ac:dyDescent="0.35">
@@ -9274,9 +9349,15 @@
       <c r="E20" s="2"/>
       <c r="F20" s="9"/>
       <c r="G20" s="2"/>
-      <c r="J20" s="2"/>
-      <c r="K20" s="9"/>
-      <c r="L20" s="2"/>
+      <c r="J20" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="K20" s="9">
+        <v>2.5</v>
+      </c>
+      <c r="L20" s="2" t="s">
+        <v>275</v>
+      </c>
     </row>
     <row r="21" spans="3:12" x14ac:dyDescent="0.35">
       <c r="C21" s="23"/>
@@ -9386,7 +9467,7 @@
       <c r="K32" s="9"/>
       <c r="L32" s="2"/>
     </row>
-    <row r="33" spans="3:15" x14ac:dyDescent="0.35">
+    <row r="33" spans="3:12" x14ac:dyDescent="0.35">
       <c r="C33" s="23"/>
       <c r="E33" s="2"/>
       <c r="F33" s="9"/>
@@ -9395,7 +9476,7 @@
       <c r="K33" s="9"/>
       <c r="L33" s="2"/>
     </row>
-    <row r="34" spans="3:15" x14ac:dyDescent="0.35">
+    <row r="34" spans="3:12" x14ac:dyDescent="0.35">
       <c r="C34" s="23"/>
       <c r="E34" s="2"/>
       <c r="F34" s="9"/>
@@ -9404,7 +9485,7 @@
       <c r="K34" s="9"/>
       <c r="L34" s="2"/>
     </row>
-    <row r="35" spans="3:15" x14ac:dyDescent="0.35">
+    <row r="35" spans="3:12" x14ac:dyDescent="0.35">
       <c r="C35" s="23"/>
       <c r="E35" s="2"/>
       <c r="F35" s="9"/>
@@ -9413,7 +9494,7 @@
       <c r="K35" s="9"/>
       <c r="L35" s="2"/>
     </row>
-    <row r="36" spans="3:15" x14ac:dyDescent="0.35">
+    <row r="36" spans="3:12" x14ac:dyDescent="0.35">
       <c r="C36" s="23"/>
       <c r="E36" s="2"/>
       <c r="F36" s="9"/>
@@ -9422,7 +9503,7 @@
       <c r="K36" s="9"/>
       <c r="L36" s="2"/>
     </row>
-    <row r="37" spans="3:15" x14ac:dyDescent="0.35">
+    <row r="37" spans="3:12" x14ac:dyDescent="0.35">
       <c r="E37" s="2"/>
       <c r="F37" s="9"/>
       <c r="G37" s="2"/>
@@ -9430,7 +9511,7 @@
       <c r="K37" s="9"/>
       <c r="L37" s="2"/>
     </row>
-    <row r="38" spans="3:15" x14ac:dyDescent="0.35">
+    <row r="38" spans="3:12" x14ac:dyDescent="0.35">
       <c r="E38" s="2"/>
       <c r="F38" s="9"/>
       <c r="G38" s="2"/>
@@ -9438,7 +9519,7 @@
       <c r="K38" s="9"/>
       <c r="L38" s="2"/>
     </row>
-    <row r="39" spans="3:15" x14ac:dyDescent="0.35">
+    <row r="39" spans="3:12" x14ac:dyDescent="0.35">
       <c r="E39" s="2"/>
       <c r="F39" s="9"/>
       <c r="G39" s="2"/>
@@ -9446,7 +9527,7 @@
       <c r="K39" s="9"/>
       <c r="L39" s="2"/>
     </row>
-    <row r="40" spans="3:15" x14ac:dyDescent="0.35">
+    <row r="40" spans="3:12" x14ac:dyDescent="0.35">
       <c r="E40" s="2"/>
       <c r="F40" s="9"/>
       <c r="G40" s="2"/>
@@ -9454,7 +9535,7 @@
       <c r="K40" s="9"/>
       <c r="L40" s="2"/>
     </row>
-    <row r="41" spans="3:15" x14ac:dyDescent="0.35">
+    <row r="41" spans="3:12" x14ac:dyDescent="0.35">
       <c r="E41" s="2"/>
       <c r="F41" s="9"/>
       <c r="G41" s="2"/>
@@ -9462,7 +9543,7 @@
       <c r="K41" s="9"/>
       <c r="L41" s="2"/>
     </row>
-    <row r="42" spans="3:15" x14ac:dyDescent="0.35">
+    <row r="42" spans="3:12" x14ac:dyDescent="0.35">
       <c r="E42" s="2"/>
       <c r="F42" s="9"/>
       <c r="G42" s="2"/>
@@ -9470,7 +9551,7 @@
       <c r="K42" s="9"/>
       <c r="L42" s="2"/>
     </row>
-    <row r="43" spans="3:15" x14ac:dyDescent="0.35">
+    <row r="43" spans="3:12" x14ac:dyDescent="0.35">
       <c r="E43" s="2"/>
       <c r="F43" s="9"/>
       <c r="G43" s="2"/>
@@ -9478,7 +9559,7 @@
       <c r="K43" s="9"/>
       <c r="L43" s="2"/>
     </row>
-    <row r="44" spans="3:15" x14ac:dyDescent="0.35">
+    <row r="44" spans="3:12" x14ac:dyDescent="0.35">
       <c r="E44" s="2"/>
       <c r="F44" s="9"/>
       <c r="G44" s="2"/>
@@ -9486,18 +9567,13 @@
       <c r="K44" s="9"/>
       <c r="L44" s="2"/>
     </row>
-    <row r="45" spans="3:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="45" spans="3:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="E45" s="3"/>
       <c r="F45" s="10"/>
       <c r="G45" s="3"/>
       <c r="J45" s="3"/>
       <c r="K45" s="10"/>
       <c r="L45" s="3"/>
-    </row>
-    <row r="48" spans="3:15" x14ac:dyDescent="0.35">
-      <c r="O48" t="s">
-        <v>218</v>
-      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -9548,7 +9624,7 @@
         <v>11</v>
       </c>
       <c r="C4" s="31" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="5" spans="2:20" x14ac:dyDescent="0.35">
@@ -9596,17 +9672,17 @@
     </row>
     <row r="11" spans="2:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C11" s="23"/>
-      <c r="E11" s="72" t="s">
+      <c r="E11" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="F11" s="73"/>
-      <c r="G11" s="74"/>
-      <c r="J11" s="72" t="s">
+      <c r="F11" s="72"/>
+      <c r="G11" s="73"/>
+      <c r="J11" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="K11" s="73"/>
-      <c r="L11" s="73"/>
-      <c r="M11" s="74"/>
+      <c r="K11" s="72"/>
+      <c r="L11" s="72"/>
+      <c r="M11" s="73"/>
     </row>
     <row r="12" spans="2:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C12" s="23"/>
@@ -9631,14 +9707,14 @@
       <c r="M12" s="34" t="s">
         <v>112</v>
       </c>
-      <c r="O12" s="75" t="s">
+      <c r="O12" s="74" t="s">
         <v>93</v>
       </c>
-      <c r="P12" s="75"/>
-      <c r="Q12" s="75"/>
-      <c r="R12" s="75"/>
-      <c r="S12" s="75"/>
-      <c r="T12" s="75"/>
+      <c r="P12" s="74"/>
+      <c r="Q12" s="74"/>
+      <c r="R12" s="74"/>
+      <c r="S12" s="74"/>
+      <c r="T12" s="74"/>
     </row>
     <row r="13" spans="2:20" x14ac:dyDescent="0.35">
       <c r="C13" s="23"/>
@@ -9662,12 +9738,12 @@
         <v>25</v>
       </c>
       <c r="M13" s="19"/>
-      <c r="O13" s="75"/>
-      <c r="P13" s="75"/>
-      <c r="Q13" s="75"/>
-      <c r="R13" s="75"/>
-      <c r="S13" s="75"/>
-      <c r="T13" s="75"/>
+      <c r="O13" s="74"/>
+      <c r="P13" s="74"/>
+      <c r="Q13" s="74"/>
+      <c r="R13" s="74"/>
+      <c r="S13" s="74"/>
+      <c r="T13" s="74"/>
     </row>
     <row r="14" spans="2:20" x14ac:dyDescent="0.35">
       <c r="C14" s="23"/>
@@ -9692,12 +9768,12 @@
       <c r="M14" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="O14" s="75"/>
-      <c r="P14" s="75"/>
-      <c r="Q14" s="75"/>
-      <c r="R14" s="75"/>
-      <c r="S14" s="75"/>
-      <c r="T14" s="75"/>
+      <c r="O14" s="74"/>
+      <c r="P14" s="74"/>
+      <c r="Q14" s="74"/>
+      <c r="R14" s="74"/>
+      <c r="S14" s="74"/>
+      <c r="T14" s="74"/>
     </row>
     <row r="15" spans="2:20" x14ac:dyDescent="0.35">
       <c r="C15" s="23"/>
@@ -9716,12 +9792,12 @@
       <c r="M15" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="O15" s="75"/>
-      <c r="P15" s="75"/>
-      <c r="Q15" s="75"/>
-      <c r="R15" s="75"/>
-      <c r="S15" s="75"/>
-      <c r="T15" s="75"/>
+      <c r="O15" s="74"/>
+      <c r="P15" s="74"/>
+      <c r="Q15" s="74"/>
+      <c r="R15" s="74"/>
+      <c r="S15" s="74"/>
+      <c r="T15" s="74"/>
     </row>
     <row r="16" spans="2:20" x14ac:dyDescent="0.35">
       <c r="C16" s="23"/>
@@ -9740,14 +9816,14 @@
       <c r="M16" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="O16" s="75" t="s">
+      <c r="O16" s="74" t="s">
         <v>110</v>
       </c>
-      <c r="P16" s="75"/>
-      <c r="Q16" s="75"/>
-      <c r="R16" s="75"/>
-      <c r="S16" s="75"/>
-      <c r="T16" s="75"/>
+      <c r="P16" s="74"/>
+      <c r="Q16" s="74"/>
+      <c r="R16" s="74"/>
+      <c r="S16" s="74"/>
+      <c r="T16" s="74"/>
     </row>
     <row r="17" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C17" s="23"/>
@@ -9766,12 +9842,12 @@
       <c r="M17" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="O17" s="75"/>
-      <c r="P17" s="75"/>
-      <c r="Q17" s="75"/>
-      <c r="R17" s="75"/>
-      <c r="S17" s="75"/>
-      <c r="T17" s="75"/>
+      <c r="O17" s="74"/>
+      <c r="P17" s="74"/>
+      <c r="Q17" s="74"/>
+      <c r="R17" s="74"/>
+      <c r="S17" s="74"/>
+      <c r="T17" s="74"/>
     </row>
     <row r="18" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C18" s="23"/>
@@ -9788,12 +9864,12 @@
         <v>151</v>
       </c>
       <c r="M18" s="2"/>
-      <c r="O18" s="75"/>
-      <c r="P18" s="75"/>
-      <c r="Q18" s="75"/>
-      <c r="R18" s="75"/>
-      <c r="S18" s="75"/>
-      <c r="T18" s="75"/>
+      <c r="O18" s="74"/>
+      <c r="P18" s="74"/>
+      <c r="Q18" s="74"/>
+      <c r="R18" s="74"/>
+      <c r="S18" s="74"/>
+      <c r="T18" s="74"/>
     </row>
     <row r="19" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C19" s="23"/>
@@ -9801,21 +9877,21 @@
       <c r="F19" s="9"/>
       <c r="G19" s="2"/>
       <c r="J19" s="4" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="K19" s="9">
         <v>13.2</v>
       </c>
       <c r="L19" s="6" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="M19" s="2"/>
-      <c r="O19" s="75"/>
-      <c r="P19" s="75"/>
-      <c r="Q19" s="75"/>
-      <c r="R19" s="75"/>
-      <c r="S19" s="75"/>
-      <c r="T19" s="75"/>
+      <c r="O19" s="74"/>
+      <c r="P19" s="74"/>
+      <c r="Q19" s="74"/>
+      <c r="R19" s="74"/>
+      <c r="S19" s="74"/>
+      <c r="T19" s="74"/>
     </row>
     <row r="20" spans="3:20" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C20" s="23"/>
@@ -9836,14 +9912,14 @@
       <c r="K21" s="9"/>
       <c r="L21" s="6"/>
       <c r="M21" s="2"/>
-      <c r="O21" s="76" t="s">
+      <c r="O21" s="75" t="s">
         <v>150</v>
       </c>
-      <c r="P21" s="76"/>
-      <c r="Q21" s="76"/>
-      <c r="R21" s="76"/>
-      <c r="S21" s="76"/>
-      <c r="T21" s="76"/>
+      <c r="P21" s="75"/>
+      <c r="Q21" s="75"/>
+      <c r="R21" s="75"/>
+      <c r="S21" s="75"/>
+      <c r="T21" s="75"/>
     </row>
     <row r="22" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C22" s="23"/>
@@ -9864,14 +9940,14 @@
       <c r="K23" s="9"/>
       <c r="L23" s="6"/>
       <c r="M23" s="2"/>
-      <c r="O23" s="75" t="s">
-        <v>178</v>
-      </c>
-      <c r="P23" s="75"/>
-      <c r="Q23" s="75"/>
-      <c r="R23" s="75"/>
-      <c r="S23" s="75"/>
-      <c r="T23" s="75"/>
+      <c r="O23" s="74" t="s">
+        <v>177</v>
+      </c>
+      <c r="P23" s="74"/>
+      <c r="Q23" s="74"/>
+      <c r="R23" s="74"/>
+      <c r="S23" s="74"/>
+      <c r="T23" s="74"/>
     </row>
     <row r="24" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C24" s="23"/>
@@ -9882,12 +9958,12 @@
       <c r="K24" s="9"/>
       <c r="L24" s="6"/>
       <c r="M24" s="2"/>
-      <c r="O24" s="75"/>
-      <c r="P24" s="75"/>
-      <c r="Q24" s="75"/>
-      <c r="R24" s="75"/>
-      <c r="S24" s="75"/>
-      <c r="T24" s="75"/>
+      <c r="O24" s="74"/>
+      <c r="P24" s="74"/>
+      <c r="Q24" s="74"/>
+      <c r="R24" s="74"/>
+      <c r="S24" s="74"/>
+      <c r="T24" s="74"/>
     </row>
     <row r="25" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C25" s="23"/>
@@ -9898,12 +9974,12 @@
       <c r="K25" s="9"/>
       <c r="L25" s="6"/>
       <c r="M25" s="2"/>
-      <c r="O25" s="75"/>
-      <c r="P25" s="75"/>
-      <c r="Q25" s="75"/>
-      <c r="R25" s="75"/>
-      <c r="S25" s="75"/>
-      <c r="T25" s="75"/>
+      <c r="O25" s="74"/>
+      <c r="P25" s="74"/>
+      <c r="Q25" s="74"/>
+      <c r="R25" s="74"/>
+      <c r="S25" s="74"/>
+      <c r="T25" s="74"/>
     </row>
     <row r="26" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C26" s="23"/>
@@ -9914,12 +9990,12 @@
       <c r="K26" s="9"/>
       <c r="L26" s="6"/>
       <c r="M26" s="2"/>
-      <c r="O26" s="75"/>
-      <c r="P26" s="75"/>
-      <c r="Q26" s="75"/>
-      <c r="R26" s="75"/>
-      <c r="S26" s="75"/>
-      <c r="T26" s="75"/>
+      <c r="O26" s="74"/>
+      <c r="P26" s="74"/>
+      <c r="Q26" s="74"/>
+      <c r="R26" s="74"/>
+      <c r="S26" s="74"/>
+      <c r="T26" s="74"/>
     </row>
     <row r="27" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C27" s="23"/>
@@ -9930,14 +10006,14 @@
       <c r="K27" s="9"/>
       <c r="L27" s="6"/>
       <c r="M27" s="2"/>
-      <c r="O27" s="75" t="s">
+      <c r="O27" s="74" t="s">
         <v>154</v>
       </c>
-      <c r="P27" s="75"/>
-      <c r="Q27" s="75"/>
-      <c r="R27" s="75"/>
-      <c r="S27" s="75"/>
-      <c r="T27" s="75"/>
+      <c r="P27" s="74"/>
+      <c r="Q27" s="74"/>
+      <c r="R27" s="74"/>
+      <c r="S27" s="74"/>
+      <c r="T27" s="74"/>
     </row>
     <row r="28" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C28" s="23"/>
@@ -9948,12 +10024,12 @@
       <c r="K28" s="9"/>
       <c r="L28" s="6"/>
       <c r="M28" s="2"/>
-      <c r="O28" s="75"/>
-      <c r="P28" s="75"/>
-      <c r="Q28" s="75"/>
-      <c r="R28" s="75"/>
-      <c r="S28" s="75"/>
-      <c r="T28" s="75"/>
+      <c r="O28" s="74"/>
+      <c r="P28" s="74"/>
+      <c r="Q28" s="74"/>
+      <c r="R28" s="74"/>
+      <c r="S28" s="74"/>
+      <c r="T28" s="74"/>
     </row>
     <row r="29" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C29" s="23"/>
@@ -9964,12 +10040,12 @@
       <c r="K29" s="9"/>
       <c r="L29" s="6"/>
       <c r="M29" s="2"/>
-      <c r="O29" s="75"/>
-      <c r="P29" s="75"/>
-      <c r="Q29" s="75"/>
-      <c r="R29" s="75"/>
-      <c r="S29" s="75"/>
-      <c r="T29" s="75"/>
+      <c r="O29" s="74"/>
+      <c r="P29" s="74"/>
+      <c r="Q29" s="74"/>
+      <c r="R29" s="74"/>
+      <c r="S29" s="74"/>
+      <c r="T29" s="74"/>
     </row>
     <row r="30" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C30" s="23"/>
@@ -9980,12 +10056,12 @@
       <c r="K30" s="9"/>
       <c r="L30" s="6"/>
       <c r="M30" s="2"/>
-      <c r="O30" s="75"/>
-      <c r="P30" s="75"/>
-      <c r="Q30" s="75"/>
-      <c r="R30" s="75"/>
-      <c r="S30" s="75"/>
-      <c r="T30" s="75"/>
+      <c r="O30" s="74"/>
+      <c r="P30" s="74"/>
+      <c r="Q30" s="74"/>
+      <c r="R30" s="74"/>
+      <c r="S30" s="74"/>
+      <c r="T30" s="74"/>
     </row>
     <row r="31" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C31" s="23"/>
@@ -9996,14 +10072,14 @@
       <c r="K31" s="9"/>
       <c r="L31" s="6"/>
       <c r="M31" s="2"/>
-      <c r="O31" s="75" t="s">
+      <c r="O31" s="74" t="s">
         <v>155</v>
       </c>
-      <c r="P31" s="75"/>
-      <c r="Q31" s="75"/>
-      <c r="R31" s="75"/>
-      <c r="S31" s="75"/>
-      <c r="T31" s="75"/>
+      <c r="P31" s="74"/>
+      <c r="Q31" s="74"/>
+      <c r="R31" s="74"/>
+      <c r="S31" s="74"/>
+      <c r="T31" s="74"/>
     </row>
     <row r="32" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C32" s="23"/>
@@ -10014,12 +10090,12 @@
       <c r="K32" s="9"/>
       <c r="L32" s="6"/>
       <c r="M32" s="2"/>
-      <c r="O32" s="75"/>
-      <c r="P32" s="75"/>
-      <c r="Q32" s="75"/>
-      <c r="R32" s="75"/>
-      <c r="S32" s="75"/>
-      <c r="T32" s="75"/>
+      <c r="O32" s="74"/>
+      <c r="P32" s="74"/>
+      <c r="Q32" s="74"/>
+      <c r="R32" s="74"/>
+      <c r="S32" s="74"/>
+      <c r="T32" s="74"/>
     </row>
     <row r="33" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C33" s="23"/>
@@ -10030,12 +10106,12 @@
       <c r="K33" s="9"/>
       <c r="L33" s="6"/>
       <c r="M33" s="2"/>
-      <c r="O33" s="75"/>
-      <c r="P33" s="75"/>
-      <c r="Q33" s="75"/>
-      <c r="R33" s="75"/>
-      <c r="S33" s="75"/>
-      <c r="T33" s="75"/>
+      <c r="O33" s="74"/>
+      <c r="P33" s="74"/>
+      <c r="Q33" s="74"/>
+      <c r="R33" s="74"/>
+      <c r="S33" s="74"/>
+      <c r="T33" s="74"/>
     </row>
     <row r="34" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C34" s="23"/>
@@ -10046,12 +10122,12 @@
       <c r="K34" s="9"/>
       <c r="L34" s="6"/>
       <c r="M34" s="2"/>
-      <c r="O34" s="75"/>
-      <c r="P34" s="75"/>
-      <c r="Q34" s="75"/>
-      <c r="R34" s="75"/>
-      <c r="S34" s="75"/>
-      <c r="T34" s="75"/>
+      <c r="O34" s="74"/>
+      <c r="P34" s="74"/>
+      <c r="Q34" s="74"/>
+      <c r="R34" s="74"/>
+      <c r="S34" s="74"/>
+      <c r="T34" s="74"/>
     </row>
     <row r="35" spans="3:20" x14ac:dyDescent="0.35">
       <c r="C35" s="23"/>
@@ -10206,7 +10282,7 @@
         <v>11</v>
       </c>
       <c r="C4" s="30" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="5" spans="2:19" x14ac:dyDescent="0.35">
@@ -10254,16 +10330,16 @@
     </row>
     <row r="11" spans="2:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C11" s="23"/>
-      <c r="E11" s="72" t="s">
+      <c r="E11" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="F11" s="73"/>
-      <c r="G11" s="74"/>
-      <c r="J11" s="72" t="s">
+      <c r="F11" s="72"/>
+      <c r="G11" s="73"/>
+      <c r="J11" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="K11" s="73"/>
-      <c r="L11" s="74"/>
+      <c r="K11" s="72"/>
+      <c r="L11" s="73"/>
     </row>
     <row r="12" spans="2:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C12" s="23"/>
@@ -10285,14 +10361,14 @@
       <c r="L12" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="N12" s="75" t="s">
+      <c r="N12" s="74" t="s">
         <v>84</v>
       </c>
-      <c r="O12" s="75"/>
-      <c r="P12" s="75"/>
-      <c r="Q12" s="75"/>
-      <c r="R12" s="75"/>
-      <c r="S12" s="75"/>
+      <c r="O12" s="74"/>
+      <c r="P12" s="74"/>
+      <c r="Q12" s="74"/>
+      <c r="R12" s="74"/>
+      <c r="S12" s="74"/>
     </row>
     <row r="13" spans="2:19" x14ac:dyDescent="0.35">
       <c r="C13" s="23"/>
@@ -10314,12 +10390,12 @@
       <c r="L13" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="N13" s="75"/>
-      <c r="O13" s="75"/>
-      <c r="P13" s="75"/>
-      <c r="Q13" s="75"/>
-      <c r="R13" s="75"/>
-      <c r="S13" s="75"/>
+      <c r="N13" s="74"/>
+      <c r="O13" s="74"/>
+      <c r="P13" s="74"/>
+      <c r="Q13" s="74"/>
+      <c r="R13" s="74"/>
+      <c r="S13" s="74"/>
     </row>
     <row r="14" spans="2:19" x14ac:dyDescent="0.35">
       <c r="C14" s="23"/>
@@ -10341,12 +10417,12 @@
       <c r="L14" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="N14" s="75"/>
-      <c r="O14" s="75"/>
-      <c r="P14" s="75"/>
-      <c r="Q14" s="75"/>
-      <c r="R14" s="75"/>
-      <c r="S14" s="75"/>
+      <c r="N14" s="74"/>
+      <c r="O14" s="74"/>
+      <c r="P14" s="74"/>
+      <c r="Q14" s="74"/>
+      <c r="R14" s="74"/>
+      <c r="S14" s="74"/>
     </row>
     <row r="15" spans="2:19" x14ac:dyDescent="0.35">
       <c r="C15" s="23"/>
@@ -10360,14 +10436,14 @@
         <v>392.666</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="N15" s="75"/>
-      <c r="O15" s="75"/>
-      <c r="P15" s="75"/>
-      <c r="Q15" s="75"/>
-      <c r="R15" s="75"/>
-      <c r="S15" s="75"/>
+        <v>206</v>
+      </c>
+      <c r="N15" s="74"/>
+      <c r="O15" s="74"/>
+      <c r="P15" s="74"/>
+      <c r="Q15" s="74"/>
+      <c r="R15" s="74"/>
+      <c r="S15" s="74"/>
     </row>
     <row r="16" spans="2:19" x14ac:dyDescent="0.35">
       <c r="C16" s="23"/>
@@ -10381,7 +10457,7 @@
         <v>110.01</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="17" spans="3:19" x14ac:dyDescent="0.35">
@@ -10396,7 +10472,7 @@
         <v>40.887999999999998</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
     </row>
     <row r="18" spans="3:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -10416,14 +10492,14 @@
       <c r="J19" s="4"/>
       <c r="K19" s="9"/>
       <c r="L19" s="2"/>
-      <c r="N19" s="86" t="s">
+      <c r="N19" s="85" t="s">
         <v>150</v>
       </c>
-      <c r="O19" s="87"/>
-      <c r="P19" s="87"/>
-      <c r="Q19" s="87"/>
-      <c r="R19" s="87"/>
-      <c r="S19" s="88"/>
+      <c r="O19" s="86"/>
+      <c r="P19" s="86"/>
+      <c r="Q19" s="86"/>
+      <c r="R19" s="86"/>
+      <c r="S19" s="87"/>
     </row>
     <row r="20" spans="3:19" x14ac:dyDescent="0.35">
       <c r="C20" s="23"/>
@@ -10433,14 +10509,14 @@
       <c r="J20" s="2"/>
       <c r="K20" s="9"/>
       <c r="L20" s="2"/>
-      <c r="N20" s="77" t="s">
-        <v>208</v>
-      </c>
-      <c r="O20" s="78"/>
-      <c r="P20" s="78"/>
-      <c r="Q20" s="78"/>
-      <c r="R20" s="78"/>
-      <c r="S20" s="79"/>
+      <c r="N20" s="76" t="s">
+        <v>207</v>
+      </c>
+      <c r="O20" s="77"/>
+      <c r="P20" s="77"/>
+      <c r="Q20" s="77"/>
+      <c r="R20" s="77"/>
+      <c r="S20" s="78"/>
     </row>
     <row r="21" spans="3:19" x14ac:dyDescent="0.35">
       <c r="C21" s="23"/>
@@ -10450,12 +10526,12 @@
       <c r="J21" s="2"/>
       <c r="K21" s="9"/>
       <c r="L21" s="2"/>
-      <c r="N21" s="80"/>
-      <c r="O21" s="81"/>
-      <c r="P21" s="81"/>
-      <c r="Q21" s="81"/>
-      <c r="R21" s="81"/>
-      <c r="S21" s="82"/>
+      <c r="N21" s="79"/>
+      <c r="O21" s="80"/>
+      <c r="P21" s="80"/>
+      <c r="Q21" s="80"/>
+      <c r="R21" s="80"/>
+      <c r="S21" s="81"/>
     </row>
     <row r="22" spans="3:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C22" s="23"/>
@@ -10465,12 +10541,12 @@
       <c r="J22" s="2"/>
       <c r="K22" s="9"/>
       <c r="L22" s="2"/>
-      <c r="N22" s="83"/>
-      <c r="O22" s="84"/>
-      <c r="P22" s="84"/>
-      <c r="Q22" s="84"/>
-      <c r="R22" s="84"/>
-      <c r="S22" s="85"/>
+      <c r="N22" s="82"/>
+      <c r="O22" s="83"/>
+      <c r="P22" s="83"/>
+      <c r="Q22" s="83"/>
+      <c r="R22" s="83"/>
+      <c r="S22" s="84"/>
     </row>
     <row r="23" spans="3:19" x14ac:dyDescent="0.35">
       <c r="C23" s="23"/>
@@ -10480,14 +10556,14 @@
       <c r="J23" s="2"/>
       <c r="K23" s="9"/>
       <c r="L23" s="2"/>
-      <c r="N23" s="77" t="s">
-        <v>259</v>
-      </c>
-      <c r="O23" s="78"/>
-      <c r="P23" s="78"/>
-      <c r="Q23" s="78"/>
-      <c r="R23" s="78"/>
-      <c r="S23" s="79"/>
+      <c r="N23" s="76" t="s">
+        <v>254</v>
+      </c>
+      <c r="O23" s="77"/>
+      <c r="P23" s="77"/>
+      <c r="Q23" s="77"/>
+      <c r="R23" s="77"/>
+      <c r="S23" s="78"/>
     </row>
     <row r="24" spans="3:19" x14ac:dyDescent="0.35">
       <c r="C24" s="23"/>
@@ -10497,12 +10573,12 @@
       <c r="J24" s="2"/>
       <c r="K24" s="9"/>
       <c r="L24" s="2"/>
-      <c r="N24" s="80"/>
-      <c r="O24" s="81"/>
-      <c r="P24" s="81"/>
-      <c r="Q24" s="81"/>
-      <c r="R24" s="81"/>
-      <c r="S24" s="82"/>
+      <c r="N24" s="79"/>
+      <c r="O24" s="80"/>
+      <c r="P24" s="80"/>
+      <c r="Q24" s="80"/>
+      <c r="R24" s="80"/>
+      <c r="S24" s="81"/>
     </row>
     <row r="25" spans="3:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C25" s="23"/>
@@ -10512,12 +10588,12 @@
       <c r="J25" s="2"/>
       <c r="K25" s="9"/>
       <c r="L25" s="2"/>
-      <c r="N25" s="83"/>
-      <c r="O25" s="84"/>
-      <c r="P25" s="84"/>
-      <c r="Q25" s="84"/>
-      <c r="R25" s="84"/>
-      <c r="S25" s="85"/>
+      <c r="N25" s="82"/>
+      <c r="O25" s="83"/>
+      <c r="P25" s="83"/>
+      <c r="Q25" s="83"/>
+      <c r="R25" s="83"/>
+      <c r="S25" s="84"/>
     </row>
     <row r="26" spans="3:19" x14ac:dyDescent="0.35">
       <c r="C26" s="23"/>
@@ -10690,7 +10766,7 @@
       <c r="L45" s="3"/>
     </row>
     <row r="49" spans="7:7" x14ac:dyDescent="0.35">
-      <c r="G49" s="65"/>
+      <c r="G49" s="64"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -10758,7 +10834,7 @@
         <v>13</v>
       </c>
       <c r="C6" s="25" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.35">
@@ -10766,7 +10842,7 @@
         <v>14</v>
       </c>
       <c r="C7" s="25" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.35">
@@ -10782,21 +10858,21 @@
         <v>32</v>
       </c>
       <c r="C9" s="26" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="10" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C10" s="23"/>
-      <c r="E10" s="72" t="s">
+      <c r="E10" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="73"/>
-      <c r="G10" s="74"/>
-      <c r="J10" s="72" t="s">
+      <c r="F10" s="72"/>
+      <c r="G10" s="73"/>
+      <c r="J10" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="K10" s="73"/>
-      <c r="L10" s="74"/>
+      <c r="K10" s="72"/>
+      <c r="L10" s="73"/>
     </row>
     <row r="11" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C11" s="23"/>
@@ -11303,7 +11379,7 @@
         <v>11</v>
       </c>
       <c r="C4" s="37" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="5" spans="2:19" x14ac:dyDescent="0.35">
@@ -11348,16 +11424,16 @@
     </row>
     <row r="10" spans="2:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C10" s="23"/>
-      <c r="E10" s="72" t="s">
+      <c r="E10" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="73"/>
-      <c r="G10" s="74"/>
-      <c r="J10" s="72" t="s">
+      <c r="F10" s="72"/>
+      <c r="G10" s="73"/>
+      <c r="J10" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="K10" s="73"/>
-      <c r="L10" s="74"/>
+      <c r="K10" s="72"/>
+      <c r="L10" s="73"/>
     </row>
     <row r="11" spans="2:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C11" s="23"/>
@@ -11421,14 +11497,14 @@
       <c r="L13" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="N13" s="75" t="s">
+      <c r="N13" s="74" t="s">
         <v>91</v>
       </c>
-      <c r="O13" s="75"/>
-      <c r="P13" s="75"/>
-      <c r="Q13" s="75"/>
-      <c r="R13" s="75"/>
-      <c r="S13" s="75"/>
+      <c r="O13" s="74"/>
+      <c r="P13" s="74"/>
+      <c r="Q13" s="74"/>
+      <c r="R13" s="74"/>
+      <c r="S13" s="74"/>
     </row>
     <row r="14" spans="2:19" x14ac:dyDescent="0.35">
       <c r="C14" s="23"/>
@@ -11450,12 +11526,12 @@
       <c r="L14" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="N14" s="75"/>
-      <c r="O14" s="75"/>
-      <c r="P14" s="75"/>
-      <c r="Q14" s="75"/>
-      <c r="R14" s="75"/>
-      <c r="S14" s="75"/>
+      <c r="N14" s="74"/>
+      <c r="O14" s="74"/>
+      <c r="P14" s="74"/>
+      <c r="Q14" s="74"/>
+      <c r="R14" s="74"/>
+      <c r="S14" s="74"/>
     </row>
     <row r="15" spans="2:19" x14ac:dyDescent="0.35">
       <c r="C15" s="23"/>
@@ -11471,12 +11547,12 @@
       <c r="L15" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="N15" s="75"/>
-      <c r="O15" s="75"/>
-      <c r="P15" s="75"/>
-      <c r="Q15" s="75"/>
-      <c r="R15" s="75"/>
-      <c r="S15" s="75"/>
+      <c r="N15" s="74"/>
+      <c r="O15" s="74"/>
+      <c r="P15" s="74"/>
+      <c r="Q15" s="74"/>
+      <c r="R15" s="74"/>
+      <c r="S15" s="74"/>
     </row>
     <row r="16" spans="2:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C16" s="23"/>
@@ -11492,12 +11568,12 @@
       <c r="L16" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="N16" s="75"/>
-      <c r="O16" s="75"/>
-      <c r="P16" s="75"/>
-      <c r="Q16" s="75"/>
-      <c r="R16" s="75"/>
-      <c r="S16" s="75"/>
+      <c r="N16" s="74"/>
+      <c r="O16" s="74"/>
+      <c r="P16" s="74"/>
+      <c r="Q16" s="74"/>
+      <c r="R16" s="74"/>
+      <c r="S16" s="74"/>
     </row>
     <row r="17" spans="3:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C17" s="23"/>
@@ -11513,14 +11589,14 @@
       <c r="L17" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="N17" s="75" t="s">
+      <c r="N17" s="74" t="s">
         <v>92</v>
       </c>
-      <c r="O17" s="75"/>
-      <c r="P17" s="75"/>
-      <c r="Q17" s="75"/>
-      <c r="R17" s="75"/>
-      <c r="S17" s="75"/>
+      <c r="O17" s="74"/>
+      <c r="P17" s="74"/>
+      <c r="Q17" s="74"/>
+      <c r="R17" s="74"/>
+      <c r="S17" s="74"/>
     </row>
     <row r="18" spans="3:19" x14ac:dyDescent="0.35">
       <c r="C18" s="23"/>
@@ -11536,12 +11612,12 @@
       <c r="L18" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="N18" s="75"/>
-      <c r="O18" s="75"/>
-      <c r="P18" s="75"/>
-      <c r="Q18" s="75"/>
-      <c r="R18" s="75"/>
-      <c r="S18" s="75"/>
+      <c r="N18" s="74"/>
+      <c r="O18" s="74"/>
+      <c r="P18" s="74"/>
+      <c r="Q18" s="74"/>
+      <c r="R18" s="74"/>
+      <c r="S18" s="74"/>
     </row>
     <row r="19" spans="3:19" x14ac:dyDescent="0.35">
       <c r="C19" s="23"/>
@@ -11557,12 +11633,12 @@
       <c r="L19" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="N19" s="75"/>
-      <c r="O19" s="75"/>
-      <c r="P19" s="75"/>
-      <c r="Q19" s="75"/>
-      <c r="R19" s="75"/>
-      <c r="S19" s="75"/>
+      <c r="N19" s="74"/>
+      <c r="O19" s="74"/>
+      <c r="P19" s="74"/>
+      <c r="Q19" s="74"/>
+      <c r="R19" s="74"/>
+      <c r="S19" s="74"/>
     </row>
     <row r="20" spans="3:19" x14ac:dyDescent="0.35">
       <c r="C20" s="23"/>
@@ -11576,14 +11652,14 @@
         <v>15</v>
       </c>
       <c r="L20" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="N20" s="75"/>
-      <c r="O20" s="75"/>
-      <c r="P20" s="75"/>
-      <c r="Q20" s="75"/>
-      <c r="R20" s="75"/>
-      <c r="S20" s="75"/>
+        <v>176</v>
+      </c>
+      <c r="N20" s="74"/>
+      <c r="O20" s="74"/>
+      <c r="P20" s="74"/>
+      <c r="Q20" s="74"/>
+      <c r="R20" s="74"/>
+      <c r="S20" s="74"/>
     </row>
     <row r="21" spans="3:19" x14ac:dyDescent="0.35">
       <c r="C21" s="23"/>
@@ -11597,7 +11673,7 @@
         <v>72</v>
       </c>
       <c r="L21" s="4" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="22" spans="3:19" x14ac:dyDescent="0.35">
@@ -11608,14 +11684,14 @@
       <c r="J22" s="2"/>
       <c r="K22" s="9"/>
       <c r="L22" s="4"/>
-      <c r="N22" s="76" t="s">
+      <c r="N22" s="75" t="s">
         <v>150</v>
       </c>
-      <c r="O22" s="76"/>
-      <c r="P22" s="76"/>
-      <c r="Q22" s="76"/>
-      <c r="R22" s="76"/>
-      <c r="S22" s="76"/>
+      <c r="O22" s="75"/>
+      <c r="P22" s="75"/>
+      <c r="Q22" s="75"/>
+      <c r="R22" s="75"/>
+      <c r="S22" s="75"/>
     </row>
     <row r="23" spans="3:19" x14ac:dyDescent="0.35">
       <c r="C23" s="23"/>
@@ -11634,14 +11710,14 @@
       <c r="J24" s="2"/>
       <c r="K24" s="9"/>
       <c r="L24" s="4"/>
-      <c r="N24" s="75" t="s">
-        <v>215</v>
-      </c>
-      <c r="O24" s="75"/>
-      <c r="P24" s="75"/>
-      <c r="Q24" s="75"/>
-      <c r="R24" s="75"/>
-      <c r="S24" s="75"/>
+      <c r="N24" s="74" t="s">
+        <v>214</v>
+      </c>
+      <c r="O24" s="74"/>
+      <c r="P24" s="74"/>
+      <c r="Q24" s="74"/>
+      <c r="R24" s="74"/>
+      <c r="S24" s="74"/>
     </row>
     <row r="25" spans="3:19" x14ac:dyDescent="0.35">
       <c r="C25" s="23"/>
@@ -11651,12 +11727,12 @@
       <c r="J25" s="2"/>
       <c r="K25" s="9"/>
       <c r="L25" s="4"/>
-      <c r="N25" s="75"/>
-      <c r="O25" s="75"/>
-      <c r="P25" s="75"/>
-      <c r="Q25" s="75"/>
-      <c r="R25" s="75"/>
-      <c r="S25" s="75"/>
+      <c r="N25" s="74"/>
+      <c r="O25" s="74"/>
+      <c r="P25" s="74"/>
+      <c r="Q25" s="74"/>
+      <c r="R25" s="74"/>
+      <c r="S25" s="74"/>
     </row>
     <row r="26" spans="3:19" x14ac:dyDescent="0.35">
       <c r="C26" s="23"/>
@@ -11666,12 +11742,12 @@
       <c r="J26" s="2"/>
       <c r="K26" s="9"/>
       <c r="L26" s="4"/>
-      <c r="N26" s="75"/>
-      <c r="O26" s="75"/>
-      <c r="P26" s="75"/>
-      <c r="Q26" s="75"/>
-      <c r="R26" s="75"/>
-      <c r="S26" s="75"/>
+      <c r="N26" s="74"/>
+      <c r="O26" s="74"/>
+      <c r="P26" s="74"/>
+      <c r="Q26" s="74"/>
+      <c r="R26" s="74"/>
+      <c r="S26" s="74"/>
     </row>
     <row r="27" spans="3:19" x14ac:dyDescent="0.35">
       <c r="C27" s="23"/>
@@ -11681,12 +11757,12 @@
       <c r="J27" s="2"/>
       <c r="K27" s="9"/>
       <c r="L27" s="4"/>
-      <c r="N27" s="75"/>
-      <c r="O27" s="75"/>
-      <c r="P27" s="75"/>
-      <c r="Q27" s="75"/>
-      <c r="R27" s="75"/>
-      <c r="S27" s="75"/>
+      <c r="N27" s="74"/>
+      <c r="O27" s="74"/>
+      <c r="P27" s="74"/>
+      <c r="Q27" s="74"/>
+      <c r="R27" s="74"/>
+      <c r="S27" s="74"/>
     </row>
     <row r="28" spans="3:19" x14ac:dyDescent="0.35">
       <c r="C28" s="23"/>
@@ -11696,14 +11772,14 @@
       <c r="J28" s="2"/>
       <c r="K28" s="9"/>
       <c r="L28" s="4"/>
-      <c r="N28" s="75" t="s">
+      <c r="N28" s="74" t="s">
         <v>153</v>
       </c>
-      <c r="O28" s="75"/>
-      <c r="P28" s="75"/>
-      <c r="Q28" s="75"/>
-      <c r="R28" s="75"/>
-      <c r="S28" s="75"/>
+      <c r="O28" s="74"/>
+      <c r="P28" s="74"/>
+      <c r="Q28" s="74"/>
+      <c r="R28" s="74"/>
+      <c r="S28" s="74"/>
     </row>
     <row r="29" spans="3:19" x14ac:dyDescent="0.35">
       <c r="C29" s="23"/>
@@ -11713,12 +11789,12 @@
       <c r="J29" s="2"/>
       <c r="K29" s="9"/>
       <c r="L29" s="4"/>
-      <c r="N29" s="75"/>
-      <c r="O29" s="75"/>
-      <c r="P29" s="75"/>
-      <c r="Q29" s="75"/>
-      <c r="R29" s="75"/>
-      <c r="S29" s="75"/>
+      <c r="N29" s="74"/>
+      <c r="O29" s="74"/>
+      <c r="P29" s="74"/>
+      <c r="Q29" s="74"/>
+      <c r="R29" s="74"/>
+      <c r="S29" s="74"/>
     </row>
     <row r="30" spans="3:19" x14ac:dyDescent="0.35">
       <c r="C30" s="23"/>
@@ -11728,12 +11804,12 @@
       <c r="J30" s="2"/>
       <c r="K30" s="9"/>
       <c r="L30" s="2"/>
-      <c r="N30" s="75"/>
-      <c r="O30" s="75"/>
-      <c r="P30" s="75"/>
-      <c r="Q30" s="75"/>
-      <c r="R30" s="75"/>
-      <c r="S30" s="75"/>
+      <c r="N30" s="74"/>
+      <c r="O30" s="74"/>
+      <c r="P30" s="74"/>
+      <c r="Q30" s="74"/>
+      <c r="R30" s="74"/>
+      <c r="S30" s="74"/>
     </row>
     <row r="31" spans="3:19" x14ac:dyDescent="0.35">
       <c r="C31" s="23"/>
@@ -11743,12 +11819,12 @@
       <c r="J31" s="2"/>
       <c r="K31" s="9"/>
       <c r="L31" s="2"/>
-      <c r="N31" s="75"/>
-      <c r="O31" s="75"/>
-      <c r="P31" s="75"/>
-      <c r="Q31" s="75"/>
-      <c r="R31" s="75"/>
-      <c r="S31" s="75"/>
+      <c r="N31" s="74"/>
+      <c r="O31" s="74"/>
+      <c r="P31" s="74"/>
+      <c r="Q31" s="74"/>
+      <c r="R31" s="74"/>
+      <c r="S31" s="74"/>
     </row>
     <row r="32" spans="3:19" x14ac:dyDescent="0.35">
       <c r="C32" s="23"/>
@@ -11955,16 +12031,16 @@
     </row>
     <row r="10" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C10" s="23"/>
-      <c r="E10" s="72" t="s">
+      <c r="E10" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="73"/>
-      <c r="G10" s="74"/>
-      <c r="J10" s="72" t="s">
+      <c r="F10" s="72"/>
+      <c r="G10" s="73"/>
+      <c r="J10" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="K10" s="73"/>
-      <c r="L10" s="74"/>
+      <c r="K10" s="72"/>
+      <c r="L10" s="73"/>
     </row>
     <row r="11" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C11" s="23"/>

</xml_diff>